<commit_message>
docs(uat): the pack quotes today's screens (build ebac9f4)
The UAT runbook and tracker quoted labels the UX packages and review fixes
changed: Needs attention, the action-named transition buttons, the per-role
sidebar with Your work, My tasks, Approval documents, Message templates,
Delegations, My profile in the account menu, My consents and My requests,
Updates, My nominations, Verify and continue, Add language, Copy an existing
notice, the participant status words, the four consent states, the DPO's
queue order, the new 404 pages and more. Sources edited, then the JSON cases,
the Word runbook and the Excel tracker rebuilt; the build under test is now
ebac9f4 on sprint-3/breach-and-correction.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/uat/COMPASS-CMP-UAT-Test-Cases.xlsx
+++ b/docs/uat/COMPASS-CMP-UAT-Test-Cases.xlsx
@@ -582,7 +582,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Branch refactor/frontend-architecture, commit 3024848 - 29 September 2026</t>
+          <t>Branch sprint-3/breach-and-correction, commit ebac9f4 - 5 October 2026</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
 3. 'Verify and continue' stays greyed out (disabled) until exactly six digits are entered. Letters typed into the box are ignored.
 4. You are signed in and land on the Dashboard. The page heading reads 'Good day, Priya'.
 5. The header shows the name 'Priya Menon' with a 'DPO' role badge and the initials 'PM'.
-6. The sidebar shows the sections Overview, Governance, Consent, Registry, Data movement, Oversight and You. Under Oversight there are 'Rights requests', 'Audit trail', 'Users', 'Delegate' and 'Messages'; under You there are 'Tickets for you', 'Notifications' and 'Your profile'. A 'Sign out' button is at the bottom of the sidebar.</t>
+6. The sidebar starts with the group 'Your work' - 'Dashboard', 'Rights requests', 'Breaches', 'My tasks', 'Projects', 'Notices' - followed by the groups Governance, Consent, Registry, Data movement and Oversight. Under Oversight there are 'Audit trail', 'Users', 'Delegations' and 'Message templates'. 'My profile' is not in the sidebar (it is in the account menu under your name at the top right), and notifications open from the bell in the header. A 'Sign out' button is at the bottom of the sidebar.</t>
         </is>
       </c>
       <c r="M2" s="11" t="inlineStr">
@@ -1437,11 +1437,11 @@
         <is>
           <t>1. The 'Verify it is you' page appears: the DCO also needs the second factor.
 2. The Dashboard opens with the heading 'Good day, Arun'. The header shows 'Arun Shetty' with the role badge 'Data Collection Owner'.
-3. The menu shows exactly: Dashboard; Projects; Consents, Consent links, Collection sites; Data sources; Collections, Exports, Imports; Delegate; Tickets for you, Notifications, Your profile. There is no 'Approvals', 'Notices', 'Purposes', 'Audit trail', 'Users' or 'Messages'.
+3. The menu shows exactly: Your work - Dashboard, My projects, Collection sites, Consent links, My tasks, Collections; Consent - Consents; Registry - Data sources; Data movement - Exports, Imports; Oversight - Delegations. There is no 'Approval documents', 'Notices', 'Purposes', 'Audit trail', 'Users' or 'Message templates'.
 4. The users register is not shown. The sidebar stays, and the page shows a notice titled 'Not part of your account' reading 'This section belongs to a different role, so there is nothing here for you.' with a 'Back to your dashboard' button.
 5. You are returned to the 'Sign in' page.
 6. The Dashboard opens with the heading 'Good day, System'. The header shows 'System Admin' with the role badge 'Administrator'.
-7. The menu shows: Dashboard; Processors, Data sources; Grievances about the DPO, Audit trail, Users, Delegate, Messages; Tickets for you, Notifications, Your profile. There is no 'Projects', 'Consents' or 'Consent links'. The rights item is labelled 'Grievances about the DPO', not 'Rights requests'.
+7. The menu shows: Your work - Dashboard, Users, Grievances about the DPO, Message templates, Processors, Data sources, Audit trail; Oversight - Delegations; You - My tasks. There is no 'Projects', 'Consents' or 'Consent links'. The rights item is labelled 'Grievances about the DPO', not 'Rights requests'.
 8. You are returned to the 'Sign in' page.</t>
         </is>
       </c>
@@ -1912,12 +1912,12 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Add a personal email and end another session from Your profile</t>
+          <t>Add a personal email and end another session from My profile</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Staff account page (Your profile)</t>
+          <t>Staff account page (My profile)</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
@@ -1955,19 +1955,19 @@
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>1. In browser 1, sign in to http://localhost:3000 as rnd@cmp.local with the password and code. Click 'Your profile' in the sidebar.
+          <t>1. In browser 1, sign in to http://localhost:3000 as rnd@cmp.local with the password and code. Click your name at the top right to open the account menu, then click 'My profile'.
 2. On the 'Contacts' tab, look at the 'Work email' row.
 3. In the 'Personal email' row, click 'Add' (or 'Change' if one is already there). Type tester01-kavya@example.org in the 'Personal email' box and click 'Save and send a code'.
 4. Type 000000 into 'Six-digit code' and click 'Confirm'.
 5. Ask the test coordinator for the code sent to tester01-kavya@example.org (from the test outbox). Replace the digits with it and click 'Confirm'.
-6. In browser 2, sign in to http://localhost:3000 as rnd@cmp.local with the password and a new code. Go back to browser 1 and refresh the 'Your account' page and click the 'Active sessions' tab.
+6. In browser 2, sign in to http://localhost:3000 as rnd@cmp.local with the password and a new code. Go back to browser 1 and refresh the 'My profile' page and click the 'Active sessions' tab.
 7. In browser 1, click 'End session' on the other session.
-8. In browser 2, click any sidebar item (for example 'Projects').</t>
+8. In browser 2, click any sidebar item (for example 'My projects').</t>
         </is>
       </c>
       <c r="L9" s="11" t="inlineStr">
         <is>
-          <t>1. The page 'Your account' opens with three tabs - 'Contacts' (selected), 'Active sessions' with a count, and 'Password' - and the 'Identity' card beside them. Identity shows Name 'Kavya Rao', Role 'R&amp;D User', Status 'Active' and a 'Session expires' time about 8 hours from now.
+          <t>1. The page 'My profile' opens with three tabs - 'Contacts' (selected), 'Active sessions' with a count, and 'Password' - and the 'Identity' card beside them. Identity shows Name 'Kavya Rao', Role 'R&amp;D User', Status 'Active' and a 'Session expires' time about 8 hours from now.
 2. It shows rnd@cmp.local with a 'Confirmed' badge. It has no 'Change', 'Add' or 'Remove' button.
 3. A green toast 'Saved' says 'We have sent a code to tester01-kavya@example.org.' The row shows the address with a 'Not confirmed' badge and a 'Six-digit code' box with 'Confirm' and 'Later' buttons.
 4. A red message 'Invalid or expired code' appears in the row; the address stays 'Not confirmed'.
@@ -2058,7 +2058,7 @@
 4. Type 000000 in both code boxes and click 'Confirm and sign in'.
 5. Ask the test coordinator for the code sent to +91 98111 22301 and the code sent to tester01@example.org (both from the test outbox). Replace the digits in each box with the matching code and click 'Confirm and sign in'.
 6. Look at the header and the sidebar.
-7. Click 'Your profile'.</t>
+7. Click your name at the top right to open the account menu, then click 'My profile'.</t>
         </is>
       </c>
       <c r="L10" s="11" t="inlineStr">
@@ -2067,14 +2067,14 @@
 2. It reads 'The law protects people under 18 differently, so we ask before an account is opened.' It does not mention a parent or guardian.
 3. The page 'Confirm your contacts' opens with the text 'If those details are new to us, a code has gone to your mobile and another to your email. Enter both.' It shows 'Code sent to your mobile' (with the mobile number under it), 'Code sent to your email' (with the email under it) and a 'Confirm and sign in' button.
 4. You stay on the page. A red banner reads 'Invalid or expired code'.
-5. Both codes are accepted even though a wrong pair was tried first. You are signed in and land on the page headed 'Your consents'.
-6. The header shows 'Tester One' with the role badge 'Data Subject'. The sidebar shows 'My consents', 'My requests', 'Notifications', 'Your profile' and 'Sign out'. There is no 'We need your date of birth' notice.
-7. 'Your account' opens. Identity shows Name 'Tester One', Mobile and Email as entered, Role 'Data Subject', Status 'Active' and Date of birth 15 Aug 1990 (no under-18 badge). In Contacts, the mobile and email both show 'Confirmed'.</t>
+5. Both codes are accepted even though a wrong pair was tried first. You are signed in and land on the page headed 'My consents'.
+6. The header shows 'Tester One' with the role badge 'Data Subject'. The sidebar shows 'My consents', 'My requests', 'My nominations', 'Updates' and 'Sign out'; 'My profile' is in the account menu under the name. There is no 'We need your date of birth' notice.
+7. 'My profile' opens. Identity shows Name 'Tester One', Mobile and Email as entered, Role 'Data Subject', Status 'Active' and Date of birth 15 Aug 1990 (no under-18 badge). In Contacts, the mobile and email both show 'Confirmed'.</t>
         </is>
       </c>
       <c r="M10" s="11" t="inlineStr">
         <is>
-          <t>A new adult can register with a mobile, an optional email and a date of birth, must confirm every contact given with its own code, and is then signed in to 'Your consents'.</t>
+          <t>A new adult can register with a mobile, an optional email and a date of birth, must confirm every contact given with its own code, and is then signed in to 'My consents'.</t>
         </is>
       </c>
       <c r="N10" s="16" t="n"/>
@@ -2419,16 +2419,16 @@
         <is>
           <t>1. The page headed 'Sign in' opens with the text 'Enter the mobile number or email address you registered with and we will send you a one-time code.' Under 'Sign in with' the 'Mobile' option is selected. At the bottom are 'Create an account', 'Your rights and how to exercise them', 'Act on their behalf here' and 'Sign in to the console'.
 2. A blue notice 'Check your messages' reads 'If +91 90000 00001 is registered with us, a six-digit code is on its way. It expires in ten minutes.' Below it are a 'Six-digit code' box, a 'Verify' button (disabled until six digits are typed) and a 'Use a different contact' button.
-3. You land on the page headed 'Your consents'. The header shows 'Anjali Verma' with the role badge 'Data Subject'.
-4. Under 'Your data' are 'My consents' and 'My requests'; under 'You' are 'Notifications' and 'Your profile'; 'Sign out' is at the bottom. There is no staff menu and no staff-account notice.
-5. The page headed 'Your requests' opens.
+3. You land on the page headed 'My consents'. The header shows 'Anjali Verma' with the role badge 'Data Subject'.
+4. Under 'Your data' are 'My consents', 'My requests', 'My nominations' and 'Updates'; 'Sign out' is at the bottom. 'My profile' is in the account menu under her name at the top right. There is no staff menu and no staff-account notice.
+5. The page headed 'My requests' opens.
 6. You are taken back to the portal 'Sign in' page.
 7. You are sent to the 'Sign in' page instead of seeing the consents.</t>
         </is>
       </c>
       <c r="M14" s="11" t="inlineStr">
         <is>
-          <t>A registered data principal signs in with just the code sent to her mobile, lands on 'Your consents', and after 'Sign out' can no longer open her pages.</t>
+          <t>A registered data principal signs in with just the code sent to her mobile, lands on 'My consents', and after 'Sign out' can no longer open her pages.</t>
         </is>
       </c>
       <c r="N14" s="16" t="n"/>
@@ -2513,7 +2513,7 @@
 3. The form returns to the contact step with the 'Send me a code' button.
 4. 'Check your messages' appears for subject@cmp.local with the 'Six-digit code' box.
 5. You stay on the page. A red banner reads 'Invalid or expired code'.
-6. The correct code is accepted and you land on 'Your consents' as Anjali Verma.
+6. The correct code is accepted and you land on 'My consents' as Anjali Verma.
 7. You are back on the portal 'Sign in' page.</t>
         </is>
       </c>
@@ -2592,28 +2592,28 @@
         <is>
           <t>1. Open http://localhost:3001/sign-in, choose 'Email', type rco@cmp.local, click 'Send me a code', then enter the code the test coordinator gives you for rco@cmp.local (from the test outbox) and click 'Verify'.
 2. Click 'My requests' in the sidebar.
-3. Click 'Notifications' in the sidebar.
-4. Click 'Your profile' in the sidebar.
+3. Click 'Updates' in the sidebar.
+4. Click your name at the top right to open the account menu, then click 'My profile'.
 5. Click the 'make a request' link on the card.
-6. Go back to 'Your consents' and click 'Add it now' in the notice.
-7. Click 'Your profile' to reach the 'Your date of birth' card. Type 1 January 2030 into 'Date of birth' and click 'Save and continue'.
+6. Go back to 'My consents' and click 'Add it now' in the notice.
+7. Open 'My profile' from the account menu to reach the 'Your date of birth' card. Type 1 January 2030 into 'Date of birth' and click 'Save and continue'.
 8. Change 'Date of birth' to 21 July 1985 and click 'Save and continue'.
-9. Click 'My consents' and then 'Notifications'.
+9. Click 'My consents' and then 'Updates'.
 10. Click 'Sign out', sign in again with rco@cmp.local and a new code.</t>
         </is>
       </c>
       <c r="L16" s="11" t="inlineStr">
         <is>
-          <t>1. You land on 'Your consents'. Above the list is a blue notice titled 'We need your date of birth' reading 'You can withdraw a consent or make a request without it, but we need it before you give a new consent.' with an 'Add it now' link.
-2. The page 'Your requests' opens normally, with the same 'We need your date of birth' notice above it. Nothing blocks this page.
-3. Instead of the notifications, a card headed 'Your date of birth' appears: 'The law protects people under 18 differently, and we do not have your date of birth yet. We need it before you can give a new consent.' It has a 'Date of birth' field, a 'Save and continue' button and links 'withdraw a consent' and 'make a request'.
+          <t>1. You land on 'My consents'. Above the list is a blue notice titled 'We need your date of birth' reading 'You can withdraw a consent or make a request without it, but we need it before you give a new consent.' with an 'Add it now' link.
+2. The page 'My requests' opens normally, with the same 'We need your date of birth' notice above it. Nothing blocks this page.
+3. Instead of the updates, a card headed 'Your date of birth' appears: 'The law protects people under 18 differently, and we do not have your date of birth yet. We need it before you can give a new consent.' It has a 'Date of birth' field, a 'Save and continue' button and links 'withdraw a consent' and 'make a request'.
 4. The same 'Your date of birth' card appears instead of the account page.
-5. 'Your requests' opens without answering the question.
-6. The 'Your date of birth' question is shown so the date can be added. (Record a defect if the link just reloads 'Your consents'.)
+5. 'My requests' opens without answering the question.
+6. The 'Your date of birth' question is shown so the date can be added. (Record a defect if the link just reloads 'My consents'.)
 7. The date is refused with 'Date of birth must be in the past' under the field; the card stays.
-8. The card disappears and the 'Your account' page opens. In Identity, 'Date of birth' shows 21 Jul 1985 with no under-18 badge.
-9. The 'We need your date of birth' notice no longer appears on 'Your consents', and 'Notifications' opens normally.
-10. You land on 'Your consents' with no date-of-birth notice; the question is not asked again.</t>
+8. The card disappears and the 'My profile' page opens. In Identity, 'Date of birth' shows 21 Jul 1985 with no under-18 badge.
+9. The 'We need your date of birth' notice no longer appears on 'My consents', and 'Updates' opens normally.
+10. You land on 'My consents' with no date-of-birth notice; the question is not asked again.</t>
         </is>
       </c>
       <c r="M16" s="11" t="inlineStr">
@@ -2689,7 +2689,7 @@
           <t>1. Open http://localhost:3001/sign-in, choose 'Email', type dpo@cmp.local and click 'Send me a code'.
 2. Enter the code the test coordinator gives you for dpo@cmp.local (from the test outbox) and click 'Verify'.
 3. Look at the header and sidebar.
-4. Click 'Your profile'. If the 'Your date of birth' card appears, enter 21 July 1985 and click 'Save and continue'.
+4. Click your name at the top right to open the account menu, then click 'My profile'. If the 'Your date of birth' card appears, enter 21 July 1985 and click 'Save and continue'.
 5. In the same window, open http://localhost:3000/users (the console).
 6. Open http://localhost:3000/sign-in in the same window.
 7. On the portal click 'Sign out'. Then sign in to the console at http://localhost:3000/sign-in as dpo@cmp.local with SeedPassw0rd!2026 and the emailed code.</t>
@@ -2698,9 +2698,9 @@
       <c r="L17" s="11" t="inlineStr">
         <is>
           <t>1. 'Check your messages' appears with the 'Six-digit code' box. No password is asked for.
-2. You land on 'Your consents'. A line across the top reads 'You are signed in with your staff account, as a data principal. Only your own consents, requests and rights are here; your console is a separate site.'
-3. The header shows 'Priya Menon' with the role badge 'Data Subject' (not 'DPO'). The sidebar has only 'My consents', 'My requests', 'Notifications', 'Your profile' and 'Sign out'.
-4. 'Your account' opens. In Identity, Role shows 'Data Subject' and an 'Account' line reads 'Your staff account, used here as a data principal.' In Contacts, the 'Email' row shows dpo@cmp.local with the hint 'Your staff address, managed by your organisation. If you may lose it one day, add a personal one below.' and no 'Change' button.
+2. You land on 'My consents'. A line across the top reads 'You are signed in with your staff account, as a data principal. Only your own consents, requests and rights are here; your console is a separate site.'
+3. The header shows 'Priya Menon' with the role badge 'Data Subject' (not 'DPO'). The sidebar has only 'My consents', 'My requests', 'My nominations', 'Updates' and 'Sign out'; 'My profile' is in the account menu.
+4. 'My profile' opens. In Identity, Role shows 'Data Subject' and an 'Account' line reads 'Your staff account, used here as a data principal.' In Contacts, the 'Email' row shows dpo@cmp.local with the hint 'Your staff address, managed by your organisation. If you may lose it one day, add a personal one below.' and no 'Change' button.
 5. No user list is shown. The console shows a page headed 'This console is for staff' reading 'You are signed in as Priya Menon. Your consents, your requests and your rights are on the consent portal.' with the buttons 'Go to the consent portal' and 'Sign out'.
 6. The console sign-in form does not stay; you are sent to the portal (http://localhost:3001), because this window holds a data principal session.
 7. The console asks for the password and the code, and only then shows the full DPO Dashboard with the 'DPO' badge. The portal code alone never gave DPO access.</t>
@@ -2778,26 +2778,26 @@
       </c>
       <c r="K18" s="11" t="inlineStr">
         <is>
-          <t>1. Click 'Your profile'.
+          <t>1. Click your name at the top right to open the account menu, then click 'My profile'.
 2. In the 'Second email' row click 'Add', type tester01@example.org and click 'Save and send a code'.
 3. Replace it with subject@cmp.local and click 'Save and send a code'.
 4. Replace it with tester01-personal@example.org and click 'Save and send a code'.
 5. Click 'Later'. Then click 'Sign out'. On 'Sign in', choose 'Email', type tester01-personal@example.org and click 'Send me a code'.
-6. Click 'Use a different contact' and sign in with the mobile +91 98111 22301 and its code from the test coordinator. Open 'Your profile'.
+6. Click 'Use a different contact' and sign in with the mobile +91 98111 22301 and its code from the test coordinator. Open 'My profile' from the account menu.
 7. Click 'Send a code'. Enter the code the test coordinator gives you for tester01-personal@example.org and click 'Confirm'.
 8. Click 'Sign out'. Sign in with 'Email' tester01-personal@example.org and the code the test coordinator gives you for it.</t>
         </is>
       </c>
       <c r="L18" s="11" t="inlineStr">
         <is>
-          <t>1. 'Your account' opens. Contacts lists 'Email' (tester01@example.org, 'Confirmed', no Change button), 'Mobile' (with 'Change') and 'Second email' ('None given', with 'Add'). Identity shows a 'Session expires' time about 8 hours after you signed in.
+          <t>1. 'My profile' opens. Contacts lists 'Email' (tester01@example.org, 'Confirmed', no Change button), 'Mobile' (with 'Change') and 'Second email' ('None given', with 'Add'). Identity shows a 'Session expires' time about 8 hours after you signed in.
 2. A red message in the row reads 'That is already the address on your account'.
 3. A red message reads 'That address belongs to another account'.
 4. Green toast 'Saved': 'We have sent a code to tester01-personal@example.org.' The row shows the address with 'Not confirmed' and a 'Six-digit code' box with 'Confirm' and 'Later'.
 5. The neutral 'Check your messages' notice appears, but the test coordinator confirms that no sign-in code was sent to tester01-personal@example.org: an unconfirmed address cannot sign anyone in.
 6. The 'Second email' row shows tester01-personal@example.org with 'Not confirmed' and a 'Send a code' button.
 7. Green toast 'Confirmed': 'tester01-personal@example.org can now sign you in.' The row shows 'Confirmed' and a 'Remove' button.
-8. You are signed in as Tester One and land on 'Your consents'.</t>
+8. You are signed in as Tester One and land on 'My consents'.</t>
         </is>
       </c>
       <c r="M18" s="11" t="inlineStr">
@@ -2872,7 +2872,7 @@
       </c>
       <c r="K19" s="11" t="inlineStr">
         <is>
-          <t>1. Click 'Your profile'. In the 'Mobile' row click 'Change'.
+          <t>1. Click your name at the top right to open the account menu, then click 'My profile'. In the 'Mobile' row click 'Change'.
 2. Replace the number with +91 90000 00001 and click 'Save and send a code'.
 3. Replace the number with +91 98111 22399 and click 'Save and send a code'.
 4. Type 000000 and click 'Confirm'.
@@ -2891,7 +2891,7 @@
 5. A new code is sent (toast 'Saved': 'We have sent a code to +91 98111 22399.') and the 'Six-digit code' box appears again.
 6. Green toast 'Confirmed': '+91 98111 22399 can now sign you in.' The row shows 'Confirmed'.
 7. Toast 'Saved': 'That contact is already confirmed, so no code was needed.' No code box appears and the badge stays 'Confirmed'.
-8. You are signed in as Tester One and land on 'Your consents'.</t>
+8. You are signed in as Tester One and land on 'My consents'.</t>
         </is>
       </c>
       <c r="M19" s="11" t="inlineStr">
@@ -2978,10 +2978,10 @@
         <is>
           <t>1. A page headed 'Verify it is you' briefly says 'Staff sign in on the console. Taking you there.' and you are then taken to the console (http://localhost:3000). With no sign-in in progress, the console shows its 'Sign in' page. There is no 'page not found'.
 2. You are sent to the portal 'Sign in' page; the address contains 'next=' followed by the my-requests path.
-3. You land on 'Your requests' (the page you asked for), not on 'Your consents'.
-4. The sign-in form does not stay; you are sent to 'Your consents'.
-5. The sign-up form does not stay; you are sent to 'Your consents'.
-6. The portal home goes straight to 'Your consents'.
+3. You land on 'My requests' (the page you asked for), not on 'My consents'.
+4. The sign-in form does not stay; you are sent to 'My consents'.
+5. The sign-up form does not stay; you are sent to 'My consents'.
+6. The portal home goes straight to 'My consents'.
 7. You are back on the portal 'Sign in' page.</t>
         </is>
       </c>
@@ -3055,18 +3055,18 @@
       </c>
       <c r="K21" s="11" t="inlineStr">
         <is>
-          <t>1. Sign in to http://localhost:3001 with 'Mobile' +91 90000 00001 and the code the test coordinator gives you. Click 'Your profile' and note the 'Session expires' time in Identity.
+          <t>1. Sign in to http://localhost:3001 with 'Mobile' +91 90000 00001 and the code the test coordinator gives you. Open 'My profile' from the account menu (your name at the top right) and note the 'Session expires' time in Identity.
 2. Click 'My consents'. Then leave the browser completely untouched (no clicks, no typing, do not switch to this window) for 31 minutes.
-3. After 31 minutes, return to the window and, if you are still on 'Your consents', click 'My requests'.
+3. After 31 minutes, return to the window and, if you are still on 'My consents', click 'My requests'.
 4. Sign in again with the mobile and a new code from the test coordinator.</t>
         </is>
       </c>
       <c r="L21" s="11" t="inlineStr">
         <is>
-          <t>1. 'Your account' opens. 'Session expires' is about 8 hours after the sign-in time (the absolute limit).
+          <t>1. 'My profile' opens. 'Session expires' is about 8 hours after the sign-in time (the absolute limit).
 2. Nothing visible happens while you wait.
 3. Your data is not shown any more. As soon as you return to the window, or at the latest when you click, you are taken to the portal 'Sign in' page (the address carries 'next='), because the session ended after 30 minutes without activity.
-4. You are signed in again and land on the page named in the address ('Your consents' or 'Your requests'), not on a blank or error page.</t>
+4. You are signed in again and land on the page named in the address ('My consents' or 'My requests'), not on a blank or error page.</t>
         </is>
       </c>
       <c r="M21" s="11" t="inlineStr">
@@ -3143,7 +3143,7 @@
       <c r="K22" s="11" t="inlineStr">
         <is>
           <t>1. Open http://localhost:3000. On the 'Sign in' page type admin@cmp.local in 'Email or username' and SeedPassw0rd!2026 in 'Password', then click 'Sign in'. On the 'Verify it is you' page, ask the test coordinator for the sign-in code sent to admin@cmp.local (from the test outbox), type it in '6-digit code' and click 'Verify and continue'.
-2. In the left-hand sidebar, under 'Oversight', click 'Users'.
+2. In the left-hand sidebar, under 'Your work', click 'Users'.
 3. Click 'Provision account'.
 4. Type 'UAT DCO 01' in 'Full name' and 'uat.dco01@cmp.local' in 'Email'. In 'Role' choose 'Data Collection Owner'. In 'Person type' choose 'Employee'. Leave the 'Data sources' boxes unticked.
 5. Click 'Create account'.
@@ -3252,7 +3252,7 @@
 2. The password is not set. The message 'The two passwords do not match' appears under 'Confirm new password'.
 3. A green panel 'Password changed' appears ('Every other session has been signed out. Taking you to sign in…') and after a few seconds the 'Sign in' page opens.
 4. The Dashboard opens. The top-right corner of the header shows 'UAT DCO 01' with the role badge 'Data Collection Owner'.
-5. The sidebar shows the Data Collection Owner's sections (for example 'Projects', 'Collection sites', 'Data sources', 'Delegate') and does NOT show 'Users'.
+5. The sidebar shows the Data Collection Owner's pages (for example 'My projects', 'Collection sites', 'Data sources', 'Delegations') and does NOT show 'Users'.
 6. You are returned to the 'Sign in' page.
 7. The Dashboard opens. The top-right corner of the header shows 'System Admin' with the role badge 'Administrator'.
 8. UAT DCO 01 now shows Status 'Active'. The 'Resend invitation' button is no longer offered for that row.</t>
@@ -3380,7 +3380,7 @@
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Users - access by role; Messages - access by role</t>
+          <t>Users - access by role; Message templates - access by role</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
@@ -3433,7 +3433,7 @@
 2. The 'Users' register opens read-only: a blue note says 'You can read the register. Provisioning, role changes and deactivation are restricted to administrators.' There is NO 'Provision account' button, and the 'Action' column of every row is empty (no 'Edit', 'Role', 'Reset MFA', 'Resend invitation' or 'End staff access').
 3. You are returned to the 'Sign in' page.
 4. The Dashboard opens. The top-right corner of the header shows 'Arun Shetty' with the role badge 'Data Collection Owner'.
-5. There is no 'Users' entry and no 'Messages' entry.
+5. There is no 'Users' entry and no 'Message templates' entry.
 6. No register is shown. A panel titled 'Not part of your account' says the section belongs to a different role, with a 'Back to your dashboard' button.
 7. The same 'Not part of your account' panel is shown; no message templates are visible.
 8. You are returned to the 'Sign in' page.
@@ -3443,7 +3443,7 @@
       </c>
       <c r="M25" s="11" t="inlineStr">
         <is>
-          <t>Only the Administrator can provision or change accounts; the DPO sees a read-only register; DCO and R&amp;D User have no Users or Messages section and are turned away if they type the address.</t>
+          <t>Only the Administrator can provision or change accounts; the DPO sees a read-only register; DCO and R&amp;D User have no Users or Message templates page and are turned away if they type the address.</t>
         </is>
       </c>
       <c r="N25" s="16" t="n"/>
@@ -4554,7 +4554,7 @@
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Messages - edit the words of a message</t>
+          <t>Message templates - edit the words of a message</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
@@ -4590,7 +4590,7 @@
       <c r="K38" s="11" t="inlineStr">
         <is>
           <t>1. Open http://localhost:3000. On the 'Sign in' page type admin@cmp.local in 'Email or username' and SeedPassw0rd!2026 in 'Password', then click 'Sign in'. On the 'Verify it is you' page, ask the test coordinator for the sign-in code sent to admin@cmp.local (from the test outbox), type it in '6-digit code' and click 'Verify and continue'.
-2. In the sidebar under 'Oversight' click 'Messages'.
+2. In the sidebar under 'Your work' click 'Message templates'.
 3. Under 'Sign-in' find the card 'Staff account invitation'.
 4. Click at the end of 'Body', press Enter twice and type 'UAT check: welcome aboard, '. Then click the variable chip '{full_name}' and type '.'
 5. Click 'Preview'.
@@ -4602,7 +4602,7 @@
       <c r="L38" s="11" t="inlineStr">
         <is>
           <t>1. The Dashboard opens. The top-right corner of the header shows 'System Admin' with the role badge 'Administrator'.
-2. The 'Messages' page opens with messages grouped under headings such as 'Sign-in', 'Consent', 'Rights' and 'Staff'.
+2. The 'Message templates' page opens with messages grouped under headings such as 'Sign-in', 'Consent', 'Rights' and 'Staff'.
 3. The card shows a 'Default words' badge, a 'Subject' field, a 'Body' field, the list 'Variables this message can use (click to insert)' (including {full_name}, {code}, {reset_url}) and the buttons 'Save' (disabled) and 'Preview'.
 4. The text '{full_name}' is inserted where the cursor was. The 'Save' button becomes enabled.
 5. A 'Preview, with sample values' box shows the email with sample values filled in, ending 'UAT check: welcome aboard, Asha Rao.'
@@ -4644,7 +4644,7 @@
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>Messages - variable check</t>
+          <t>Message templates - variable check</t>
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr">
@@ -4680,7 +4680,7 @@
       </c>
       <c r="K39" s="11" t="inlineStr">
         <is>
-          <t>1. Click 'Messages' and find the card 'Staff sign-in code' under 'Sign-in'.
+          <t>1. In the sidebar under 'Oversight' click 'Message templates' and find the card 'Staff sign-in code' under 'Sign-in'.
 2. Replace the whole 'Body' with 'Dear {full_name}, your code is {code}.' and click 'Save'.
 3. Change the 'Body' to 'Your code is {code}.' (only an allowed variable) and click 'Preview' - do NOT click 'Save'.
 4. Reload the page and look at the 'Staff sign-in code' card.</t>
@@ -4727,7 +4727,7 @@
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Delegate - Delegate my work</t>
+          <t>Delegations - Delegate my work</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
@@ -4766,21 +4766,21 @@
       <c r="K40" s="11" t="inlineStr">
         <is>
           <t>1. Open http://localhost:3000. On the 'Sign in' page type dco@cmp.local in 'Email or username' and SeedPassw0rd!2026 in 'Password', then click 'Sign in'. On the 'Verify it is you' page, ask the test coordinator for the sign-in code sent to dco@cmp.local (from the test outbox), type it in '6-digit code' and click 'Verify and continue'.
-2. In the sidebar under 'Oversight' click 'Delegate'.
+2. In the sidebar under 'Oversight' click 'Delegations'.
 3. Click 'Delegate my work' and open the 'Who takes over' drop-down.
 4. Choose UAT DCO 01, set 'Until' to 7 days from today, type 'UAT - annual leave cover' in 'Why' and click 'Delegate'.
 5. Click 'Sign out' at the bottom of the left-hand sidebar.
 6. Open http://localhost:3000. On the 'Sign in' page type uat.dco01@cmp.local in 'Email or username' and UatPassw0rd!2026 in 'Password', then click 'Sign in'. On the 'Verify it is you' page, ask the test coordinator for the sign-in code sent to uat.dco01@cmp.local (from the test outbox), type it in '6-digit code' and click 'Verify and continue'.
-7. Click 'Delegate'.
+7. Click 'Delegations' in the sidebar.
 8. Click 'Sign out' at the bottom of the left-hand sidebar.
 9. Open http://localhost:3000. On the 'Sign in' page type dco@cmp.local in 'Email or username' and SeedPassw0rd!2026 in 'Password', then click 'Sign in'. On the 'Verify it is you' page, ask the test coordinator for the sign-in code sent to dco@cmp.local (from the test outbox), type it in '6-digit code' and click 'Verify and continue'.
-10. Click 'Delegate' and click 'End now' on the UAT DCO 01 arrangement.</t>
+10. Click 'Delegations' and click 'End now' on the UAT DCO 01 arrangement.</t>
         </is>
       </c>
       <c r="L40" s="11" t="inlineStr">
         <is>
           <t>1. The Dashboard opens. The top-right corner of the header shows 'Arun Shetty' with the role badge 'Data Collection Owner'.
-2. The 'Delegate' page opens with a 'Delegate my work' button and the cards 'My delegations' ('You have not delegated your work to anybody') and 'Work delegated to me'.
+2. The 'Delegations' page opens with a 'Delegate my work' button and the cards 'My delegations' ('You have not delegated your work to anybody') and 'Work delegated to me'.
 3. A dialog 'Delegate my work' opens. 'Who takes over' lists colleagues in the same role, including 'UAT DCO 01 · uat.dco01@cmp.local'.
 4. 'Work delegated' appears. 'My delegations' lists UAT DCO 01 with 'until &lt;date&gt;' and the quoted reason, and an 'End now' button.
 5. You are returned to the 'Sign in' page.
@@ -4824,7 +4824,7 @@
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>Delegate - access by role</t>
+          <t>Delegations - access by role</t>
         </is>
       </c>
       <c r="E41" s="11" t="inlineStr">
@@ -4864,16 +4864,16 @@
 2. Look through the sidebar, then open http://localhost:3000/delegate directly.
 3. Click 'Sign out' at the bottom of the left-hand sidebar.
 4. Open http://localhost:3000. On the 'Sign in' page type admin@cmp.local in 'Email or username' and SeedPassw0rd!2026 in 'Password', then click 'Sign in'. On the 'Verify it is you' page, ask the test coordinator for the sign-in code sent to admin@cmp.local (from the test outbox), type it in '6-digit code' and click 'Verify and continue'.
-5. Click 'Delegate'.
+5. Under 'Oversight' click 'Delegations'.
 6. Click 'Sign out' at the bottom of the left-hand sidebar.
 7. Open http://localhost:3000. On the 'Sign in' page type dpo@cmp.local in 'Email or username' and SeedPassw0rd!2026 in 'Password', then click 'Sign in'. On the 'Verify it is you' page, ask the test coordinator for the sign-in code sent to dpo@cmp.local (from the test outbox), type it in '6-digit code' and click 'Verify and continue'.
-8. Click 'Delegate', then 'Delegate my work'.</t>
+8. Under 'Oversight' click 'Delegations', then 'Delegate my work'.</t>
         </is>
       </c>
       <c r="L41" s="11" t="inlineStr">
         <is>
           <t>1. The Dashboard opens. The top-right corner of the header shows 'Kavya Rao' with the role badge 'R&amp;D User'.
-2. There is no 'Delegate' entry; the address shows 'Not part of your account' with 'Back to your dashboard'.
+2. There is no 'Delegations' entry; the address shows 'Not part of your account' with 'Back to your dashboard'.
 3. You are returned to the 'Sign in' page.
 4. The Dashboard opens. The top-right corner of the header shows 'System Admin' with the role badge 'Administrator'.
 5. The page shows NO 'Delegate my work' button; a blue note explains delegation applies to roles whose access is defined by assignment. An 'Everyone, right now' card shows live arrangements across the organisation (or 'No delegation is in place').
@@ -4884,7 +4884,7 @@
       </c>
       <c r="M41" s="11" t="inlineStr">
         <is>
-          <t>R&amp;D Users cannot reach Delegate, the Administrator can only oversee (not arrange), and a DPO with no same-role colleague cannot delegate.</t>
+          <t>R&amp;D Users cannot reach Delegations, the Administrator can only oversee (not arrange), and a DPO with no same-role colleague cannot delegate.</t>
         </is>
       </c>
       <c r="N41" s="16" t="n"/>
@@ -5137,8 +5137,8 @@
         <is>
           <t>1. Click 'Projects' in the sidebar, type 'UAT Study 01' in 'Search' (the list updates as you type). Click 'UAT Study 01'.
 2. Find the card titled 'What happens next'.
-3. Read the warning lines under 'Move to Pending Approval'.
-4. Try to click the 'Pending Approval' button on that row.
+3. Read the warning lines under 'Moves the project to Pending Approval'.
+4. Try to click the 'Submit for approval' button on that row.
 5. Look at the 'Notices' card.
 6. Look at the 'Approvals' card.
 7. Look at the buttons at the top of the page.</t>
@@ -5147,12 +5147,12 @@
       <c r="L44" s="11" t="inlineStr">
         <is>
           <t>1. The project page opens with status 'In Draft'.
-2. It reads 'Currently In Draft. These are the moves your role can make from here.' and shows one row 'Move to Pending Approval'.
+2. It reads 'Currently In Draft. These are the moves your role can make from here.' and shows one row 'Moves the project to Pending Approval' with a 'Submit for approval' button.
 3. All six missing items are listed at once, each with a warning icon: 'The project has no notice'; 'The notice has no purposes attached'; 'The notice is missing required Rule 3 elements'; 'The notice does not say who it applies to'; 'The notice has no text yet - add at least one language'; 'No approval with a proof file'.
 4. The button is greyed out (disabled); nothing happens and the status stays 'In Draft'.
-5. It shows 'No notice yet' with the buttons 'Upload a notice document' and 'Use an existing notice'.
+5. It shows 'No notice yet' with the buttons 'Upload a notice document' and 'Copy an existing notice'.
 6. It shows count 0, 'No approval uploaded', the text 'A security approval with its proof file is what unlocks the move to pending approval.' and an 'Upload an approval' button.
-7. 'Edit', 'Upload a notice document', 'Use an existing notice', 'Upload approval' and 'Add site' are shown. There is NO 'New notice' button.</t>
+7. 'Edit', 'Upload a notice document', 'Copy an existing notice', 'Upload approval' and 'Add site' are shown. There is NO 'New notice' button.</t>
         </is>
       </c>
       <c r="M44" s="11" t="inlineStr">
@@ -5336,8 +5336,8 @@
 4. If the document names a different project (the example file names 'Gait Identification Study 2026') a warning says 'The document names the project ... but this project is 'UAT Study 01'. Check you are uploading to the right one.' This is expected with the example file.
 5. An excerpt of the notice wording is shown.
 6. The dialog closes and a green toast 'Notice created' says 'NTC-UAT-STUDY-01-2026 carries 9 purposes. The DPO activates them before it can be published.'
-7. It lists 'NTC-UAT-STUDY-01-2026 v1' with '9 purpose(s) · 1 language(s)' and the status badge 'Draft'.
-8. Under 'Move to Pending Approval' only one line remains: 'No approval with a proof file'. The 'Pending Approval' button is still disabled.
+7. It lists 'NTC-UAT-STUDY-01-2026 v1' with '9 purposes · 1 language(s)' and the status badge 'Draft'.
+8. Under 'Moves the project to Pending Approval' only one line remains: 'No approval with a proof file'. The 'Submit for approval' button is still disabled.
 9. The notice page opens titled 'NTC-UAT-STUDY-01-2026 · version 1' with 'Draft. Nothing here has been shown to a data subject yet.' The 'Purposes' card lists 9 purposes, each with the status 'Draft'.</t>
         </is>
       </c>
@@ -5374,7 +5374,7 @@
       </c>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>Use an existing notice</t>
+          <t>Copy an existing notice</t>
         </is>
       </c>
       <c r="E47" s="11" t="inlineStr">
@@ -5414,7 +5414,7 @@
       <c r="K47" s="11" t="inlineStr">
         <is>
           <t>1. Click 'Projects' &gt; 'Register a project'. Enter the name and description from the test data, tick 'SEED' and click 'Register project'.
-2. In the 'Notices' card click 'Use an existing notice'.
+2. In the 'Notices' card click 'Copy an existing notice'.
 3. Open 'Notice to copy'.
 4. Choose 'NTC-GAIT-2026 v1 — Gait Identification Study 2026'.
 5. Click 'Copy into this project'.
@@ -5425,7 +5425,7 @@
       <c r="L47" s="11" t="inlineStr">
         <is>
           <t>1. Toast 'Project registered'; the 'UAT Study 02' page opens with status 'In Draft'.
-2. A dialog 'Use an existing notice' opens: 'Copies the wording, the purposes and every language rendition into this project as a fresh draft.' with a 'Notice to copy' list and a disabled 'Copy into this project' button.
+2. A dialog 'Copy an existing notice' opens: 'Copies the wording, the purposes and every language rendition into this project as a fresh draft.' with a 'Notice to copy' list and a disabled 'Copy into this project' button.
 3. Every approved or published notice on the platform is offered, from any project and whoever wrote it - for example 'NTC-GAIT-2026 v1 — Gait Identification Study 2026'. Notices marked '(approved, not yet published)' come first. No draft notice is offered.
 4. A yellow box 'What comes across, and what does not' explains the legal approvals are not copied and each rendition must be re-approved. 'Copy into this project' becomes clickable.
 5. The dialog closes; a toast 'Copied into NTC-UAT-STUDY-02-2026' says 'It is a fresh draft. Review the wording, then approve and publish it.'
@@ -5513,12 +5513,12 @@
       </c>
       <c r="L48" s="11" t="inlineStr">
         <is>
-          <t>1. 'Upload a notice document' and 'Use an existing notice' are shown; there is NO 'New notice' button.
+          <t>1. 'Upload a notice document' and 'Copy an existing notice' are shown; there is NO 'New notice' button.
 2. The notice page opens. The header shows the 'Draft' badge but NO 'Edit' button.
 3. It is visible to the R&amp;D User and reads '... item(s) blocking publication:' followed by lines such as 'the purpose ... is draft, not activated' and 'the english text is not legally approved', each with a 'fix this' link. There is NO 'Publish this notice' button.
-4. The English wording is displayed read-only with 'Not legally approved — the project cannot be approved until it is'. There is NO 'Edit this rendition' button.
-5. Each purpose shows the 'Draft' status. There is NO 'Manage', NO 'Activate' and NO 'Narrow for this notice' button.
-6. The english row shows 'Not legally approved'. There is NO 'Add a rendition', NO 'Edit' and NO 'Approve' button.</t>
+4. The English wording is displayed read-only with 'Not legally approved — the project cannot be approved until it is'. There is NO 'Edit English text' button.
+5. Each purpose shows the 'Draft' status. There is NO 'Manage', NO 'Activate' and NO 'Customise for this notice' button.
+6. The english row shows 'Not legally approved'. There is NO 'Add language', NO 'Edit' and NO 'Approve' button.</t>
         </is>
       </c>
       <c r="M48" s="11" t="inlineStr">
@@ -5600,7 +5600,7 @@
 5. Click 'Proof'.
 6. Look at 'What happens next'.
 7. Scroll to the bottom of the page.
-8. Click 'Pending Approval' (at the top or in 'Next steps' - either one).
+8. Click 'Submit for approval' (at the top or in 'Next steps' - either one).
 9. Look at 'What happens next' again, and at the 'History' card.</t>
         </is>
       </c>
@@ -5611,8 +5611,8 @@
 3. The dialog closes; toast 'Approval uploaded' says 'The project can now move to pending approval.'
 4. Count 1; the row reads 'Security SEC-UAT-0001', 'Approved &lt;today&gt; · uploaded ... by Kavya Rao', a short hash, and a 'Proof' button.
 5. The file downloads and a toast 'Proof downloaded' says 'Hash matches the record.'
-6. 'Move to Pending Approval' has no warning lines and the 'Pending Approval' button is active (highlighted).
-7. A 'Next steps' card repeats 'Move to Pending Approval' with the same active 'Pending Approval' button, and under 'Other actions' the buttons from the top of the page (for example 'Upload approval') with the status badge. Nothing at the top of the page has gone.
+6. 'Moves the project to Pending Approval' has no warning lines and the 'Submit for approval' button is active (highlighted).
+7. A 'Next steps' card repeats 'Moves the project to Pending Approval' with the same active 'Submit for approval' button, and under 'Other actions' the buttons from the top of the page (for example 'Upload approval') with the status badge. Nothing at the top of the page has gone.
 8. Toast 'Moved to Pending Approval'. The status badge changes to 'Pending Approval' and the progress bar moves to its second step.
 9. 'What happens next' reads 'There is nothing for your role to do at this stage.' History shows 'In Draft → Pending Approval' by 'Kavya Rao (Rnd user)' with the time. The 'Edit' button is no longer shown in the page header.</t>
         </is>
@@ -5687,12 +5687,12 @@
       </c>
       <c r="K50" s="11" t="inlineStr">
         <is>
-          <t>1. On the 'Dashboard' look at 'Needs you today'.
+          <t>1. On the 'Dashboard' look at 'Needs attention'.
 2. Click 'Projects' in the sidebar, set 'Status' to 'Pending Approval', and click 'UAT Study 01'.
 3. Look at the 'What happens next' card.
-4. Read the warning lines under 'Move to Approved'.
-5. Under 'Move to In Draft' note the hint, then click the 'In Draft' button.
-6. Leave 'Reason' empty and click 'Confirm'.
+4. Read the warning lines under 'Moves the project to Approved'.
+5. Under 'Moves the project to In Draft' note the hint, then click the 'Return to draft' button.
+6. Leave 'Reason' empty and click 'Return to draft' in the panel.
 7. Click 'Cancel' in the panel.
 8. Click the 'Open the notice' link on the blocker line.</t>
         </is>
@@ -5701,9 +5701,9 @@
         <is>
           <t>1. A row 'Projects pending approval' shows a count of 1 or more.
 2. The project page opens with status 'Pending Approval'.
-3. It reads 'Currently Pending Approval.' and offers two rows: 'Move to Approved' (with the tag 'publishes the notice') and 'Move to In Draft'.
-4. Both DPO-side blockers are listed: 'The notice text is not legally approved - approve every language on the notice first' with a link 'Approve the notice', and 'The notice carries purposes that are not activated - activate them before approving' with a link 'Open the notice'. The 'Approved' button is disabled.
-5. The hint reads 'A reason is required and is recorded in the history.' A panel 'Move to In Draft' opens with a required 'Reason' box.
+3. It reads 'Currently Pending Approval.' and offers two rows: 'Moves the project to Approved' (with the tag 'publishes the notice' and an 'Approve project' button) and 'Moves the project to In Draft' (with a 'Return to draft' button).
+4. Both DPO-side blockers are listed: 'The notice text is not legally approved - approve every language on the notice first' with a link 'Approve the notice', and 'The notice carries purposes that are not activated - activate them before approving' with a link 'Open the notice'. The 'Approve project' button is disabled.
+5. The hint reads 'A reason is required and is recorded in the history.' A panel 'Return to draft' opens with a required 'Reason' box.
 6. The message 'A reason is required for this transition.' appears; the project stays 'Pending Approval'.
 7. The panel closes; status is still 'Pending Approval' and History has no new entry.
 8. The notice page 'NTC-UAT-STUDY-01-2026 · version 1' opens.</t>
@@ -5866,10 +5866,10 @@
       </c>
       <c r="K52" s="11" t="inlineStr">
         <is>
-          <t>1. On notice NTC-UAT-STUDY-01-2026 v1, find the 'Notice text' card and click 'Edit this rendition'.
-2. Add the extra sentence at the end of the text and click 'Save rendition'.
-3. In the 'Legal approval, per language' card click 'Add a rendition'.
-4. Choose Language 'Hindi', paste the Hindi text and click 'Save rendition'.
+          <t>1. On notice NTC-UAT-STUDY-01-2026 v1, find the 'Notice text' card and click 'Edit English text'.
+2. Add the extra sentence at the end of the text and click 'Save text'.
+3. In the 'Legal approval, per language' card click 'Add language'.
+4. Choose Language 'Hindi', paste the Hindi text and click 'Save text'.
 5. Look at the 'Publication checklist'.
 6. Read the English text, then click 'Approve' on the English row.
 7. Click the 'hindi' tab in 'Notice text', read it, then click 'Approve' on the Hindi row.
@@ -5878,9 +5878,9 @@
       </c>
       <c r="L52" s="11" t="inlineStr">
         <is>
-          <t>1. A dialog 'Edit english' opens: 'This exact text is hashed at publication and becomes the record of what was agreed to.' 'Language' is locked to English; 'Notice text' holds the current wording.
+          <t>1. A dialog 'Edit English text' opens: 'This exact text is hashed at publication and becomes the record of what was agreed to.' 'Language' is locked to English; 'Notice text' holds the current wording.
 2. Toast 'Rendition saved' says 'It must be legally approved before the notice can be published.' The new sentence is visible in the 'Notice text' card.
-3. A dialog 'Add a rendition' opens with 'Language' and 'Notice text'.
+3. A dialog 'Add language' opens with 'Language' and 'Notice text'.
 4. Toast 'Rendition saved'. The card now lists English and Hindi, both 'Not legally approved'. The 'Notice text' card shows language tabs (english / hindi).
 5. Lines 'the english text is not legally approved' and 'the hindi text is not legally approved' are shown; 'Languages' stat is 2, 'Approved' is 0.
 6. Toast 'english approved' says 'Its hash is what a data subject's consent will be matched against.' The row shows 'Approved' with 'Priya Menon' and the time.
@@ -5959,9 +5959,9 @@
       <c r="K53" s="11" t="inlineStr">
         <is>
           <t>1. Click the project name link at the top of the notice page ('UAT Study 01') to return to the project.
-2. Look at 'Move to Approved' in 'What happens next'.
-3. Click 'Approved'.
-4. Type the note and click 'Confirm'.
+2. Look at 'Moves the project to Approved' in 'What happens next'.
+3. Click 'Approve project'.
+4. Type the note and click 'Approve project' in the panel.
 5. Check the page header and progress bar.
 6. Look at the 'Notices' card.
 7. Look at the 'History' card.
@@ -5971,8 +5971,8 @@
       <c r="L53" s="11" t="inlineStr">
         <is>
           <t>1. The project page opens with status 'Pending Approval'.
-2. No warning lines remain; the 'Approved' button is active and the row carries the tag 'publishes the notice'.
-3. A panel 'Move to Approved' opens with a yellow warning: 'This publishes the project's notice. Its text and hash are frozen at that moment and cannot be edited afterwards - a correction requires a new version...' and an optional 'Note (optional)' box.
+2. No warning lines remain; the 'Approve project' button is active and the row carries the tag 'publishes the notice'.
+3. A panel 'Approve project' opens with a yellow warning: 'This publishes the project's notice. Its text and hash are frozen at that moment and cannot be edited afterwards - a correction requires a new version...' and an optional 'Note (optional)' box.
 4. Toast 'Moved to Approved' says 'The notice has been published and its text is now frozen.'
 5. Status badge 'Approved'; progress bar at the last step.
 6. 'NTC-UAT-STUDY-01-2026 v1' shows the badge 'Published' and '· published &lt;date/time&gt;'.
@@ -6063,7 +6063,7 @@
       <c r="L54" s="11" t="inlineStr">
         <is>
           <t>1. The notice page shows 'Published &lt;date&gt;. This text is frozen.' and the badge 'Published'.
-2. There is NO 'Edit' in the header, NO 'Edit this rendition', NO 'Manage', NO 'Activate', NO 'Narrow for this notice', NO 'Add a rendition' and NO 'Publish this notice'. The 'Publication checklist' card is not shown.
+2. There is NO 'Edit' in the header, NO 'Edit English text', NO 'Manage', NO 'Activate', NO 'Customise for this notice', NO 'Add language' and NO 'Publish this notice'. The 'Publication checklist' card is not shown.
 3. 'This notice is published. Its text and hashes are immutable — the database refuses an edit. To change anything, publish a new version.'
 4. It shows the recipient text fixed at publication (no longer 'Generated from the project's sites at publication').
 5. The 'Upload a notice document' dialog opens.
@@ -6880,11 +6880,11 @@
       </c>
       <c r="K63" s="11" t="inlineStr">
         <is>
-          <t>1. Open project 'UAT Study 01'. In the header click 'Use an existing notice', choose 'NTC-GAIT-2026 v1 — Gait Identification Study 2026' and click 'Copy into this project'.
+          <t>1. Open project 'UAT Study 01'. In the header click 'Copy an existing notice', choose 'NTC-GAIT-2026 v1 — Gait Identification Study 2026' and click 'Copy into this project'.
 2. Open the new notice. In 'Legal approval, per language' click 'Approve' on each language row.
 3. Click 'Publish this notice', then 'Publish and freeze'.
 4. Return to the project and look at the 'Notices' card.
-5. In a private window open the CIT 'new URL' saved in PRJ-19. Send a code to +91 90000 00001, type the relayed code and click 'Confirm and read the notice'.
+5. In a private window open the CIT 'new URL' saved in PRJ-19. Send a code to +91 90000 00001, type the relayed code and click 'Verify and continue'.
 6. Back in the console, on 'UAT Study 01' click 'New notice', then 'Set the code myself', type NTC-GAIT-2026 in 'Notice code', fill the other required fields and click 'Create notice'.</t>
         </is>
       </c>
@@ -6974,7 +6974,7 @@
 2. Look at the form before typing anything.
 3. Type +91 90000 00001 in 'Mobile number' and click 'Send the code'.
 4. Type only five digits in 'Six-digit code'.
-5. Complete the code with the one the coordinator relays and click 'Confirm and read the notice'.
+5. Complete the code with the one the coordinator relays and click 'Verify and continue'.
 6. Scroll to the card 'What are you agreeing to?'.
 7. Click 'I agree' on 'Gait model training' only.
 8. On 'Recording quality assurance' click 'I do not agree', then change your mind and click 'I agree'.
@@ -6985,17 +6985,17 @@
       </c>
       <c r="L64" s="11" t="inlineStr">
         <is>
-          <t>1. The page opens with a coloured banner showing 'Gait Identification Study 2026' and 'CIT'. A step bar shows 'Your details', 'Confirm', 'The notice', 'Done' with 'Your details' current. A card 'Your details' says consent is recorded against your account so you can read and withdraw it.
+          <t>1. The page opens with a coloured banner showing 'Gait Identification Study 2026' and 'CIT'. A step bar shows 'Your details', 'Confirm', 'The notice', 'Done' with 'Your details' current. A card 'Your details' says 'Confirm your mobile number or email to read the notice and make your choices.' Because this notice is in more than one language, a 'Read the notice in' drop-down showing 'English' is above 'Send my code to'.
 2. Under 'Send my code to' the 'Mobile' option is already selected ('Email' is the other option). There is ONE box, 'Mobile number', with the hint 'The one your account is registered with.' There is no box for a name, date of birth or a second contact. 'Send the code' is greyed out. Below it: 'No account yet? Create one — it takes a minute, and this page will be waiting when you come back.'
-3. The card changes to 'Confirm your mobile': 'We have sent a six-digit code to +91 90000 00001. It expires in ten minutes.' The step bar moves to 'Confirm'.
-4. The box accepts digits only, and 'Confirm and read the notice' stays greyed out.
+3. The card changes to 'Confirm your mobile': 'We have sent a six-digit code to +91 90000 00001. It expires in ten minutes.' Below the code box are 'Send a new code' and 'Use a different contact'. The step bar moves to 'Confirm'.
+4. The box accepts digits only, and 'Verify and continue' stays greyed out.
 5. No date-of-birth question appears (Anjali already gave one). The step bar moves to 'The notice'. A 'Read this in' dropdown shows 'English'. A card 'The notice' shows the notice text (starting 'NOTICE UNDER SECTION 5, DIGITAL PERSONAL DATA PROTECTION ACT 2023'), then 'Data Protection Officer:', 'Who else sees your data:', the links 'Exercise your rights', 'Withdraw consent', 'Complain to the Data Protection Board', and 'Version 1 · content hash …'.
 6. Two purposes are listed: 'Gait model training' and 'Recording quality assurance'. Each shows a description, 'What this allows:', 'Data collected:' and 'Kept for:', and two buttons of the same size, 'I agree' and 'I do not agree'. NEITHER button is selected on either purpose. 'Record my choices' is greyed out and the line 'Answer every purpose above, or decline the whole notice.' is shown. 'Decline everything' is active and the same size as 'Record my choices'.
 7. That choice is highlighted. 'Record my choices' is still greyed out and the line 'Answer every purpose above, or decline the whole notice.' is still shown.
 8. The highlight moves from 'I do not agree' to 'I agree'. 'Record my choices' becomes active and the 'Answer every purpose above…' line disappears.
-9. The step bar moves to 'Done'. A green tick and the heading 'Your choices are recorded' appear, with 'We have sent you a receipt. You can review or withdraw your consent at any time - withdrawing is as easy as this was.' Below: 'Your reference:' followed by a long code (write it down), and the links 'Review your consents' and 'Your rights'.
+9. The step bar moves to 'Done'. A green tick and the heading 'Your choices are recorded' appear, with 'A receipt is on its way to you. You can review or withdraw your consent at any time - withdrawing is as easy as this was.' Below: 'Your reference:' followed by a long code (write it down), and the links 'Review your consents' and 'Your rights'.
 10. A receipt message for this consent is in the outbox.
-11. The portal page 'Your consents' opens, signed in as Anjali, with a card 'Gait Identification Study 2026', status 'Consented' and the line 'You agreed to 2 of 2 purpose(s).'</t>
+11. The portal page 'My consents' opens, signed in as Anjali, with a card 'Gait Identification Study 2026', status 'Consented' and the line 'You agreed to both purposes.'</t>
         </is>
       </c>
       <c r="M64" s="11" t="inlineStr">
@@ -7075,11 +7075,11 @@
           <t>1. Open the CIT consent link and look at the 'Your details' card.
 2. With 'Mobile' selected, type +91 98100 00002 in 'Mobile number' and click 'Send the code'.
 3. Ask the coordinator to check the test outbox for +91 98100 00002.
-4. Type 123456 in 'Six-digit code' and click 'Confirm and read the notice'.
+4. Type 123456 in 'Six-digit code' and click 'Verify and continue'.
 5. Reload the page. Under 'Send my code to' select 'Email', type tester09@example.org in 'Email address' and click 'Send the code'.
 6. Reload the page. With 'Mobile' selected type +91 90000 00001 (a registered number) and click 'Send the code'.
-7. Type 123456 (not the code that was sent) and click 'Confirm and read the notice'.
-8. Clear the box, type the correct code relayed by the coordinator and click 'Confirm and read the notice'.</t>
+7. Type 123456 (not the code that was sent) and click 'Verify and continue'.
+8. Clear the box, type the correct code relayed by the coordinator and click 'Verify and continue'.</t>
         </is>
       </c>
       <c r="L65" s="11" t="inlineStr">
@@ -7175,7 +7175,7 @@
 3. Type only the mobile code the coordinator relays.
 4. Type the email code as well and click 'Confirm and sign in'.
 5. On the 'Your details' card select 'Email' under 'Send my code to', type tester01@example.org in 'Email address' and click 'Send the code'.
-6. Type the code the coordinator relays and click 'Confirm and read the notice'.
+6. Type the code the coordinator relays and click 'Verify and continue'.
 7. In 'Read this in' choose 'हिन्दी'.
 8. Switch 'Read this in' to 'English', then back to 'हिन्दी'.
 9. With Hindi showing, click 'I agree' on 'Gait model training' and 'I do not agree' on 'Recording quality assurance', then click 'Record my choices'.
@@ -7193,7 +7193,7 @@
 7. The notice text changes to Hindi (it starts 'धारा 5, डिजिटल व्यक्तिगत डेटा संरक्षण अधिनियम 2023'). The purposes and the 'I agree' / 'I do not agree' buttons are still shown.
 8. The text switches each time without any error message. Hindi is showing at the end.
 9. The Done step shows 'Your choices are recorded' and 'Your reference:' with a code.
-10. 'Your consents' opens with a card 'Gait Identification Study 2026' whose small line reads 'NTC-GAIT-2026 v1 · hindi · &lt;date and time&gt;', status 'Partial', and 'You agreed to 1 of 2 purpose(s).'</t>
+10. 'My consents' opens with a card 'Gait Identification Study 2026' whose small line reads 'NTC-GAIT-2026 v1 · hindi · &lt;date and time&gt;', status 'Partial', and 'You agreed to 1 of 2 purposes.'</t>
         </is>
       </c>
       <c r="M66" s="11" t="inlineStr">
@@ -7274,7 +7274,7 @@
 2. Click 'Create account' with every field empty.
 3. Fill in 'Full name', 'Mobile number' and 'Date of birth' from the test data, leave 'Email address' empty and click 'Create account'.
 4. Type the code the coordinator relays and click 'Confirm and sign in'.
-5. In the same browser window open the CIT consent link. Leave 'Mobile' selected, type +91 98100 00022, click 'Send the code', type the relayed code and click 'Confirm and read the notice'.
+5. In the same browser window open the CIT consent link. Leave 'Mobile' selected, type +91 98100 00022, click 'Send the code', type the relayed code and click 'Verify and continue'.
 6. Without answering any purpose, click 'Decline everything'.
 7. Click 'Review your consents'.
 8. Click 'See what you were asked'.</t>
@@ -7285,10 +7285,10 @@
           <t>1. The page 'Create your account' opens with 'Full name', 'Mobile number', 'Email address' (hint starts 'Optional.') and 'Date of birth', and a 'Create account' button.
 2. Nothing is sent. Messages appear under the fields, including 'Enter your full name' and 'Enter your date of birth'.
 3. 'Confirm your contacts' opens with 'If that number is new to us, a code has gone to your mobile. Enter it to finish.' and only one box, 'Code sent to your mobile'.
-4. You are signed in and 'Your consents' opens with the empty message 'No consent records' / 'When you agree to a notice, it will appear here.'
+4. You are signed in and 'My consents' opens with the empty message 'No consent records' / 'When you agree to a notice, it will appear here.'
 5. The notice opens with the two purposes, neither pre-selected.
 6. The Done step shows a grey cross, the heading 'You have declined' and 'Nothing will be collected from you for this project. You can come back to this link if you change your mind.' plus 'Your reference:' with a code. It does not look like an error.
-7. The card 'Gait Identification Study 2026' shows status 'Declined' and 'You were asked about 2 purpose(s) and agreed to none.' The first button reads 'See what you were asked'. There is no 'Withdraw everything' button.
+7. The card 'Gait Identification Study 2026' shows status 'Declined' and 'You were asked about 2 purposes and agreed to none.' The first button reads 'See what you were asked'. There is no 'Withdraw everything' button.
 8. Both purposes are listed with the badge 'Declined' and no 'Withdraw just this one' button.</t>
         </is>
       </c>
@@ -7367,13 +7367,13 @@
       <c r="K68" s="11" t="inlineStr">
         <is>
           <t>1. Open the CIT consent link. On the 'Your details' card select 'Email' under 'Send my code to', type dcoadmin@cmp.local in 'Email address' and click 'Send the code'.
-2. Type the code the coordinator relays and click 'Confirm and read the notice'.
+2. Type the code the coordinator relays and click 'Verify and continue'.
 3. Click 'Save and continue' with the field empty.
 4. Enter tomorrow's date in 'Date of birth' and click 'Save and continue'.
 5. Enter 21/07/1985 and click 'Save and continue'.
 6. Click 'I agree' on both purposes and click 'Record my choices'.
 7. Click 'Review your consents'.
-8. Open the CIT consent link again in a new private window, identify with dcoadmin@cmp.local and the new code, and click 'Confirm and read the notice'.</t>
+8. Open the CIT consent link again in a new private window, identify with dcoadmin@cmp.local and the new code, and click 'Verify and continue'.</t>
         </is>
       </c>
       <c r="L68" s="11" t="inlineStr">
@@ -7384,7 +7384,7 @@
 4. The message 'Date of birth must be in the past' appears (or the date picker will not allow a future date). The notice is not shown.
 5. The step bar moves to 'The notice' and the notice with its two purposes is shown.
 6. The Done step shows 'Your choices are recorded' with a reference.
-7. 'Your consents' shows the card 'Gait Identification Study 2026' with status 'Consented' and 'You agreed to 2 of 2 purpose(s).'
+7. 'My consents' shows the card 'Gait Identification Study 2026' with status 'Consented' and 'You agreed to both purposes.'
 8. The notice opens directly; the date-of-birth question is NOT asked again. Close the tab without recording anything.</t>
         </is>
       </c>
@@ -7555,13 +7555,13 @@
       <c r="K70" s="11" t="inlineStr">
         <is>
           <t>1. Open the CIT consent link. On the 'Your details' card select 'Email' under 'Send my code to', type tester07@example.org in 'Email address' and click 'Send the code'.
-2. Type the relayed code and click 'Confirm and read the notice'.
+2. Type the relayed code and click 'Verify and continue'.
 3. Enter 01/06/2011 and click 'Save and continue'.
 4. Click 'I agree' on both purposes and click 'Record my choices'.
 5. Click 'Decline everything'.
 6. Look over the whole page, including the notice links.
 7. Open http://localhost:3001/my-consents in the same window.
-8. Click 'Your profile' in the sidebar and look at 'Date of birth'.
+8. Click your name at the top right to open the account menu, click 'My profile' and look at 'Date of birth'.
 9. In the console, as the DPO, open 'Consents' and look for this account's name.</t>
         </is>
       </c>
@@ -7573,7 +7573,7 @@
 4. A red message appears at the top of the page: 'We cannot register or record consent for a person under eighteen. If you think your date of birth is wrong, contact the Privacy Office.' The page stays on the notice. No Done step and no reference are shown.
 5. The same refusal message appears. There is no 'You have declined' screen: a child's refusal is not recorded either.
 6. Nothing offers a parent or guardian route: no link, button, form or contact field for a guardian.
-7. 'Your consents' shows 'No consent records'.
+7. 'My consents' shows 'No consent records'.
 8. It shows the date entered, marked as under 18. Nothing on the page offers a way for a parent or guardian to consent. The badge reads 'Under 18 — we cannot record consent from you'.
 9. There is no consent record for this account.</t>
         </is>
@@ -7749,12 +7749,12 @@
       </c>
       <c r="L72" s="11" t="inlineStr">
         <is>
-          <t>1. After 'Send me a code' a blue box 'Check your messages' says 'If tester01@example.org is registered with us, a six-digit code is on its way. It expires in ten minutes.' After 'Verify' the page 'Your consents' opens and 'My consents' is highlighted in the sidebar.
-2. Description: 'Everything you have agreed to, the exact wording you were shown, and who it has been shared with. You can withdraw at any time.' The card shows 'NTC-GAIT-2026 v1 · hindi · &lt;date and time&gt;', status 'Partial', 'You agreed to 1 of 2 purpose(s).' and the buttons 'See what you agreed to', 'What was recorded', 'Withdraw everything' and 'Ask about this consent'.
+          <t>1. After 'Send me a code' a blue box 'Check your messages' says 'If tester01@example.org is registered with us, a six-digit code is on its way. It expires in ten minutes.' After 'Verify' the page 'My consents' opens and 'My consents' is highlighted in the sidebar.
+2. Description: 'Everything you have agreed to, the exact wording you were shown, and who it has been shared with. You can withdraw at any time.' The card shows 'NTC-GAIT-2026 v1 · hindi · &lt;date and time&gt;', status 'Partial', 'You agreed to 1 of 2 purposes.' and the buttons 'See what you agreed to', 'What was recorded', 'Withdraw everything' and 'Ask about this consent'.
 3. The button changes to 'Hide details'. 'Gait model training' shows the badge 'Consented' and a 'Withdraw just this one' button; 'Recording quality assurance' shows 'Declined' and no withdraw button. Each shows 'Data:' and 'Kept for:'.
 4. A box shows 'Served &lt;date and time&gt;', a green 'Integrity verified', the Hindi notice text exactly as it was shown at the link (starting 'धारा 5'), and 'Hash recorded at capture:' with a code.
 5. A panel 'What was recorded' opens ('The same record the Privacy Office sees, for this consent and every change to it. Oldest first.') listing at least the consent being given. The button now reads 'Hide the record'.
-6. Before any export (CON-14): 'Not shared with anyone' / 'No export containing your record has been generated.' After CON-14: an entry naming the processor 'SEED' with the project name and date.
+6. Before any export (CON-14): 'No sharing recorded here' / 'This lists every file of your details this platform has sent to a processor. None has been sent.' After CON-14: an entry naming the processor 'SEED' with the project name and date.
 7. Both sections close. Nothing has changed: the status is still 'Partial'.</t>
         </is>
       </c>
@@ -7829,7 +7829,7 @@
       <c r="K73" s="11" t="inlineStr">
         <is>
           <t>1. Open http://localhost:3001/sign-in. Under 'Sign in with' select 'Email', type dcoadmin@cmp.local in 'Email address' and click 'Send me a code'. Then type the code the coordinator relays into 'Six-digit code' and click 'Verify'.
-2. On the card 'Gait Identification Study 2026' (status 'Consented', 'You agreed to 2 of 2 purpose(s).') click 'Withdraw everything'.
+2. On the card 'Gait Identification Study 2026' (status 'Consented', 'You agreed to both purposes.') click 'Withdraw everything'.
 3. Click 'Keep my consent'.
 4. Click 'Withdraw everything' again, then 'Withdraw'.
 5. Look at the card.
@@ -7840,11 +7840,11 @@
       </c>
       <c r="L73" s="11" t="inlineStr">
         <is>
-          <t>1. After 'Send me a code' a blue box 'Check your messages' says 'If dcoadmin@cmp.local is registered with us, a six-digit code is on its way. It expires in ten minutes.' After 'Verify' the page 'Your consents' opens and 'My consents' is highlighted in the sidebar.
+          <t>1. After 'Send me a code' a blue box 'Check your messages' says 'If dcoadmin@cmp.local is registered with us, a six-digit code is on its way. It expires in ten minutes.' After 'Verify' the page 'My consents' opens and 'My consents' is highlighted in the sidebar.
 2. A warning 'Withdraw all purposes?' appears: 'Processing for these purposes will stop. Data already collected is not deleted by a withdrawal — if you want it erased, make a rights request.' with the buttons 'Withdraw' and 'Keep my consent'.
 3. The warning closes and the status is still 'Consented'.
 4. A notice 'Withdrawal recorded' appears with 'Stopped: Gait model training, Recording quality assurance.' (the order may differ).
-5. The status is 'Withdrawn' and the text reads 'You were asked about 2 purpose(s) and agreed to none.' The 'Withdraw everything' button is gone.
+5. The status is 'Withdrawn' and the text reads 'You were asked about 2 purposes and agreed to none.' The 'Withdraw everything' button is gone.
 6. Both purposes show 'Declined'. The notice box still shows the English text originally served, with 'Integrity verified'.
 7. The list shows the consent and, after it, the withdrawal.
 8. A withdrawal confirmation message is present.</t>
@@ -7925,7 +7925,7 @@
 2. Look below the note.
 3. Click 'Add it now' in the note.
 4. Click 'My requests' in the sidebar.
-5. Click 'Your profile' in the sidebar.
+5. Click your name at the top right to open the account menu, then click 'My profile'.
 6. Click the 'withdraw a consent' link on that card.
 7. Do not enter a date. Click 'Sign out'.
 8. Only if the coordinator supplied an account with no date of birth and an active consent: sign in as it, click 'Withdraw everything' on its card, then 'Withdraw'.</t>
@@ -7933,12 +7933,12 @@
       </c>
       <c r="L74" s="11" t="inlineStr">
         <is>
-          <t>1. 'Your consents' opens — it is NOT replaced by a date-of-birth question. A blue note 'We need your date of birth' reads 'You can withdraw a consent or make a request without it, but we need it before you give a new consent.' with a link 'Add it now'.
+          <t>1. 'My consents' opens — it is NOT replaced by a date-of-birth question. A blue note 'We need your date of birth' reads 'You can withdraw a consent or make a request without it, but we need it before you give a new consent.' with a link 'Add it now'.
 2. The page works normally; with no consents it shows 'No consent records'.
-3. 'Your profile' opens and shows the card 'Your date of birth' with 'Save and continue'. Do not enter a date.
+3. 'My profile' opens and shows the card 'Your date of birth' with 'Save and continue'. Do not enter a date.
 4. The requests page opens normally, with the same 'We need your date of birth' note.
 5. The page is replaced by the card 'Your date of birth' with 'Save and continue', and the line 'You can still withdraw a consent or make a request without it.'
-6. 'Your consents' opens again, with the note.
+6. 'My consents' opens again, with the note.
 7. You are signed out; no date of birth was saved.
 8. 'Withdrawal recorded' appears and the card shows 'Withdrawn'. No date of birth was asked for at any point.</t>
         </is>
@@ -8110,7 +8110,7 @@
           <t>1. Sign in as dco@cmp.local and click 'Consents'.
 2. Open one of them.
 3. Sign out, sign in as rco@cmp.local and click 'Consents'.
-4. As the RCO click 'Projects', type 'Gait Identification' in 'Search' (the list updates as you type), open 'Gait Identification Study 2026', click 'Generate export' and then 'Generate the export'.
+4. As the RCO click 'My projects', type 'Gait Identification' in 'Search' (the list updates as you type), open 'Gait Identification Study 2026', click 'Generate export' and then 'Generate the export'.
 5. Sign out, sign in as rnd@cmp.local and look at the sidebar.
 6. Type http://localhost:3000/consents in the address bar, then http://localhost:3000/exports.
 7. Sign out, sign in as admin@cmp.local and look at the sidebar; then open http://localhost:3000/consents.</t>
@@ -8878,11 +8878,11 @@
       </c>
       <c r="L84" s="11" t="inlineStr">
         <is>
-          <t>1. After 'Send me a code' a blue box 'Check your messages' says 'If +91 90000 00001 is registered with us, a six-digit code is on its way. It expires in ten minutes.' After 'Verify' the page 'Your consents' opens and 'My consents' is highlighted in the sidebar.
+          <t>1. After 'Send me a code' a blue box 'Check your messages' says 'If +91 90000 00001 is registered with us, a six-digit code is on its way. It expires in ten minutes.' After 'Verify' the page 'My consents' opens and 'My consents' is highlighted in the sidebar.
 2. At least one entry names the processor 'SEED' with 'Gait Identification Study 2026 · &lt;date and time&gt;' of the export.
 3. Both purposes show 'Consented', each with a 'Withdraw just this one' button.
 4. The notice 'Withdrawal recorded' / 'Stopped: Recording quality assurance.' appears.
-5. The line reads 'You agreed to 1 of 2 purpose(s).' 'Recording quality assurance' now shows 'Declined' and 'Gait model training' still shows 'Consented'. The status badge reads 'Partial', not 'Withdrawn'.
+5. The line reads 'You agreed to 1 of 2 purposes.' 'Recording quality assurance' now shows 'Declined' and 'Gait model training' still shows 'Consented'. The status badge reads 'Partial', not 'Withdrawn'.
 6. A 'Withdraw just this one' button is still offered under 'Gait model training' (and 'Withdraw everything' on the card), so the rest can be withdrawn as easily as consent was given (s.6(4)).
 7. The list shows the original consent followed by the withdrawal.
 8. A withdrawal confirmation message is present.
@@ -8977,7 +8977,7 @@
       <c r="L85" s="11" t="inlineStr">
         <is>
           <t>1. A 'Check your messages' box appears after the first click. After 'Verify' you are signed in and the 'My consents' page opens; the sidebar shows 'My consents' and 'My requests'.
-2. The page 'Your requests' opens with the text 'Ask for access to your data, a correction, erasure, or raise a grievance...' and a 'Make a request' button at the top right. Lower down is the card 'Somebody to act for you'.
+2. The page 'My requests' opens with the text 'Ask for access to your data, a correction or erasure, or raise a complaint...' and a 'Make a request' button at the top right. At the foot of the page a line says naming someone to act for you is under 'My nominations'.
 3. A dialog titled 'Make a request' opens with the line 'You are signed in, so this counts as verified and the clock starts now.' It has 'What are you asking for', 'About', 'Your request' and a 'Send the request' button.
 4. A blue note under it reads 'A summary of the personal data we hold about you, what we do with it, and who it has been shared with.'
 5. The dialog closes. A message 'Recorded as RR-YYYY-NNNNNN' appears with 'You will hear from us by &lt;date&gt;.' Write down the reference (RR-A).
@@ -9243,7 +9243,7 @@
       <c r="K88" s="11" t="inlineStr">
         <is>
           <t>1. In 'My requests' click 'Make a request', choose 'Access (s.11)', type 'short' in 'Your request' and click 'Send the request'.
-2. In the same dialog change 'What are you asking for' to 'Grievance (s.13)'.
+2. In the same dialog change 'What are you asking for' to 'Complaint (grievance) (s.13)'.
 3. In the private window open http://localhost:3001/rights. In 'Make a request' type 'ab' in 'The email or mobile you registered with', a full sentence in 'Your request', and click 'Send the request'.
 4. Click 'Already have a reference and a code? Verify it here.'
 5. Type 12345 in 'Your reference' and 12ab in 'The code we sent'. Click 'Confirm it is me'.
@@ -9545,7 +9545,7 @@
       </c>
       <c r="L91" s="11" t="inlineStr">
         <is>
-          <t>1. The Dashboard opens, signed in as Priya Menon (DPO). The sidebar shows 'Rights requests' under 'Oversight'.
+          <t>1. The Dashboard opens, signed in as Priya Menon (DPO). The sidebar shows 'Rights requests' under 'Your work'.
 2. The page 'Rights requests' opens with the text 'Access, correction, erasure and grievance - sections 11 to 14...' and a 'Log a request received by email' button. Filters 'Status', 'Kind', 'Clock' and 'Tickets' are shown, and the columns 'Reference', 'Who', 'Kind', 'Status', 'Received', 'Due'.
 3. Only access requests are listed. RR-A shows 'Anjali Verma' and her contact, 'Access · s.11', 'Received', its received time, and a due date with 'N days left' under it.
 4. The heading is RR-A, the line under it reads 'Access · s.11 · Portal', and the badges 'Access · s.11' and 'Received' are at the right. The details show 'Who' (Anjali Verma with email and mobile), 'Contact given', 'Received' and 'Acknowledged', followed by her request text. Cards 'Clock' and 'The path, and where it can end early' follow.
@@ -9750,10 +9750,10 @@
       </c>
       <c r="L93" s="11" t="inlineStr">
         <is>
-          <t>1. It reads 'Third-party data removed. The DPO signs off - nothing releases automatically. An access response is a file she downloads from her own account.' There is no yellow warning, and 'Outcome' shows 'Complete'.
+          <t>1. It reads 'Third-party data removed. The DPO signs off - nothing releases automatically. An access response is a file the requester downloads from their own account.' There is no yellow warning, and 'Outcome' shows 'Complete'.
 2. 'Release and close' is greyed out.
 3. The file is listed with its size and a small X to remove it.
-4. The message 'Released and closed' with 'She has been told; 1 file released with the response.' appears. The header badge reads 'Complete'. A 'Response' card shows 'Complete · &lt;date&gt; · downloadable by her until &lt;date&gt;', the response text, a 'Download the file' button and 'Released with the response' listing access-extract.pdf.
+4. The message 'Released and closed' with 'The requester has been told; 1 file released with the response.' appears. The header badge reads 'Complete'. A 'Response' card shows 'Complete · &lt;date&gt; · downloadable by the requester until &lt;date&gt;', the response text, a 'Download the file' button and 'Released with the response' listing access-extract.pdf.
 5. It reads 'Closed. Disagreement with the outcome is a grievance - a new request linked to this one.'
 6. A mail telling her the response to RR-A is ready is in the outbox, with a summary including what SEED returned.
 7. The badge reads 'Complete'. A box 'Our response · &lt;date&gt;' shows the text. 'Files released with this response' lists access-extract.pdf with 'Download'. Buttons 'Download the file' (with 'until &lt;date&gt;') and 'Dispute this response' are shown, with the note about the Data Protection Board.
@@ -9839,17 +9839,17 @@
 2. In '4 · Withdrawal, or erasure?' read the yellow box.
 3. Check 'This is a request for' shows 'Erasure (s.12(3))' and click 'Confirm classification'.
 4. Look at 'What happens next'.
-5. Click 'She means erasure'.
+5. Click 'They mean erasure'.
 6. In 'What happens next' click 'In progress'.
 7. In Browser A, on 'My requests', make a new request: 'Erasure (s.12(3))' with the RR-W text. Note its reference (RR-W).
-8. In Browser B open RR-W and click 'She meant withdrawal'.
+8. In Browser B open RR-W and click 'They meant withdrawal'.
 9. In Browser A reload 'My requests' and look at RR-W, then open 'My consents'.</t>
         </is>
       </c>
       <c r="L94" s="11" t="inlineStr">
         <is>
           <t>1. The line under the heading reads 'Erasure · s.12(3) · Portal'. The cards include '4 · Withdrawal, or erasure?', '7–9 · Holders, instructions, confirmations' and '5–6 · Scope determined; inside the one-year floor?'.
-2. It is headed 'Does she mean erasure, or withdrawal?' and explains 'Withdrawal stops future processing and is hers to do from her consent record... Confirm which before anything is deleted.' with buttons 'She means erasure' and 'She meant withdrawal'.
+2. It is headed 'Does the requester mean erasure, or withdrawal?' and explains 'Withdrawal stops future processing, and the requester can do it from their consent record... Confirm which before anything is deleted.' with buttons 'They mean erasure' and 'They meant withdrawal'.
 3. 'Classified' appears; the card shows 'Classified as erasure on &lt;date&gt;.'
 4. 'Move to in progress' carries the warning 'Whether she means withdrawal or erasure is not yet confirmed' and 'In progress' is greyed out.
 5. The message 'Erasure confirmed' appears, the yellow box disappears and the card reads 'Erasure confirmed on &lt;date&gt;.'
@@ -9861,7 +9861,7 @@
       </c>
       <c r="M94" s="11" t="inlineStr">
         <is>
-          <t>Work on an erasure cannot start until the DPO confirms intent; 'She means erasure' unblocks it; 'She meant withdrawal' closes the request as 'Handled as withdrawal' with the explanation, without touching her consents.</t>
+          <t>Work on an erasure cannot start until the DPO confirms intent; 'They mean erasure' unblocks it; 'They meant withdrawal' closes the request as 'Handled as withdrawal' with the explanation, without touching her consents.</t>
         </is>
       </c>
       <c r="N94" s="16" t="n"/>
@@ -10032,20 +10032,20 @@
 4. Change 'Decision' to 'Retain - a floor binds, erased when it passes'. Set 'Until' to yesterday, type the retain basis and click 'Record the decision'.
 5. Set 'Until' to the date next year and click 'Record the decision'.
 6. Click 'Apply'.
-7. Change 'Decision' to 'Erase - the asset holds only her', replace the basis with the erase basis and click 'Record the decision'.
+7. Change 'Decision' to 'Erase - the asset holds only the requester', replace the basis with the erase basis and click 'Record the decision'.
 8. Open 'Decision' on asset A once more without changing it.</t>
         </is>
       </c>
       <c r="L96" s="11" t="inlineStr">
         <is>
-          <t>1. A blue note reads 'Consent artefacts are never erased. They are the evidence that past processing was lawful...' and the card says 'No scope yet. Derive it from the records she appears in.' with a button 'Derive from asset_consent'.
-2. 'Scope derived' with '2 appearances of her in collected assets.' appears. Two rows show: asset A with its type badge and 'only her', and asset B with a warning badge 'holds 1 other person'. Each row names the project, source (SRC-SRIB-SE), 'held by SRIB' and the collection date.
-3. 'Decision' shows 'Erase - the asset holds only her'. 'Basis' is empty and 'Record the decision' is greyed out.
+          <t>1. A blue note reads 'Consent artefacts are never erased. They are the evidence that past processing was lawful...' and the card says 'No scope yet. Derive it from the records the requester appears in.' with a button 'Derive from asset_consent'.
+2. 'Scope derived' with '2 appearances of the requester in collected assets.' appears. Two rows show: asset A with its type badge and 'only the requester', and asset B with a warning badge 'holds 1 other person'. Each row names the project, source (SRC-SRIB-SE), 'held by SRIB' and the collection date.
+3. 'Decision' shows 'Erase - the asset holds only the requester'. 'Basis' is empty and 'Record the decision' is greyed out.
 4. An 'Until' field appeared when Retain was chosen. The message 'Not recorded' with 'A retention floor in the past is not a floor' appears.
 5. 'Decision recorded' appears. The row shows 'decided: retain', 'Retained until &lt;date&gt;', the basis in quotes, and an 'Apply' button.
 6. The message 'Not applied' with 'Retained until &lt;date&gt;. The floor binds even against her request; it is applied when it passes.' appears. The row still shows 'decided: retain' and nothing is quarantined.
 7. The 'Until' field disappears. 'Decision recorded' appears and the row shows 'decided: erase' with the new basis. Do not click 'Apply' yet (RGT-14).
-8. The four options are 'Erase - the asset holds only her', 'Redact - remove her, keep the others', 'Retain - a floor binds, erased when it passes' and 'Quarantine - removal cannot be assured; the DPO decides'.</t>
+8. The four options are 'Erase - the asset holds only the requester', 'Redact - remove the requester, keep the others', 'Retain - a floor binds, erased when it passes' and 'Quarantine - removal cannot be assured; the DPO decides'.</t>
         </is>
       </c>
       <c r="M96" s="11" t="inlineStr">
@@ -10119,8 +10119,8 @@
       <c r="K97" s="11" t="inlineStr">
         <is>
           <t>1. On the asset B row look at the badges, the 'Decision' field and the text beside 'Record the decision'.
-2. Open 'Decision' and try to choose 'Erase - the asset holds only her'.
-3. Keep 'Redact - remove her, keep the others', type the redact basis and click 'Record the decision'.
+2. Open 'Decision' and try to choose 'Erase - the asset holds only the requester'.
+3. Keep 'Redact - remove the requester, keep the others', type the redact basis and click 'Record the decision'.
 4. Click 'Apply'.
 5. Read the list of stores under the row.
 6. Look at the buttons on the row.</t>
@@ -10128,7 +10128,7 @@
       </c>
       <c r="L97" s="11" t="inlineStr">
         <is>
-          <t>1. The row carries the warning badge 'holds 1 other person'. 'Decision' is preset to 'Redact - remove her, keep the others'. Beside the button: 'Erase is not offered: deleting this asset would erase the other people's validly given consent.'
+          <t>1. The row carries the warning badge 'holds 1 other person'. 'Decision' is preset to 'Redact - remove the requester, keep the others'. Beside the button: 'Erase is not offered: deleting this asset would erase the other people's validly given consent.'
 2. The Erase option is greyed out and cannot be chosen.
 3. 'Decision recorded' appears; the row shows 'decided: redact' and an 'Apply' button.
 4. The message 'Quarantined' with 'It is out of use now; it is erased when every store holding it is confirmed.' appears. The row now shows the badge 'quarantined - being redacted'; the decision fields are gone.
@@ -10225,7 +10225,7 @@
 4. The message 'Tried again' with 'Something is still outstanding; it is shown below.' appears. The lines and the 'quarantined - being erased' badge are unchanged.
 5. The 'Decision' and 'Basis' fields are gone for asset A; the decision stands.
 6. The request is still 'Awaiting holders'; 'Move to collating' is still blocked by 'A holder has not returned its ticket - escalate once before responding partial'.
-7. RR-E shows 'Awaiting holders'. Nothing on her card says her data has been erased.</t>
+7. RR-E shows 'Waiting for responses'. Nothing on her card says her data has been erased.</t>
         </is>
       </c>
       <c r="M98" s="11" t="inlineStr">
@@ -10256,12 +10256,12 @@
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>In-house respondent answers the ticket on 'Tickets for you' (thread, attach file, return)</t>
+          <t>In-house respondent answers the ticket on 'My tasks' (thread, attach file, return)</t>
         </is>
       </c>
       <c r="D99" s="11" t="inlineStr">
         <is>
-          <t>Console - Tickets for you; request detail - ticket thread</t>
+          <t>Console - My tasks; request detail - ticket thread</t>
         </is>
       </c>
       <c r="E99" s="11" t="inlineStr">
@@ -10305,13 +10305,13 @@
         <is>
           <t>1. In Browser C sign in to http://localhost:3000 as rco@cmp.local with password SeedPassw0rd!2026 (enter the relayed code if 'Verify it is you' appears).
 2. Type http://localhost:3000/requests in the address bar.
-3. Click 'Tickets for you'.
+3. Click 'My tasks'.
 4. Click 'Respond'.
 5. Type the question, choose srib-inventory.csv under 'Attach a file' and click 'Send' (leave the checkbox unticked).
 6. In Browser B (DPO) open 'Rights requests' and then RR-E.
 7. Click 'Thread' on the SRIB row.
 8. Type the DPO reply and click 'Send'. Close the dialog.
-9. In Browser C reload 'Tickets for you'.
+9. In Browser C reload 'My tasks'.
 10. Type the return text, attach srib-deletion-log.pdf and tick 'This is my return - close the ticket with it'.
 11. Click 'Return the ticket'.
 12. In Browser B reload RR-E.
@@ -10320,9 +10320,9 @@
       </c>
       <c r="L99" s="11" t="inlineStr">
         <is>
-          <t>1. Meera Iyer's dashboard opens. Under 'You' the sidebar shows 'Tickets for you' with a count; there is no 'Rights requests' link.
+          <t>1. Meera Iyer's dashboard opens. Under 'Your work' the sidebar shows 'My tasks' with a count; there is no 'Rights requests' link.
 2. A box 'Not part of your account' says 'This section belongs to a different role, so there is nothing here for you...' with a 'Back to your dashboard' button. No requests are shown.
-3. The page 'Tickets for you' shows tiles 'Open', 'Overdue', 'Due within 7 days', 'Unread from the Privacy Office' and a section 'Open · 1'. The ticket card shows RR-E, 'Erasure · s.12(3)', 'Issued', 'For SRIB · about Anjali Verma · issued &lt;date&gt;', the due date and an 'Instruction'.
+3. The page 'My tasks' shows tiles 'Open', 'Overdue', 'Due within 7 days', 'Unread from the Privacy Office' and a section 'Open · 1'. The ticket card shows RR-E, 'Erasure · s.12(3)', 'Issued', 'For SRIB · about Anjali Verma · issued &lt;date&gt;', the due date and an 'Instruction'.
 4. A dialog 'RR-E · SRIB' opens with 'What the platform already knows', the messages so far, a 'Message' box ('Ask the Privacy Office a question, or say what you hold and where.'), 'Attach a file', the checkbox 'This is my return - close the ticket with it', and a 'Send' button greyed out while the box is empty.
 5. The message appears in the thread with 'File: srib-inventory.csv'. The ticket stays open.
 6. RR-E's row carries a '1 new' badge. On the request, the SRIB row shows '1 new' and a 'Thread' button with a count.
@@ -10422,7 +10422,7 @@
         <is>
           <t>1. No yellow warning is shown. 'Outcome' shows 'Complete', which can be chosen.
 2. It reads 'What was decided for each item, what has been carried out, and why. Say only what was done: the record lists each item as it stands.'
-3. 'Released and closed' with 'She has been told the response is ready.' appears. The header badge reads 'Complete' and a 'Response' card shows 'Complete · &lt;date&gt; ...'.
+3. 'Released and closed' with 'The requester has been told the response is ready.' appears. The header badge reads 'Complete' and a 'Response' card shows 'Complete · &lt;date&gt; ...'.
 4. Asset A still shows 'erased' and asset B 'redacted'. No 'Apply', 'Try again now', 'Place a legal hold' or 'Derive from asset_consent' buttons are offered.
 5. It has a section 'WHAT WAS DONE WITH EACH ITEM' with '- &lt;asset A&gt;: Erased.' and '- &lt;asset B&gt;: Redacted: your part removed; the material holds other people and was kept.', followed by 'Kept, because they are the record of what happened and are never rewritten: your consent records, the audit trail, the files of data sent to processors before your request, and earlier responses given to you.' There is no 'NOT YET DONE' section.
 6. RR-E shows 'Complete', 'Our response' with the text, 'Download the file' and 'Dispute this response'.
@@ -10508,13 +10508,13 @@
       <c r="K101" s="11" t="inlineStr">
         <is>
           <t>1. In Browser A make an erasure request ('Erasure (s.12(3))') with the test text. Note RR-H.
-2. In Browser B open RR-H: click 'Confirm classification', then 'She means erasure', then 'In progress' in 'What happens next'.
+2. In Browser B open RR-H: click 'Confirm classification', then 'They mean erasure', then 'In progress' in 'What happens next'.
 3. In the holders card click 'Derive from the records', choose 'Meera Iyer · rco@cmp.local · portal' in 'Respondent', click 'Confirm', then 'Issue tickets' and 'Issue the ticket'.
-4. In the scope card click 'Derive from asset_consent'. On asset H keep 'Erase - the asset holds only her', type the erase basis and click 'Record the decision'.
+4. In the scope card click 'Derive from asset_consent'. On asset H keep 'Erase - the asset holds only the requester', type the erase basis and click 'Record the decision'.
 5. On asset H click 'Place a legal hold'.
 6. Type the hold reason and click 'Place the hold'.
 7. Click 'Apply' on asset H.
-8. In Browser C (Meera) open 'Tickets for you', click 'Respond' on RR-H, type the return text, tick 'This is my return - close the ticket with it' and click 'Return the ticket'.
+8. In Browser C (Meera) open 'My tasks', click 'Respond' on RR-H, type the return text, tick 'This is my return - close the ticket with it' and click 'Return the ticket'.
 9. In Browser B reload RR-H.
 10. Look at '10 · Respond and close'.
 11. On asset H click 'Release hold'.
@@ -10527,7 +10527,7 @@
           <t>1. 'Recorded as RR-...' appears.
 2. 'Classified', 'Erasure confirmed' and 'Moved to In progress' appear in turn.
 3. SRIB shows 'confirmed', 'on the portal' and 'Issued'. The request is 'Awaiting holders'.
-4. 'Scope derived' shows 1 appearance; asset H shows 'only her' and 'decided: erase'.
+4. 'Scope derived' shows 1 appearance; asset H shows 'only the requester' and 'decided: erase'.
 5. A field 'Why this asset must not be erased' appears with the hint 'Sealed, and shown only to the Privacy Office.' and buttons 'Place the hold' (greyed out until at least 3 characters are typed) and 'Cancel'.
 6. The message 'Legal hold placed' with 'Nothing covered by it is erased until it is released.' appears.
 7. 'Quarantined' appears. The row shows a red badge 'legal hold' with a lock and the line 'Legal hold: stopped until the hold is released'. There is no 'Try again now' and no 'erased' badge; a 'Release hold' button is offered.
@@ -10615,7 +10615,7 @@
       <c r="K102" s="11" t="inlineStr">
         <is>
           <t>1. In Browser A make an erasure request with the test text. Note RR-P.
-2. In Browser B open RR-P, click 'Confirm classification', 'She means erasure' and then 'In progress'. Do NOT derive or add holders.
+2. In Browser B open RR-P, click 'Confirm classification', 'They mean erasure' and then 'In progress'. Do NOT derive or add holders.
 3. In the scope card click 'Derive from asset_consent'.
 4. In 'What happens next' look at both rows, then click 'Collating'.
 5. Look at '10 · Respond and close'. Type any text in 'The response'.
@@ -10631,7 +10631,7 @@
         <is>
           <t>1. 'Recorded as RR-...' appears.
 2. The request is 'In progress'; the holders card reads 'No holders yet...'.
-3. One row, asset P, 'only her', undecided.
+3. One row, asset P, 'only the requester', undecided.
 4. 'Move to awaiting holders' is blocked by 'No tickets have been issued yet'; 'Move to collating' is allowed. After the click 'Moved to Collating' appears.
 5. A warning reads 'Every item in the erasure scope needs a decision and the basis for it'. 'Release and close' stays greyed out.
 6. 'Quarantined' appears. Asset P shows 'quarantined - being erased' with 'The holder's copy: no holder has been asked for this asset's copy - confirm the source's holder and issue its ticket' and 'The platform's pointer to it: cleared'.
@@ -10728,7 +10728,7 @@
 2. 'Classified' and 'Moved to In progress' appear.
 3. 'Moved to Collating' appears and the card '9–10 · Collate, review, release' is shown.
 4. The warning reads 'Nothing in this request has been corrected: no item in scope has been carried out and no holder has returned its ticket. Answer it as partial, or as no records if nothing is held.' 'Complete' is greyed out; 'Partial - a gap is named' is selected.
-5. The hint reads 'What she is being given, and what could not be provided.' 'Released and closed' appears and the badge reads 'Partial'.
+5. The hint reads 'What the requester is being given, and what could not be provided.' 'Released and closed' appears and the badge reads 'Partial'.
 6. RR-C shows 'Partial' with the response and a 'Dispute this response' button.</t>
         </is>
       </c>
@@ -10814,7 +10814,7 @@
 5. Click 'See RR-A in full'.
 6. In Browser B open RR-G from 'Rights requests'.
 7. Look at '4 · Linked, and about whom?'.
-8. Click 'Confirm classification' (Grievance (s.13)) and then 'In progress'.
+8. Click 'Confirm classification' (Complaint (grievance) (s.13)) and then 'In progress'.
 9. Change 'Decision' to 'Not upheld', type the finding and click 'Decide and close'.
 10. In Browser A reload 'My requests' and look at RR-G.</t>
         </is>
@@ -10824,9 +10824,9 @@
           <t>1. A dialog 'Dispute RR-A' opens: 'A grievance under section 13. Say what was wrong with the handling - late, incomplete, sent the wrong way, or the outcome itself.' with 'What was wrong', the checkbox 'This is about the Data Protection Officer's own decisions.', 'Cancel' and 'Raise the grievance'.
 2. The error 'Say what you are asking for, in a sentence or two.' appears; nothing is recorded.
 3. 'Grievance recorded as RR-...' with 'It is linked to the original request.' appears. Note RR-G.
-4. RR-G shows 'Grievance · s.13', 'Received' and a box 'What you disputed' naming RR-A with 'Complete: &lt;start of the answer&gt;' and 'See RR-A in full'. RR-A shows 'You disputed this in RR-G' with 'See it'.
+4. RR-G shows 'Complaint (grievance) · s.13', 'Received' and a box 'What you disputed' naming RR-A with 'Complete: &lt;start of the answer&gt;' and 'See RR-A in full'. RR-A shows 'You disputed this in RR-G' with 'See it'.
 5. The page scrolls to RR-A and briefly highlights it.
-6. The line under the heading reads 'Grievance · s.13 · Portal'. 'About' shows RR-A with 'the request under dispute, shown below', and a card 'The request under dispute' shows RR-A's dates, what was asked and its answer.
+6. The line under the heading reads 'Complaint (grievance) · s.13 · Portal'. 'About' shows RR-A with 'the request under dispute, shown below', and a card 'The request under dispute' shows RR-A's dates, what was asked and its answer.
 7. It contains 'Is the complaint about the DPO?' with the text '...Recuse if this concerns your handling.' and a button 'This is about me - escalate' (do not click it).
 8. The request is 'In progress' and a card '6 · Is it upheld?' appears with 'Decision' ('Upheld'), 'What was found, and why', 'Remedy' and a ticked checkbox 'Re-run RR-A as a new request linked to this decision.' 'Decide and close' is greyed out.
 9. 'Remedy' and the re-run checkbox disappear. After the click, 'Not upheld' appears and the header badge reads 'Not upheld'.
@@ -10901,7 +10901,7 @@
       </c>
       <c r="J105" s="11" t="inlineStr">
         <is>
-          <t>- What are you asking for: Grievance (s.13)
+          <t>- What are you asking for: Complaint (grievance) (s.13)
 - Your request: The DPO refused my request without explaining why. I want somebody else to review it.
 - Tick: This complaint is about the Data Protection Officer's own decisions.
 - Reviewer: System Admin · admin@cmp.local
@@ -10911,7 +10911,7 @@
       </c>
       <c r="K105" s="11" t="inlineStr">
         <is>
-          <t>1. In Browser A click 'Make a request', choose 'Grievance (s.13)', type the text, tick 'This complaint is about the Data Protection Officer's own decisions.' and click 'Send the request'.
+          <t>1. In Browser A click 'Make a request', choose 'Complaint (grievance) (s.13)', type the text, tick 'This complaint is about the Data Protection Officer's own decisions.' and click 'Send the request'.
 2. In Browser B (DPO) open 'Rights requests'.
 3. Open RR-D and read 'Reviewer' and '4 · Linked, and about whom?'.
 4. Click 'Confirm classification', then look at 'What happens next'.
@@ -10974,7 +10974,7 @@
       </c>
       <c r="D106" s="11" t="inlineStr">
         <is>
-          <t>Portal - 'Somebody to act for you'; nomination acceptance link</t>
+          <t>Portal - My nominations - 'Somebody to act for you'; nomination acceptance link</t>
         </is>
       </c>
       <c r="E106" s="11" t="inlineStr">
@@ -11011,21 +11011,21 @@
           <t>- Their name: Rahul Verma
 - Their mobile: +91 90000 00077
 - Their email: rahul.nominee@example.org
-- Rights: keep 'Access (s.11)' and 'Erasure (s.12(3))' ticked; untick 'Correction (s.12)' and 'Grievance (s.13)'
+- Rights: keep 'Access (s.11)' and 'Erasure (s.12(3))' ticked; untick 'Correction (s.12)' and 'Complaint (grievance) (s.13)'
 - Wrong code: 000000</t>
         </is>
       </c>
       <c r="K106" s="11" t="inlineStr">
         <is>
-          <t>1. In Browser A on 'My requests' scroll to 'Somebody to act for you'.
-2. Fill in the test data, untick 'Correction (s.12)' and 'Grievance (s.13)', and click 'Nominate'.
+          <t>1. In Browser A click 'My nominations' in the sidebar and find the card 'Somebody to act for you'.
+2. Fill in the test data, untick 'Correction (s.12)' and 'Complaint (grievance) (s.13)', and click 'Nominate'.
 3. Look at the card.
 4. Ask the coordinator for the acceptance link sent to Rahul Verma and open it in Browser D (not signed in).
 5. Choose 'Mobile' and click 'Send me a code'.
 6. Type 000000 and click 'Accept the nomination'.
 7. Ask the coordinator for the code sent to +91 90000 00077, type it and click 'Accept the nomination'.
 8. Click 'Copy'.
-9. In Browser A reload 'My requests'.
+9. In Browser A reload 'My nominations'.
 10. In Browser D open the acceptance link again.</t>
         </is>
       </c>
@@ -11130,8 +11130,8 @@
 7. Click 'Confirm classification', then look at 'What happens next' and the classification card.
 8. Click 'Evidenced to our standard'.
 9. Click 'In progress'.
-10. In Browser A (Anjali) reload 'My requests'.
-11. In Browser D sign in at http://localhost:3001/sign-in with 'Mobile' and +91 90000 00077 (code from the coordinator), then open 'My requests'.
+10. In Browser A (Anjali) open 'My nominations'.
+11. In Browser D sign in at http://localhost:3001/sign-in with 'Mobile' and +91 90000 00077 (code from the coordinator), then open 'My nominations'.
 12. Click 'Show the request'.</t>
         </is>
       </c>
@@ -11146,7 +11146,7 @@
 7. 'Move to in progress' is blocked by 'The triggering event is not evidenced'. The card shows 'Is the triggering event evidenced?' with 'Rahul Verma says the principal cannot act...' and buttons 'Evidenced to our standard' and 'Not evidenced - refuse'.
 8. 'Event evidenced' appears; the card reads 'Event evidenced on &lt;date&gt;.'; the Nominee detail adds 'Evidenced &lt;date&gt; · the principal keeps their account and can follow this request'.
 9. 'Moved to In progress' appears.
-10. The nomination card shows 'Rahul Verma acted for you on &lt;date&gt;' with 'They reported that you cannot act for yourself. You keep this account and can follow the request they made. Their request is RR-N, under your requests above. The Privacy Office found the event evidenced on &lt;date&gt;.'
+10. The nomination card shows 'Rahul Verma acted for you on &lt;date&gt;' with 'They reported that you cannot act for yourself. You keep this account and can follow the request they made. Their request is RR-N, under My requests. The Privacy Office found the event evidenced on &lt;date&gt;.'
 11. A card 'Somebody has named you to act for them' shows Anjali Verma, 'In place' and 'You acted on &lt;date&gt;', with a 'Show the request' button.
 12. RR-N is shown with its status 'In progress', clock and path. There is no 'Dispute this response' button for the nominee.</t>
         </is>
@@ -11229,10 +11229,10 @@
           <t>1. In Browser D (signed out) open http://localhost:3001/rights/nominee, type the made-up reference and +91 90000 00077 and click 'Send me a code'.
 2. Open http://localhost:3001/rights/nominee?nomination=&lt;real reference&gt;, type +91 90000 00077 and click 'Send me a code'. Type 000000 in 'The code we sent', choose 'Access (s.11)', type a request of 10+ characters, choose 'They are unable to act' and click 'Record the request'.
 3. Reload the page, send a new code, enter the correct relayed code, choose 'Correction (s.12)' and click 'Record the request'.
-4. In Browser A on 'My requests' click 'Revoke this nomination'.
+4. In Browser A on 'My nominations' click 'Revoke this nomination'.
 5. In the form type Anjali Verma in 'Their name' and +91 90000 00001 in 'Their mobile', leave the rights ticked and click 'Nominate'.
 6. In Browser D open the nominee page with the revoked reference, type +91 90000 00077 and click 'Send me a code'.
-7. In Browser D (signed in as the nominee) reload 'My requests'.</t>
+7. In Browser D (signed in as the nominee) reload 'My nominations'.</t>
         </is>
       </c>
       <c r="L108" s="11" t="inlineStr">
@@ -11367,7 +11367,7 @@
       </c>
       <c r="D110" s="11" t="inlineStr">
         <is>
-          <t>Dashboard - 'Needs you today', queues, recent activity</t>
+          <t>Dashboard - 'Needs attention', queues, recent activity</t>
         </is>
       </c>
       <c r="E110" s="11" t="inlineStr">
@@ -11408,10 +11408,10 @@
         <is>
           <t>1. Open http://localhost:3000. Type dpo@cmp.local in 'Email or username' and SeedPassw0rd!2026 in 'Password', click 'Sign in'. On the 'Verify it is you' page type the six-digit code the test coordinator relays into '6-digit code' and click 'Verify and continue'.
 2. Read the line under the heading.
-3. Look at the first card, 'Needs you today'.
+3. Look at the first card, 'Needs attention'.
 4. Check the card for rows that belong to other roles.
-5. Click one of the rows in 'Needs you today' (for example 'Projects pending approval' or 'Rights requests due within 7 days').
-6. Scroll down past 'Needs you today' to the queue cards.
+5. Click one of the rows in 'Needs attention' (for example 'Projects pending approval' or 'Rights requests due within 7 days').
+6. Scroll down past 'Needs attention' to the queue cards.
 7. Scroll further to the cards 'Projects by stage' and 'Consent position'.
 8. Look at the 'Recent activity' card at the bottom.
 9. Click 'Full audit trail'.</t>
@@ -11421,18 +11421,18 @@
         <is>
           <t>1. You land on the Dashboard with the heading 'Good day, Priya'. The top right of the header shows the person's name with the role badge 'DPO'.
 2. It reads 'Notices awaiting publication, projects awaiting your review, and the consent position across the platform.'
-3. Each row shows a number, a label and an arrow, and the card's top right says how many things there are (e.g. '3 things'). Every label is one of: 'Tickets past their date', 'Rights requests overdue', 'Rights requests due within 7 days', 'Requests awaiting verification', 'Teams have written on their tickets', 'Grievances about the DPO to escalate', 'Retention floors passed, erasure due', 'Tickets addressed to you', 'Notice text awaiting approval', 'Projects pending approval', 'New collectors awaiting your decision'. If nothing is waiting the card says 'Nothing needs you today. The queues below are clear or waiting on somebody else.'
-4. There is no row about lockouts, sign-ins, access denials, 'Staff invitations not yet accepted', 'Sites awaiting a data source', 'Sources with nobody accountable' or 'Imports that did not reconcile'.
+3. Each row shows a number, a label and an arrow; the card's heading carries no overall count. Every label is one of: 'Breach duties overdue', 'Breach duties outstanding', 'Tickets past their date', 'Rights requests overdue', 'Rights requests due within 7 days', 'Requests awaiting verification', 'Teams have written on their tickets', 'Grievances about the DPO to escalate', 'Retention floors passed, erasure due', 'Tickets addressed to you', 'Notice text awaiting approval', 'Projects pending approval', 'New collectors awaiting your decision'. If nothing is waiting the card says 'Nothing needs your attention. The queues below are clear or waiting on somebody else.'
+4. There is no row about lockouts, sign-ins, access denials, 'Staff invitations not yet accepted', 'Sites awaiting a data source', 'Sources without an owner' or 'Imports that did not reconcile'.
 5. The list behind that number opens already filtered (e.g. the Projects page showing only projects pending approval, or the Rights requests page). The number of rows matches the count on the dashboard. Use the browser Back button to return.
-6. Queues with work appear as cards named from: 'Rights requests, soonest due first', 'Tickets past their date', 'Teams have written on their tickets', 'Drafts whose purposes are not activated', 'Pending Approval', 'New collectors awaiting your decision', 'Retention floors passed - erasure due'. Each card shows a count badge. Empty queues are listed together in one grey line that starts 'Clear:'. People's names in queue rows are readable.
-7. 'Projects by stage' shows bars labelled 'In draft', 'Pending approval' and 'Approved' with numbers; 'Consent position' shows one bar split into 'Still standing' and 'Withdrawn' with the caption 'Every record counted once, at its current state.'
+6. Queues with work appear as cards, in this order: 'Tickets past their date', 'Rights requests, soonest due first', 'Teams have written on their tickets', 'Retention floors passed - erasure due', 'Pending Approval', 'New collectors awaiting your decision', 'Drafts whose purposes are not activated'. Each card shows a count badge; a queue at its 25-row limit shows '25+' and a 'See all' link. Empty queues are listed together in one grey line that starts 'Clear:'. People's names in queue rows are readable.
+7. 'Projects by stage' shows bars labelled 'In draft', 'Pending approval' and 'Approved' with numbers; 'Consent position' shows one bar split into 'Agreed to all purposes', 'Agreed to some', 'Declined' and 'Withdrawn' with the caption 'Every record counted once, at its current state.'
 8. Up to 8 entries, newest first, each with an event name, a time, who did it (name and role badge) and the record it concerns. No sign-in events (titles starting 'Auth ...') are listed. A 'Full audit trail' link is at the card's top right.
 9. The 'Audit trail' page opens.</t>
         </is>
       </c>
       <c r="M110" s="11" t="inlineStr">
         <is>
-          <t>'Needs you today' contains only DPO-actionable rows from the listed set, each row opens a filtered list that matches its count, queues and position cards render, and Recent activity shows no sign-in events and links to the full audit trail.</t>
+          <t>'Needs attention' contains only DPO-actionable rows from the listed set, each row opens a filtered list that matches its count, queues and position cards render, and Recent activity shows no sign-in events and links to the full audit trail.</t>
         </is>
       </c>
       <c r="N110" s="16" t="n"/>
@@ -11463,7 +11463,7 @@
       </c>
       <c r="D111" s="11" t="inlineStr">
         <is>
-          <t>Dashboard - 'Needs you today', queues, recent activity</t>
+          <t>Dashboard - 'Needs attention', queues, recent activity</t>
         </is>
       </c>
       <c r="E111" s="11" t="inlineStr">
@@ -11504,8 +11504,8 @@
         <is>
           <t>1. Open http://localhost:3000. Type admin@cmp.local in 'Email or username' and SeedPassw0rd!2026 in 'Password', click 'Sign in'. On the 'Verify it is you' page type the six-digit code the test coordinator relays into '6-digit code' and click 'Verify and continue'.
 2. Read the line under the heading.
-3. Look at 'Needs you today'.
-4. Check 'Needs you today' for rows the administrator cannot act on.
+3. Look at 'Needs attention'.
+4. Check 'Needs attention' for rows the administrator cannot act on.
 5. If 'Staff invitations not yet accepted' is shown, click it.
 6. Scroll to the queue cards and the 'Clear:' line.
 7. Look for the cards 'Projects by stage' and 'Consent position'.
@@ -11515,18 +11515,18 @@
       <c r="L111" s="11" t="inlineStr">
         <is>
           <t>1. You land on the Dashboard with the heading 'Good day, System'. The top right of the header shows the person's name with the role badge 'Administrator'.
-2. It reads 'Accounts, lockouts, and the state of the processor and source registry.'
-3. Only these labels can appear (each only when its count is above zero): 'Staff invitations not yet accepted', 'Grievances about the DPO to review', 'Tickets addressed to you'. Otherwise the card says 'Nothing needs you today. The queues below are clear or waiting on somebody else.'
+2. It reads 'Invitations waiting, access problems, grievances about the DPO, and the processor and source registry.'
+3. Only these labels can appear (each only when its count is above zero): 'Staff invitations not yet accepted', 'Grievances about the DPO to review', 'Tickets addressed to you'. Otherwise the card says 'Nothing needs your attention. The queues below are clear or waiting on somebody else.'
 4. There is no row about lockouts, access denials, consent withdrawals, projects, notices, or rights requests overdue.
 5. The 'Users' page opens filtered to pending accounts; it lists staff whose invitation is not yet accepted and no data principals. Use Back to return. (If the row is absent, note 'no pending invitations' and continue.)
-6. The queues are 'Grievances about the DPO - yours to review', 'Lockouts (24h)' and 'Suspended sources and processors' (as cards, or named in the 'Clear:' line when empty). A lockout from the last 24 hours appears as a row in 'Lockouts (24h)' with the person's readable name - here, and not in 'Needs you today'.
+6. The queues are 'Grievances about the DPO - yours to review', 'Lockouts (24h)' and 'Suspended sources and processors' (as cards, or named in the 'Clear:' line when empty). A lockout from the last 24 hours appears as a row in 'Lockouts (24h)' with the person's readable name - here, and not in 'Needs attention'.
 7. Neither card is shown to the administrator.
 8. Entries are refused requests - title 'Auth access denied' with the sentence 'A request was refused by the permission matrix.' - each with who and when. A 'Full audit trail' link is at the card's top right.</t>
         </is>
       </c>
       <c r="M111" s="11" t="inlineStr">
         <is>
-          <t>Administrator 'Needs you today' holds only invitations, grievances about the DPO and own tickets; lockouts appear only in the 'Lockouts (24h)' queue; no project or consent charts; Recent activity shows access denials with a 'Full audit trail' link.</t>
+          <t>Administrator 'Needs attention' holds only invitations, grievances about the DPO and own tickets; lockouts appear only in the 'Lockouts (24h)' queue; no project or consent charts; Recent activity shows access denials with a 'Full audit trail' link.</t>
         </is>
       </c>
       <c r="N111" s="16" t="n"/>
@@ -11557,7 +11557,7 @@
       </c>
       <c r="D112" s="11" t="inlineStr">
         <is>
-          <t>Dashboard - 'Needs you today', queues, recent activity</t>
+          <t>Dashboard - 'Needs attention', queues, recent activity</t>
         </is>
       </c>
       <c r="E112" s="11" t="inlineStr">
@@ -11597,24 +11597,24 @@
       <c r="K112" s="11" t="inlineStr">
         <is>
           <t>1. Open http://localhost:3000. Type dco@cmp.local in 'Email or username' and SeedPassw0rd!2026 in 'Password', click 'Sign in'. On the 'Verify it is you' page type the six-digit code the test coordinator relays into '6-digit code' and click 'Verify and continue'.
-2. Read the line under the heading, then look at 'Needs you today'.
-3. Check 'Needs you today' for rows belonging to other roles.
+2. Read the line under the heading, then look at 'Needs attention'.
+3. Check 'Needs attention' for rows belonging to other roles.
 4. Find the 'Import exceptions' queue (a card, or named in the 'Clear:' line). If it is a card, click its first row.
 5. Look at the 'Recent activity' card.
 6. Click 'Sign out' at the bottom of the sidebar. Then sign in again as rco@cmp.local (password SeedPassw0rd!2026, code from the coordinator, 'Verify and continue').
-7. Read the line under the heading and 'Needs you today'.
+7. Read the line under the heading and 'Needs attention'.
 8. Look at the 'Recent activity' card.</t>
         </is>
       </c>
       <c r="L112" s="11" t="inlineStr">
         <is>
           <t>1. You land on the Dashboard with the heading 'Good day, Arun'. The top right of the header shows the person's name with the role badge 'Data Collection Owner'.
-2. The line reads 'Your approved projects, the links collecting against them, and anything that failed to reconcile on import.' 'Needs you today' holds only rows from: 'Tickets past their date', 'Tickets addressed to you', 'Imports that did not reconcile', 'Assets with unmapped subjects' - or the sentence 'Nothing needs you today. ...'.
+2. The line reads 'Your approved projects, the links collecting against them, and anything that failed to reconcile on import.' 'Needs attention' holds only rows from: 'Tickets past their date', 'Tickets addressed to you', 'Imports that did not reconcile', 'Assets with unmapped subjects' - or the sentence 'Nothing needs your attention. ...'.
 3. No 'Projects pending approval', 'Rights requests overdue', 'Notice text awaiting approval', 'Staff invitations not yet accepted', lockout or 'Sites awaiting a data source' row appears.
-4. A card row names a collection and a project and says '&lt;n&gt; declared, &lt;m&gt; mapped — &lt;k&gt; unaccounted for'. Clicking it opens that collection's page (not 'Not part of your account'). Use Back to return.
+4. The queues are 'Import exceptions' and 'Approved projects ready to collect' (as cards, or named in the 'Clear:' line). An 'Import exceptions' row names a collection and a project and says '&lt;n&gt; declared, &lt;m&gt; mapped — &lt;k&gt; unaccounted for'. Clicking it opens that collection's page (not 'Not part of your account'). Use Back to return.
 5. It lists events on Arun's own projects or done by him, with no sign-in ('Auth ...') events. There is NO 'Full audit trail' link on the card, because a DCO has no audit page.
 6. The Dashboard opens with the heading 'Good day, Meera' and the role badge 'R&amp;D Collection Owner'.
-7. The line reads 'The collection your team runs itself — your approved projects, the links collecting against them, and anything that failed to reconcile on import.' 'Needs you today' uses the same four DCO labels only.
+7. The line reads 'The collection your team runs itself — your approved projects, the links collecting against them, and anything that failed to reconcile on import.' 'Needs attention' uses the same four DCO labels only.
 8. Events on Meera's projects only, no sign-in events, and no 'Full audit trail' link.</t>
         </is>
       </c>
@@ -11651,7 +11651,7 @@
       </c>
       <c r="D113" s="11" t="inlineStr">
         <is>
-          <t>Dashboard - 'Needs you today', queues, recent activity</t>
+          <t>Dashboard - 'Needs attention', queues, recent activity</t>
         </is>
       </c>
       <c r="E113" s="11" t="inlineStr">
@@ -11691,12 +11691,12 @@
       <c r="K113" s="11" t="inlineStr">
         <is>
           <t>1. Open http://localhost:3000. Type dcoadmin@cmp.local in 'Email or username' and SeedPassw0rd!2026 in 'Password', click 'Sign in'. On the 'Verify it is you' page type the six-digit code the test coordinator relays into '6-digit code' and click 'Verify and continue'.
-2. Read the line under the heading and look at 'Needs you today'.
+2. Read the line under the heading and look at 'Needs attention'.
 3. If 'Sites awaiting a data source' is listed, click it.
-4. If 'Sources with nobody accountable' is listed, click it.
+4. If 'Sources without an owner' is listed, click it.
 5. Look at 'Recent activity'.
 6. Click 'Sign out' at the bottom of the sidebar. Then sign in again as rnd@cmp.local (password SeedPassw0rd!2026, code from the coordinator, 'Verify and continue').
-7. Read the line under the heading and look at 'Needs you today'.
+7. Read the line under the heading and look at 'Needs attention'.
 8. If 'Projects needing something from you' is listed, click it, then click the first row of the queue it jumps to.
 9. Scroll to the bottom of the dashboard.</t>
         </is>
@@ -11704,14 +11704,14 @@
       <c r="L113" s="11" t="inlineStr">
         <is>
           <t>1. You land on the Dashboard with the heading 'Good day, Nikhil'. The top right of the header shows the person's name with the role badge 'DCO Admin'.
-2. The line reads 'Projects collected by a third party: which sites are still waiting for a data source, and who picks them up when you attach one.' Rows come only from: 'Tickets past their date', 'Sites awaiting a data source', 'Sources with nobody accountable', 'Processors with no collection set up', 'Tickets addressed to you'.
+2. The line reads 'Projects collected by a third party: which sites are still waiting for a data source, and who picks them up when you attach one.' Rows come only from: 'Tickets past their date', 'Sites awaiting a data source', 'Sources without an owner', 'Processors with no collection set up', 'Tickets addressed to you'.
 3. The page scrolls down to the 'Sites awaiting a data source' queue card on the same dashboard; each row names a project and says 'Attach the data source that will collect here'.
 4. The 'Data sources' page opens (not 'Not part of your account'). Use Back to return.
 5. No sign-in events and no 'Full audit trail' link.
 6. The Dashboard opens with the heading 'Good day, Kavya' and the role badge 'R&amp;D User'.
 7. The line reads 'Your projects and what each one needs from you before it can move forward.' Rows come only from 'Projects needing something from you' and 'Tickets addressed to you'.
 8. The page scrolls to the 'Needs your action' queue; rows name Kavya's draft projects with 'Upload a security approval with its proof file'. Clicking a row opens that project's page.
-9. 'Projects by stage' is shown (counting only Kavya's projects); there is no 'Consent position' card; 'Recent activity' has no 'Full audit trail' link.</t>
+9. A 'Waiting for DPO review' queue lists Kavya's projects pending approval (or is named in the 'Clear:' line). 'Projects by stage' is shown (counting only Kavya's projects); there is no 'Consent position' card; 'Recent activity' has no 'Full audit trail' link.</t>
         </is>
       </c>
       <c r="M113" s="11" t="inlineStr">
@@ -11799,18 +11799,18 @@
       <c r="L114" s="11" t="inlineStr">
         <is>
           <t>1. You land on the Dashboard with the heading 'Good day, Priya'. The top right of the header shows the person's name with the role badge 'DPO'.
-2. In this order: OVERVIEW - Dashboard; GOVERNANCE - Projects, Approvals, Notices, Purposes; CONSENT - Consents, Consent links, Collection sites; REGISTRY - Processors, Data sources; DATA MOVEMENT - Collections, Exports, Imports; OVERSIGHT - Rights requests, Audit trail, Users, Delegate, Messages; YOU - Tickets for you, Notifications, Your profile. A 'Sign out' button sits at the bottom.
-3. Every link opens a page with its own heading. None shows 'This page could not be found' or 'Not part of your account'. The link for the open page is highlighted.
+2. In this order: YOUR WORK - Dashboard, Rights requests, Breaches, My tasks, Projects, Notices; GOVERNANCE - Approval documents, Purposes; CONSENT - Consents, Consent links, Collection sites; REGISTRY - Processors, Data sources; DATA MOVEMENT - Collections, Exports, Imports; OVERSIGHT - Audit trail, Users, Delegations, Message templates. There is no 'My profile' or 'Notifications' entry: 'My profile' is in the account menu (click your name at the top right) and notifications open from the bell in the header. A 'Sign out' button sits at the bottom.
+3. Every link opens a page with its own heading. None shows 'We can't find that page' or 'Not part of your account'. The link for the open page is highlighted.
 4. The Dashboard opens with the heading 'Good day, System' and the role badge 'Administrator'.
-5. OVERVIEW - Dashboard; REGISTRY - Processors, Data sources; OVERSIGHT - Grievances about the DPO, Audit trail, Users, Delegate, Messages; YOU - Tickets for you, Notifications, Your profile.
-6. There are no GOVERNANCE, CONSENT or DATA MOVEMENT headings and no links to Projects, Approvals, Notices, Purposes, Consents, Consent links, Collection sites, Collections, Exports or Imports. There is no 'Rights requests' link - that slot reads 'Grievances about the DPO'.
+5. YOUR WORK - Dashboard, Users, Grievances about the DPO, Message templates, Processors, Data sources, Audit trail; OVERSIGHT - Delegations; YOU - My tasks.
+6. There are no GOVERNANCE, CONSENT, REGISTRY or DATA MOVEMENT headings and no links to Projects, Approval documents, Notices, Purposes, Consents, Consent links, Collection sites, Collections, Exports or Imports. There is no 'Rights requests' link - that slot reads 'Grievances about the DPO'.
 7. A page headed 'Grievances about the DPO' opens.
-8. Every link opens a page with its own heading; none shows 'This page could not be found' or 'Not part of your account'.</t>
+8. Every link opens a page with its own heading; none shows 'We can't find that page' or 'Not part of your account'.</t>
         </is>
       </c>
       <c r="M114" s="11" t="inlineStr">
         <is>
-          <t>The DPO sees all 21 links in 7 sections; the Administrator sees exactly the 11 links listed, with the rights link relabelled 'Grievances about the DPO', and every link opens.</t>
+          <t>The DPO sees the 20 links listed, starting with the 'Your work' group; the Administrator sees exactly the 9 links listed, with the rights link relabelled 'Grievances about the DPO', and every link opens.</t>
         </is>
       </c>
       <c r="N114" s="16" t="n"/>
@@ -11894,18 +11894,18 @@
       <c r="L115" s="11" t="inlineStr">
         <is>
           <t>1. You land on the Dashboard with the heading 'Good day, Arun'. The top right of the header shows the person's name with the role badge 'Data Collection Owner'.
-2. OVERVIEW - Dashboard; GOVERNANCE - Projects; CONSENT - Consents, Consent links, Collection sites; REGISTRY - Data sources; DATA MOVEMENT - Collections, Exports, Imports; OVERSIGHT - Delegate; YOU - Tickets for you, Notifications, Your profile.
-3. OVERSIGHT holds only 'Delegate'. There is no 'Audit trail', 'Users', 'Rights requests' or 'Messages', and no 'Approvals', 'Notices', 'Purposes' or 'Processors' anywhere in the sidebar.
-4. Every link opens a page with its own heading; none shows 'This page could not be found' or 'Not part of your account'.
+2. YOUR WORK - Dashboard, My projects, Collection sites, Consent links, My tasks, Collections; CONSENT - Consents; REGISTRY - Data sources; DATA MOVEMENT - Exports, Imports; OVERSIGHT - Delegations. 'My profile' is in the account menu and notifications open from the bell in the header.
+3. OVERSIGHT holds only 'Delegations'. There is no 'Audit trail', 'Users', 'Rights requests' or 'Message templates', and no 'Approval documents', 'Notices', 'Purposes' or 'Processors' anywhere in the sidebar.
+4. Every link opens a page with its own heading; none shows 'We can't find that page' or 'Not part of your account'.
 5. The Dashboard opens with the heading 'Good day, Nikhil' and the role badge 'DCO Admin'.
-6. Exactly the same links as the DCO; no 'Audit trail', 'Users', 'Rights requests', 'Messages', 'Approvals', 'Notices', 'Purposes' or 'Processors'.
+6. YOUR WORK - Dashboard, Collection sites, Data sources, My tasks, Consent links, Projects; CONSENT - Consents; DATA MOVEMENT - Collections, Exports, Imports; OVERSIGHT - Delegations. These are the DCO's pages in a different order, and the projects link reads 'Projects' (not 'My projects'). No 'Audit trail', 'Users', 'Rights requests', 'Message templates', 'Approval documents', 'Notices', 'Purposes' or 'Processors'.
 7. The Dashboard opens with the heading 'Good day, Meera' and the role badge 'R&amp;D Collection Owner'.
-8. Exactly the same links as the DCO; no 'Audit trail' and none of the other absent links.</t>
+8. Exactly the same links, in the same order, as the DCO (including 'My projects'); no 'Audit trail' and none of the other absent links.</t>
         </is>
       </c>
       <c r="M115" s="11" t="inlineStr">
         <is>
-          <t>All three collection roles see the same 13 links, OVERSIGHT contains only 'Delegate', and no audit, user, rights, message, approval, notice, purpose or processor link is offered.</t>
+          <t>All three collection roles see the same 11 pages, starting with their own 'Your work' group; OVERSIGHT contains only 'Delegations', and no audit, user, rights, message-template, approval, notice, purpose or processor link is offered.</t>
         </is>
       </c>
       <c r="N115" s="16" t="n"/>
@@ -11984,15 +11984,15 @@
       <c r="L116" s="11" t="inlineStr">
         <is>
           <t>1. You land on the Dashboard with the heading 'Good day, Kavya'. The top right of the header shows the person's name with the role badge 'R&amp;D User'.
-2. OVERVIEW - Dashboard; GOVERNANCE - Projects, Approvals, Notices; REGISTRY - Processors; DATA MOVEMENT - Collections, Imports; YOU - Tickets for you, Notifications, Your profile.
-3. There is no CONSENT heading and no OVERSIGHT heading. There are no links to Purposes, Consents, Consent links, Collection sites, Data sources, Exports, Rights requests, Audit trail, Users, Delegate or Messages.
+2. YOUR WORK - Dashboard, My projects, Approval documents, My tasks, Notices; REGISTRY - Processors; DATA MOVEMENT - Collections, Imports. 'My profile' is in the account menu and notifications open from the bell in the header.
+3. There is no CONSENT heading and no OVERSIGHT heading. There are no links to Purposes, Consents, Consent links, Collection sites, Data sources, Exports, Rights requests, Audit trail, Users, Delegations or Message templates.
 4. A page headed 'Notices' opens (the R&amp;D User authors notices).
-5. Every link opens a page with its own heading; none shows 'This page could not be found' or 'Not part of your account'.</t>
+5. Every link opens a page with its own heading; none shows 'We can't find that page' or 'Not part of your account'.</t>
         </is>
       </c>
       <c r="M116" s="11" t="inlineStr">
         <is>
-          <t>The R&amp;D User sees exactly the 10 links listed, no Consent or Oversight section, and every link opens.</t>
+          <t>The R&amp;D User sees exactly the 8 links listed, no Consent or Oversight section, and every link opens.</t>
         </is>
       </c>
       <c r="N116" s="16" t="n"/>
@@ -12166,7 +12166,7 @@
       <c r="K118" s="11" t="inlineStr">
         <is>
           <t>1. Open http://localhost:3000. Type dpo@cmp.local in 'Email or username' and SeedPassw0rd!2026 in 'Password', click 'Sign in'. On the 'Verify it is you' page type the six-digit code the test coordinator relays into '6-digit code' and click 'Verify and continue'.
-2. In the sidebar under YOU, click 'Notifications' (the bell icon).
+2. Click the bell icon at the top right of the header (its label is 'Notifications').
 3. Find an entry titled 'Consent withdrawn'.
 4. Find an entry titled 'Auth login locked out' (from the precondition).
 5. Click the body of the 'Consent withdrawn' entry (not the link).
@@ -12182,9 +12182,9 @@
 3. Its explanation reads 'Consent was withdrawn. The earlier record still stands as evidence of what was agreed at the time.' Its record link reads 'Consent record: &lt;person's name&gt; — &lt;project&gt;' with the name readable.
 4. Its explanation reads 'An account was locked after repeated failed sign-ins.' and its record link reads 'Account: &lt;name of the locked account&gt;'.
 5. A dialog titled 'Consent withdrawn' opens showing 'What', 'When', 'Who', 'About', 'Event' (consent.withdrawn) and 'Record', the note 'This entry is append-only and part of a hash chain. ...', and the buttons 'Open consent record' and 'Close'.
-6. The consent record page opens, headed with the person's name and an 'All consents' back link - not 'Not part of your account' and not 'This page could not be found'.
+6. The consent record page opens, headed with the person's name and an 'All consents' back link - not 'Not part of your account' and not 'We can't find that page'.
 7. The 'Users' page opens.
-8. Each link opens a page the DPO can use; none shows 'Not part of your account' or 'This page could not be found'.</t>
+8. Each link opens a page the DPO can use; none shows 'Not part of your account' or 'We can't find that page'.</t>
         </is>
       </c>
       <c r="M118" s="11" t="inlineStr">
@@ -12262,7 +12262,7 @@
       <c r="K119" s="11" t="inlineStr">
         <is>
           <t>1. Open http://localhost:3000. Type admin@cmp.local in 'Email or username' and SeedPassw0rd!2026 in 'Password', click 'Sign in'. On the 'Verify it is you' page type the six-digit code the test coordinator relays into '6-digit code' and click 'Verify and continue'.
-2. In the sidebar under YOU, click 'Notifications'.
+2. Click the bell icon at the top right of the header.
 3. Find the 'Auth login locked out' entry for the account locked in the precondition.
 4. Scroll the whole list looking for 'Consent withdrawn'.
 5. Scroll the list looking for project events.
@@ -12356,13 +12356,13 @@
       <c r="K120" s="11" t="inlineStr">
         <is>
           <t>1. Open http://localhost:3000. Type dco@cmp.local in 'Email or username' and SeedPassw0rd!2026 in 'Password', click 'Sign in'. On the 'Verify it is you' page type the six-digit code the test coordinator relays into '6-digit code' and click 'Verify and continue'.
-2. Click 'Notifications' in the sidebar and read the list.
+2. Click the bell icon in the header to open 'Notifications', and read the list.
 3. Look for 'Consent withdrawn' and 'Auth login locked out' entries.
-4. Note the project named on two entries, then click 'Projects' in the sidebar.
+4. Note the project named on two entries, then click 'My projects' in the sidebar.
 5. Back on 'Notifications', click a 'Project: &lt;name&gt;' link, then an 'Export' link on an 'Export generated' entry (if present).
 6. If a 'Notice published' entry is present, click its 'Notice: ...' link (or 'Open notice' in its dialog).
 7. Click 'Sign out' at the bottom of the sidebar. Then sign in again as rnd@cmp.local (password SeedPassw0rd!2026, code from the coordinator, 'Verify and continue').
-8. Click 'Notifications' and read the list.
+8. Click the bell icon in the header and read the 'Notifications' list.
 9. Click the record link on each entry shown, including any 'Export generated' entry's 'Export' link.</t>
         </is>
       </c>
@@ -12371,7 +12371,7 @@
           <t>1. You land on the Dashboard with the heading 'Good day, Arun'. The top right of the header shows the person's name with the role badge 'Data Collection Owner'.
 2. Entries are only of these kinds: 'Project transitioned', 'Notice published', 'Import rejected', 'Export generated', plus events on tickets addressed to Arun. Each names a project (or a notice, import or export on one).
 3. Neither appears, although the DPO's feed shows both.
-4. Both projects are in Arun's Projects list - no entry concerns a project he cannot see.
+4. Both projects are in Arun's projects list - no entry concerns a project he cannot see.
 5. The project page and the 'Exports' page open normally.
 6. A page Arun can use opens. It must NOT show 'Not part of your account' (the rule is that no notification link leads to a page the reader cannot open). If it does, record a defect.
 7. The Dashboard opens with the heading 'Good day, Kavya' and the role badge 'R&amp;D User'.
@@ -12934,7 +12934,7 @@
 5. Click 'Notices', open a notice and click 'Audit trail'.
 6. Click 'Rights requests', open a request by its 'Reference' and click 'Audit trail'.
 7. Click 'Sign out' at the bottom of the sidebar. Then sign in again as dco@cmp.local (password SeedPassw0rd!2026, code from the coordinator, 'Verify and continue').
-8. Click 'Consents', open a record, then open a project from 'Projects'.
+8. Click 'Consents', open a record, then open a project from 'My projects'.
 9. Sign out, sign in as rnd@cmp.local and open one of Kavya's projects.</t>
         </is>
       </c>
@@ -13044,7 +13044,7 @@
 5. No email address appears in the details; the person is identified only through 'Who' / 'About' and the record link.
 6. 'Nothing matches these filters'.
 7. 'Nothing matches these filters' both times - no contact is written into the trail.
-8. The details show 'Reason given' yes/no and no reason text. The button opens the 'Delegate' page. If it shows 'This page could not be found', record a defect.</t>
+8. The details show 'Reason given' yes/no and no reason text. The button opens the 'Delegations' page. If it shows 'We can't find that page', record a defect.</t>
         </is>
       </c>
       <c r="M127" s="11" t="inlineStr">
@@ -13177,7 +13177,7 @@
       </c>
       <c r="D129" s="11" t="inlineStr">
         <is>
-          <t>Notifications (data principal portal)</t>
+          <t>Updates - notifications (data principal portal)</t>
         </is>
       </c>
       <c r="E129" s="11" t="inlineStr">
@@ -13217,24 +13217,24 @@
         <is>
           <t>1. Open http://localhost:3001/sign-in. Under 'Sign in with' choose 'Email', type subject@cmp.local in 'Email address' and click 'Send me a code'.
 2. Type the code the test coordinator relays and click 'Verify'.
-3. Click 'Notifications'.
+3. Click 'Updates'.
 4. Check the list for events that are not hers to see.
 5. Click the body of a 'Consent given' entry.
 6. Click 'Open consent record'.
-7. Back on 'Notifications', click the record link on a rights request entry (if present) and on a 'Subject registered' entry ('Account: Anjali Verma' / 'Open account').
+7. Back on 'Updates', click the record link on a rights request entry (if present) and on a 'Subject registered' entry ('Account: Anjali Verma' / 'Open account').
 8. Type http://localhost:3001/users in the address bar, then http://localhost:3001/audit.</t>
         </is>
       </c>
       <c r="L129" s="11" t="inlineStr">
         <is>
           <t>1. A 'Check your messages' notice appears and a 'Six-digit code' box is shown.
-2. The 'Your consents' page opens. The sidebar shows YOUR DATA - 'My consents', 'My requests' and YOU - 'Notifications', 'Your profile', and nothing else.
-3. The page 'Notifications' opens with 'What has happened that concerns you, taken from the audit trail itself.' Entries are about Anjali only, e.g. 'Consent given', 'Consent withdrawn', 'Notice served', 'Subject registered', 'Rights request received'. If there are none it says 'Nothing to report'.
+2. The 'My consents' page opens. The sidebar shows YOUR DATA - 'My consents', 'My requests', 'My nominations' and 'Updates', and nothing else; 'My profile' is in the account menu under her name at the top right.
+3. The page 'Updates' opens with 'What has happened that concerns you, taken from the audit trail itself.' Entries are about Anjali only, e.g. 'Consent given', 'Consent withdrawn', 'Notice served', 'Subject registered', 'Rights request received'. If there are none it says 'Nothing to report'.
 4. No sign-in events ('Auth ...'), no 'Project transitioned', no office working on her request (e.g. 'Rights ticket issued', 'Rights holders derived') and no events about other people.
 5. A dialog shows 'What' ('Consent record: Anjali Verma — &lt;project&gt;'), 'When', 'Who', 'Event' (consent.given) and 'Record', with an 'Open consent record' button. All names are readable; no 'SE::' text.
-6. The 'Your consents' page on the portal opens - not a staff page and not 'Not part of your account'.
-7. The request link opens 'My requests'. The account link opens her own account page ('Your account'). If either shows 'This page could not be found', record a defect.
-8. Both show the '404 | This page could not be found.' page - no staff screen exists on the portal.</t>
+6. The 'My consents' page on the portal opens - not a staff page and not 'Not part of your account'.
+7. The request link opens 'My requests'. The account link opens her own account page ('My profile'). If either shows 'We can't find that page', record a defect.
+8. Both show the portal's 404 page, headed 'We can't find that page', with the buttons 'Go to My consents' and 'Your rights' - no staff screen exists on the portal.</t>
         </is>
       </c>
       <c r="M129" s="11" t="inlineStr">
@@ -13309,7 +13309,7 @@
         <is>
           <t>1. Open http://localhost:3000. Type dpo@cmp.local in 'Email or username' and SeedPassw0rd!2026 in 'Password', click 'Sign in'. On the 'Verify it is you' page type the six-digit code the test coordinator relays into '6-digit code' and click 'Verify and continue'.
 2. Click 'Projects' in the sidebar and look to the right of the logo in the header.
-3. Press Ctrl+K (⌘K on a Mac), or click 'Search or jump to…'. Type 'aud'.
+3. Press Ctrl+K (⌘K on a Mac), or click 'Jump to page…'. Type 'aud'.
 4. Press Enter.
 5. Open the box again (Ctrl+K / ⌘K) without typing.
 6. Click Priya's name at the top right of the header.
@@ -13321,12 +13321,12 @@
       <c r="L130" s="11" t="inlineStr">
         <is>
           <t>1. You land on the Dashboard with the heading 'Good day, Priya'. The top right of the header shows the person's name with the role badge 'DPO'.
-2. A breadcrumb reads 'Governance › Projects'. In the header are a box 'Search or jump to…' showing ⌘K (on a Mac) or Ctrl K, a help (?) button, a bell, and Priya's name with the 'DPO' badge and her initials.
+2. A breadcrumb reads 'Governance › Projects'. In the header are a box 'Jump to page…' showing ⌘K (on a Mac) or Ctrl K, a help (?) button, a bell, and Priya's name with the 'DPO' badge and her initials.
 3. A search box opens over the page ('Search pages and actions…'). Typing narrows the list to 'Audit trail' under the heading 'Oversight'. The footer reads '↑ ↓ to move', '↵ to open', 'Esc to close'.
 4. The 'Audit trail' page opens and the box closes. The breadcrumb reads 'Oversight › Audit trail'.
 5. A 'Recent' group lists the pages just visited (for example 'Projects'), but not the page you are on. An 'Actions' group offers 'Open the help manual', 'Switch to dark theme' and 'Sign out'. Type 'zzz': it says 'Nothing matches “zzz”'. Press Esc to close it.
-6. An account menu opens showing 'Priya Menon' and 'DPO', then 'Your profile', 'Help manual', 'Switch to dark theme' and 'Sign out'. Press Esc: it closes and nothing else changes.
-7. The first click folds away Projects, Approvals, Notices and Purposes; the second brings them back. The group holding the page you are on cannot be folded away.
+6. An account menu opens showing 'Priya Menon' and 'DPO', then 'My profile', 'Help manual', 'Switch to dark theme' and 'Sign out'. Press Esc: it closes and nothing else changes.
+7. The first click folds away 'Approval documents' and 'Purposes'; the second brings them back. The group holding the page you are on cannot be folded away.
 8. The sidebar becomes a narrow strip of icons (hovering an icon shows its name) and stays that way after the reload. Click 'Expand sidebar' to restore it.
 9. The card folds to its heading, so the working cards below move up. Clicking it again unfolds it. On a project page, the 'History' card folds the same way and shows its number of entries.</t>
         </is>
@@ -13406,7 +13406,7 @@
 3. Type 'export' in 'Search the manual'.
 4. Scroll to the end of the manual.
 5. Sign in to the console as dco@cmp.local (SeedPassw0rd!2026 and the relayed code). Click the help (?) button in the header.
-6. Choose 'Every role' in the role box. Then click 'Back to the console', press Ctrl+K (⌘K) and choose 'Open the help manual'.
+6. Choose 'Every role' in the role box. Then click 'Back to where you were', press Ctrl+K (⌘K) and choose 'Open the help manual'.
 7. Open http://localhost:3001/sign-in and click 'Help manual' next to 'Your rights and how to exercise them'.
 8. Narrow the browser window to phone width (or use a phone) and look at the portal manual.</t>
         </is>
@@ -13417,7 +13417,7 @@
 2. The page scrolls to section 16 'Rights requests', whose badges read 'DPO' and 'Administrator'. Its numbered steps show the screen's own words in grey label boxes, for example 'Confirm classification'.
 3. Only sections that mention exports remain, and the line under the box reads '8 of 24 sections mentioning “export”' (Exports, Purposes, Processors, the audit trail and others). Clicking the × clears it.
 4. A panel 'Have any questions? Contact us' shows the Privacy Office's email address and response time, and says to ask your administrator about sign-in or role problems.
-5. The manual opens already set to 'For the DCO', reading '15 of 24 sections for the DCO'. Section numbers keep their places (for example 8, 12, 13, 14). The top-right button now reads 'Back to the console'.
+5. The manual opens already set to 'For the DCO', reading '15 of 24 sections for the DCO'. Section numbers keep their places (for example 8, 12, 13, 14). The top-right button now reads 'Back to where you were'.
 6. 'Every role' shows all 24 sections. The command palette opens the manual again.
 7. The page 'Consent Portal Manual' opens without signing in, with 15 sections written for data principals (creating an account, giving consent through a link, withdrawing, requests, nominations) and no role choice.
 8. The table of contents folds into a 'Table of contents · 15' bar above the sections; opening it lists them. Nothing is cut off at the side.</t>
@@ -13671,7 +13671,7 @@
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>The sidebar shows the sections Overview, Governance, Consent, Registry, Data movement, Oversight and You. Under Oversight there are 'Rights requests', 'Audit trail', 'Users', 'Delegate' and 'Messages'; under You there are 'Tickets for you', 'Notifications' and 'Your profile'. A 'Sign out' button is at the bottom of the sidebar.</t>
+          <t>The sidebar starts with the group 'Your work' - 'Dashboard', 'Rights requests', 'Breaches', 'My tasks', 'Projects', 'Notices' - followed by the groups Governance, Consent, Registry, Data movement and Oversight. Under Oversight there are 'Audit trail', 'Users', 'Delegations' and 'Message templates'. 'My profile' is not in the sidebar (it is in the account menu under your name at the top right), and notifications open from the bell in the header. A 'Sign out' button is at the bottom of the sidebar.</t>
         </is>
       </c>
       <c r="F7" s="16" t="n"/>
@@ -13752,7 +13752,7 @@
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>The menu shows exactly: Dashboard; Projects; Consents, Consent links, Collection sites; Data sources; Collections, Exports, Imports; Delegate; Tickets for you, Notifications, Your profile. There is no 'Approvals', 'Notices', 'Purposes', 'Audit trail', 'Users' or 'Messages'.</t>
+          <t>The menu shows exactly: Your work - Dashboard, My projects, Collection sites, Consent links, My tasks, Collections; Consent - Consents; Registry - Data sources; Data movement - Exports, Imports; Oversight - Delegations. There is no 'Approval documents', 'Notices', 'Purposes', 'Audit trail', 'Users' or 'Message templates'.</t>
         </is>
       </c>
       <c r="F10" s="16" t="n"/>
@@ -13860,7 +13860,7 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>The menu shows: Dashboard; Processors, Data sources; Grievances about the DPO, Audit trail, Users, Delegate, Messages; Tickets for you, Notifications, Your profile. There is no 'Projects', 'Consents' or 'Consent links'. The rights item is labelled 'Grievances about the DPO', not 'Rights requests'.</t>
+          <t>The menu shows: Your work - Dashboard, Users, Grievances about the DPO, Message templates, Processors, Data sources, Audit trail; Oversight - Delegations; You - My tasks. There is no 'Projects', 'Consents' or 'Consent links'. The rights item is labelled 'Grievances about the DPO', not 'Rights requests'.</t>
         </is>
       </c>
       <c r="F14" s="16" t="n"/>
@@ -14657,7 +14657,7 @@
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
-          <t>Add a personal email and end another session from Your profile</t>
+          <t>Add a personal email and end another session from My profile</t>
         </is>
       </c>
       <c r="C44" s="11" t="n">
@@ -14665,12 +14665,12 @@
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>In browser 1, sign in to http://localhost:3000 as rnd@cmp.local with the password and code. Click 'Your profile' in the sidebar.</t>
+          <t>In browser 1, sign in to http://localhost:3000 as rnd@cmp.local with the password and code. Click your name at the top right to open the account menu, then click 'My profile'.</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
         <is>
-          <t>The page 'Your account' opens with three tabs - 'Contacts' (selected), 'Active sessions' with a count, and 'Password' - and the 'Identity' card beside them. Identity shows Name 'Kavya Rao', Role 'R&amp;D User', Status 'Active' and a 'Session expires' time about 8 hours from now.</t>
+          <t>The page 'My profile' opens with three tabs - 'Contacts' (selected), 'Active sessions' with a count, and 'Password' - and the 'Identity' card beside them. Identity shows Name 'Kavya Rao', Role 'R&amp;D User', Status 'Active' and a 'Session expires' time about 8 hours from now.</t>
         </is>
       </c>
       <c r="F44" s="16" t="n"/>
@@ -14684,7 +14684,7 @@
       </c>
       <c r="B45" s="11" t="inlineStr">
         <is>
-          <t>Add a personal email and end another session from Your profile</t>
+          <t>Add a personal email and end another session from My profile</t>
         </is>
       </c>
       <c r="C45" s="11" t="n">
@@ -14711,7 +14711,7 @@
       </c>
       <c r="B46" s="11" t="inlineStr">
         <is>
-          <t>Add a personal email and end another session from Your profile</t>
+          <t>Add a personal email and end another session from My profile</t>
         </is>
       </c>
       <c r="C46" s="11" t="n">
@@ -14738,7 +14738,7 @@
       </c>
       <c r="B47" s="11" t="inlineStr">
         <is>
-          <t>Add a personal email and end another session from Your profile</t>
+          <t>Add a personal email and end another session from My profile</t>
         </is>
       </c>
       <c r="C47" s="11" t="n">
@@ -14765,7 +14765,7 @@
       </c>
       <c r="B48" s="11" t="inlineStr">
         <is>
-          <t>Add a personal email and end another session from Your profile</t>
+          <t>Add a personal email and end another session from My profile</t>
         </is>
       </c>
       <c r="C48" s="11" t="n">
@@ -14792,7 +14792,7 @@
       </c>
       <c r="B49" s="11" t="inlineStr">
         <is>
-          <t>Add a personal email and end another session from Your profile</t>
+          <t>Add a personal email and end another session from My profile</t>
         </is>
       </c>
       <c r="C49" s="11" t="n">
@@ -14800,7 +14800,7 @@
       </c>
       <c r="D49" s="11" t="inlineStr">
         <is>
-          <t>In browser 2, sign in to http://localhost:3000 as rnd@cmp.local with the password and a new code. Go back to browser 1 and refresh the 'Your account' page and click the 'Active sessions' tab.</t>
+          <t>In browser 2, sign in to http://localhost:3000 as rnd@cmp.local with the password and a new code. Go back to browser 1 and refresh the 'My profile' page and click the 'Active sessions' tab.</t>
         </is>
       </c>
       <c r="E49" s="11" t="inlineStr">
@@ -14819,7 +14819,7 @@
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>Add a personal email and end another session from Your profile</t>
+          <t>Add a personal email and end another session from My profile</t>
         </is>
       </c>
       <c r="C50" s="11" t="n">
@@ -14846,7 +14846,7 @@
       </c>
       <c r="B51" s="11" t="inlineStr">
         <is>
-          <t>Add a personal email and end another session from Your profile</t>
+          <t>Add a personal email and end another session from My profile</t>
         </is>
       </c>
       <c r="C51" s="11" t="n">
@@ -14854,7 +14854,7 @@
       </c>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>In browser 2, click any sidebar item (for example 'Projects').</t>
+          <t>In browser 2, click any sidebar item (for example 'My projects').</t>
         </is>
       </c>
       <c r="E51" s="11" t="inlineStr">
@@ -14994,7 +14994,7 @@
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>Both codes are accepted even though a wrong pair was tried first. You are signed in and land on the page headed 'Your consents'.</t>
+          <t>Both codes are accepted even though a wrong pair was tried first. You are signed in and land on the page headed 'My consents'.</t>
         </is>
       </c>
       <c r="F56" s="16" t="n"/>
@@ -15021,7 +15021,7 @@
       </c>
       <c r="E57" s="11" t="inlineStr">
         <is>
-          <t>The header shows 'Tester One' with the role badge 'Data Subject'. The sidebar shows 'My consents', 'My requests', 'Notifications', 'Your profile' and 'Sign out'. There is no 'We need your date of birth' notice.</t>
+          <t>The header shows 'Tester One' with the role badge 'Data Subject'. The sidebar shows 'My consents', 'My requests', 'My nominations', 'Updates' and 'Sign out'; 'My profile' is in the account menu under the name. There is no 'We need your date of birth' notice.</t>
         </is>
       </c>
       <c r="F57" s="16" t="n"/>
@@ -15043,12 +15043,12 @@
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Click 'Your profile'.</t>
+          <t>Click your name at the top right to open the account menu, then click 'My profile'.</t>
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>'Your account' opens. Identity shows Name 'Tester One', Mobile and Email as entered, Role 'Data Subject', Status 'Active' and Date of birth 15 Aug 1990 (no under-18 badge). In Contacts, the mobile and email both show 'Confirmed'.</t>
+          <t>'My profile' opens. Identity shows Name 'Tester One', Mobile and Email as entered, Role 'Data Subject', Status 'Active' and Date of birth 15 Aug 1990 (no under-18 badge). In Contacts, the mobile and email both show 'Confirmed'.</t>
         </is>
       </c>
       <c r="F58" s="16" t="n"/>
@@ -15507,7 +15507,7 @@
       </c>
       <c r="E75" s="11" t="inlineStr">
         <is>
-          <t>You land on the page headed 'Your consents'. The header shows 'Anjali Verma' with the role badge 'Data Subject'.</t>
+          <t>You land on the page headed 'My consents'. The header shows 'Anjali Verma' with the role badge 'Data Subject'.</t>
         </is>
       </c>
       <c r="F75" s="16" t="n"/>
@@ -15534,7 +15534,7 @@
       </c>
       <c r="E76" s="11" t="inlineStr">
         <is>
-          <t>Under 'Your data' are 'My consents' and 'My requests'; under 'You' are 'Notifications' and 'Your profile'; 'Sign out' is at the bottom. There is no staff menu and no staff-account notice.</t>
+          <t>Under 'Your data' are 'My consents', 'My requests', 'My nominations' and 'Updates'; 'Sign out' is at the bottom. 'My profile' is in the account menu under her name at the top right. There is no staff menu and no staff-account notice.</t>
         </is>
       </c>
       <c r="F76" s="16" t="n"/>
@@ -15561,7 +15561,7 @@
       </c>
       <c r="E77" s="11" t="inlineStr">
         <is>
-          <t>The page headed 'Your requests' opens.</t>
+          <t>The page headed 'My requests' opens.</t>
         </is>
       </c>
       <c r="F77" s="16" t="n"/>
@@ -15777,7 +15777,7 @@
       </c>
       <c r="E85" s="11" t="inlineStr">
         <is>
-          <t>The correct code is accepted and you land on 'Your consents' as Anjali Verma.</t>
+          <t>The correct code is accepted and you land on 'My consents' as Anjali Verma.</t>
         </is>
       </c>
       <c r="F85" s="16" t="n"/>
@@ -15831,7 +15831,7 @@
       </c>
       <c r="E87" s="11" t="inlineStr">
         <is>
-          <t>You land on 'Your consents'. Above the list is a blue notice titled 'We need your date of birth' reading 'You can withdraw a consent or make a request without it, but we need it before you give a new consent.' with an 'Add it now' link.</t>
+          <t>You land on 'My consents'. Above the list is a blue notice titled 'We need your date of birth' reading 'You can withdraw a consent or make a request without it, but we need it before you give a new consent.' with an 'Add it now' link.</t>
         </is>
       </c>
       <c r="F87" s="16" t="n"/>
@@ -15858,7 +15858,7 @@
       </c>
       <c r="E88" s="11" t="inlineStr">
         <is>
-          <t>The page 'Your requests' opens normally, with the same 'We need your date of birth' notice above it. Nothing blocks this page.</t>
+          <t>The page 'My requests' opens normally, with the same 'We need your date of birth' notice above it. Nothing blocks this page.</t>
         </is>
       </c>
       <c r="F88" s="16" t="n"/>
@@ -15880,12 +15880,12 @@
       </c>
       <c r="D89" s="11" t="inlineStr">
         <is>
-          <t>Click 'Notifications' in the sidebar.</t>
+          <t>Click 'Updates' in the sidebar.</t>
         </is>
       </c>
       <c r="E89" s="11" t="inlineStr">
         <is>
-          <t>Instead of the notifications, a card headed 'Your date of birth' appears: 'The law protects people under 18 differently, and we do not have your date of birth yet. We need it before you can give a new consent.' It has a 'Date of birth' field, a 'Save and continue' button and links 'withdraw a consent' and 'make a request'.</t>
+          <t>Instead of the updates, a card headed 'Your date of birth' appears: 'The law protects people under 18 differently, and we do not have your date of birth yet. We need it before you can give a new consent.' It has a 'Date of birth' field, a 'Save and continue' button and links 'withdraw a consent' and 'make a request'.</t>
         </is>
       </c>
       <c r="F89" s="16" t="n"/>
@@ -15907,7 +15907,7 @@
       </c>
       <c r="D90" s="11" t="inlineStr">
         <is>
-          <t>Click 'Your profile' in the sidebar.</t>
+          <t>Click your name at the top right to open the account menu, then click 'My profile'.</t>
         </is>
       </c>
       <c r="E90" s="11" t="inlineStr">
@@ -15939,7 +15939,7 @@
       </c>
       <c r="E91" s="11" t="inlineStr">
         <is>
-          <t>'Your requests' opens without answering the question.</t>
+          <t>'My requests' opens without answering the question.</t>
         </is>
       </c>
       <c r="F91" s="16" t="n"/>
@@ -15961,12 +15961,12 @@
       </c>
       <c r="D92" s="11" t="inlineStr">
         <is>
-          <t>Go back to 'Your consents' and click 'Add it now' in the notice.</t>
+          <t>Go back to 'My consents' and click 'Add it now' in the notice.</t>
         </is>
       </c>
       <c r="E92" s="11" t="inlineStr">
         <is>
-          <t>The 'Your date of birth' question is shown so the date can be added. (Record a defect if the link just reloads 'Your consents'.)</t>
+          <t>The 'Your date of birth' question is shown so the date can be added. (Record a defect if the link just reloads 'My consents'.)</t>
         </is>
       </c>
       <c r="F92" s="16" t="n"/>
@@ -15988,7 +15988,7 @@
       </c>
       <c r="D93" s="11" t="inlineStr">
         <is>
-          <t>Click 'Your profile' to reach the 'Your date of birth' card. Type 1 January 2030 into 'Date of birth' and click 'Save and continue'.</t>
+          <t>Open 'My profile' from the account menu to reach the 'Your date of birth' card. Type 1 January 2030 into 'Date of birth' and click 'Save and continue'.</t>
         </is>
       </c>
       <c r="E93" s="11" t="inlineStr">
@@ -16020,7 +16020,7 @@
       </c>
       <c r="E94" s="11" t="inlineStr">
         <is>
-          <t>The card disappears and the 'Your account' page opens. In Identity, 'Date of birth' shows 21 Jul 1985 with no under-18 badge.</t>
+          <t>The card disappears and the 'My profile' page opens. In Identity, 'Date of birth' shows 21 Jul 1985 with no under-18 badge.</t>
         </is>
       </c>
       <c r="F94" s="16" t="n"/>
@@ -16042,12 +16042,12 @@
       </c>
       <c r="D95" s="11" t="inlineStr">
         <is>
-          <t>Click 'My consents' and then 'Notifications'.</t>
+          <t>Click 'My consents' and then 'Updates'.</t>
         </is>
       </c>
       <c r="E95" s="11" t="inlineStr">
         <is>
-          <t>The 'We need your date of birth' notice no longer appears on 'Your consents', and 'Notifications' opens normally.</t>
+          <t>The 'We need your date of birth' notice no longer appears on 'My consents', and 'Updates' opens normally.</t>
         </is>
       </c>
       <c r="F95" s="16" t="n"/>
@@ -16074,7 +16074,7 @@
       </c>
       <c r="E96" s="11" t="inlineStr">
         <is>
-          <t>You land on 'Your consents' with no date-of-birth notice; the question is not asked again.</t>
+          <t>You land on 'My consents' with no date-of-birth notice; the question is not asked again.</t>
         </is>
       </c>
       <c r="F96" s="16" t="n"/>
@@ -16128,7 +16128,7 @@
       </c>
       <c r="E98" s="11" t="inlineStr">
         <is>
-          <t>You land on 'Your consents'. A line across the top reads 'You are signed in with your staff account, as a data principal. Only your own consents, requests and rights are here; your console is a separate site.'</t>
+          <t>You land on 'My consents'. A line across the top reads 'You are signed in with your staff account, as a data principal. Only your own consents, requests and rights are here; your console is a separate site.'</t>
         </is>
       </c>
       <c r="F98" s="16" t="n"/>
@@ -16155,7 +16155,7 @@
       </c>
       <c r="E99" s="11" t="inlineStr">
         <is>
-          <t>The header shows 'Priya Menon' with the role badge 'Data Subject' (not 'DPO'). The sidebar has only 'My consents', 'My requests', 'Notifications', 'Your profile' and 'Sign out'.</t>
+          <t>The header shows 'Priya Menon' with the role badge 'Data Subject' (not 'DPO'). The sidebar has only 'My consents', 'My requests', 'My nominations', 'Updates' and 'Sign out'; 'My profile' is in the account menu.</t>
         </is>
       </c>
       <c r="F99" s="16" t="n"/>
@@ -16177,12 +16177,12 @@
       </c>
       <c r="D100" s="11" t="inlineStr">
         <is>
-          <t>Click 'Your profile'. If the 'Your date of birth' card appears, enter 21 July 1985 and click 'Save and continue'.</t>
+          <t>Click your name at the top right to open the account menu, then click 'My profile'. If the 'Your date of birth' card appears, enter 21 July 1985 and click 'Save and continue'.</t>
         </is>
       </c>
       <c r="E100" s="11" t="inlineStr">
         <is>
-          <t>'Your account' opens. In Identity, Role shows 'Data Subject' and an 'Account' line reads 'Your staff account, used here as a data principal.' In Contacts, the 'Email' row shows dpo@cmp.local with the hint 'Your staff address, managed by your organisation. If you may lose it one day, add a personal one below.' and no 'Change' button.</t>
+          <t>'My profile' opens. In Identity, Role shows 'Data Subject' and an 'Account' line reads 'Your staff account, used here as a data principal.' In Contacts, the 'Email' row shows dpo@cmp.local with the hint 'Your staff address, managed by your organisation. If you may lose it one day, add a personal one below.' and no 'Change' button.</t>
         </is>
       </c>
       <c r="F100" s="16" t="n"/>
@@ -16285,12 +16285,12 @@
       </c>
       <c r="D104" s="11" t="inlineStr">
         <is>
-          <t>Click 'Your profile'.</t>
+          <t>Click your name at the top right to open the account menu, then click 'My profile'.</t>
         </is>
       </c>
       <c r="E104" s="11" t="inlineStr">
         <is>
-          <t>'Your account' opens. Contacts lists 'Email' (tester01@example.org, 'Confirmed', no Change button), 'Mobile' (with 'Change') and 'Second email' ('None given', with 'Add'). Identity shows a 'Session expires' time about 8 hours after you signed in.</t>
+          <t>'My profile' opens. Contacts lists 'Email' (tester01@example.org, 'Confirmed', no Change button), 'Mobile' (with 'Change') and 'Second email' ('None given', with 'Add'). Identity shows a 'Session expires' time about 8 hours after you signed in.</t>
         </is>
       </c>
       <c r="F104" s="16" t="n"/>
@@ -16420,7 +16420,7 @@
       </c>
       <c r="D109" s="11" t="inlineStr">
         <is>
-          <t>Click 'Use a different contact' and sign in with the mobile +91 98111 22301 and its code from the test coordinator. Open 'Your profile'.</t>
+          <t>Click 'Use a different contact' and sign in with the mobile +91 98111 22301 and its code from the test coordinator. Open 'My profile' from the account menu.</t>
         </is>
       </c>
       <c r="E109" s="11" t="inlineStr">
@@ -16479,7 +16479,7 @@
       </c>
       <c r="E111" s="11" t="inlineStr">
         <is>
-          <t>You are signed in as Tester One and land on 'Your consents'.</t>
+          <t>You are signed in as Tester One and land on 'My consents'.</t>
         </is>
       </c>
       <c r="F111" s="16" t="n"/>
@@ -16501,7 +16501,7 @@
       </c>
       <c r="D112" s="11" t="inlineStr">
         <is>
-          <t>Click 'Your profile'. In the 'Mobile' row click 'Change'.</t>
+          <t>Click your name at the top right to open the account menu, then click 'My profile'. In the 'Mobile' row click 'Change'.</t>
         </is>
       </c>
       <c r="E112" s="11" t="inlineStr">
@@ -16695,7 +16695,7 @@
       </c>
       <c r="E119" s="11" t="inlineStr">
         <is>
-          <t>You are signed in as Tester One and land on 'Your consents'.</t>
+          <t>You are signed in as Tester One and land on 'My consents'.</t>
         </is>
       </c>
       <c r="F119" s="16" t="n"/>
@@ -16776,7 +16776,7 @@
       </c>
       <c r="E122" s="11" t="inlineStr">
         <is>
-          <t>You land on 'Your requests' (the page you asked for), not on 'Your consents'.</t>
+          <t>You land on 'My requests' (the page you asked for), not on 'My consents'.</t>
         </is>
       </c>
       <c r="F122" s="16" t="n"/>
@@ -16803,7 +16803,7 @@
       </c>
       <c r="E123" s="11" t="inlineStr">
         <is>
-          <t>The sign-in form does not stay; you are sent to 'Your consents'.</t>
+          <t>The sign-in form does not stay; you are sent to 'My consents'.</t>
         </is>
       </c>
       <c r="F123" s="16" t="n"/>
@@ -16830,7 +16830,7 @@
       </c>
       <c r="E124" s="11" t="inlineStr">
         <is>
-          <t>The sign-up form does not stay; you are sent to 'Your consents'.</t>
+          <t>The sign-up form does not stay; you are sent to 'My consents'.</t>
         </is>
       </c>
       <c r="F124" s="16" t="n"/>
@@ -16857,7 +16857,7 @@
       </c>
       <c r="E125" s="11" t="inlineStr">
         <is>
-          <t>The portal home goes straight to 'Your consents'.</t>
+          <t>The portal home goes straight to 'My consents'.</t>
         </is>
       </c>
       <c r="F125" s="16" t="n"/>
@@ -16906,12 +16906,12 @@
       </c>
       <c r="D127" s="11" t="inlineStr">
         <is>
-          <t>Sign in to http://localhost:3001 with 'Mobile' +91 90000 00001 and the code the test coordinator gives you. Click 'Your profile' and note the 'Session expires' time in Identity.</t>
+          <t>Sign in to http://localhost:3001 with 'Mobile' +91 90000 00001 and the code the test coordinator gives you. Open 'My profile' from the account menu (your name at the top right) and note the 'Session expires' time in Identity.</t>
         </is>
       </c>
       <c r="E127" s="11" t="inlineStr">
         <is>
-          <t>'Your account' opens. 'Session expires' is about 8 hours after the sign-in time (the absolute limit).</t>
+          <t>'My profile' opens. 'Session expires' is about 8 hours after the sign-in time (the absolute limit).</t>
         </is>
       </c>
       <c r="F127" s="16" t="n"/>
@@ -16960,7 +16960,7 @@
       </c>
       <c r="D129" s="11" t="inlineStr">
         <is>
-          <t>After 31 minutes, return to the window and, if you are still on 'Your consents', click 'My requests'.</t>
+          <t>After 31 minutes, return to the window and, if you are still on 'My consents', click 'My requests'.</t>
         </is>
       </c>
       <c r="E129" s="11" t="inlineStr">
@@ -16992,7 +16992,7 @@
       </c>
       <c r="E130" s="11" t="inlineStr">
         <is>
-          <t>You are signed in again and land on the page named in the address ('Your consents' or 'Your requests'), not on a blank or error page.</t>
+          <t>You are signed in again and land on the page named in the address ('My consents' or 'My requests'), not on a blank or error page.</t>
         </is>
       </c>
       <c r="F130" s="16" t="n"/>
@@ -17041,7 +17041,7 @@
       </c>
       <c r="D132" s="11" t="inlineStr">
         <is>
-          <t>In the left-hand sidebar, under 'Oversight', click 'Users'.</t>
+          <t>In the left-hand sidebar, under 'Your work', click 'Users'.</t>
         </is>
       </c>
       <c r="E132" s="11" t="inlineStr">
@@ -17343,7 +17343,7 @@
       </c>
       <c r="E143" s="11" t="inlineStr">
         <is>
-          <t>The sidebar shows the Data Collection Owner's sections (for example 'Projects', 'Collection sites', 'Data sources', 'Delegate') and does NOT show 'Users'.</t>
+          <t>The sidebar shows the Data Collection Owner's pages (for example 'My projects', 'Collection sites', 'Data sources', 'Delegations') and does NOT show 'Users'.</t>
         </is>
       </c>
       <c r="F143" s="16" t="n"/>
@@ -17721,7 +17721,7 @@
       </c>
       <c r="E157" s="11" t="inlineStr">
         <is>
-          <t>There is no 'Users' entry and no 'Messages' entry.</t>
+          <t>There is no 'Users' entry and no 'Message templates' entry.</t>
         </is>
       </c>
       <c r="F157" s="16" t="n"/>
@@ -20119,12 +20119,12 @@
       </c>
       <c r="D246" s="11" t="inlineStr">
         <is>
-          <t>In the sidebar under 'Oversight' click 'Messages'.</t>
+          <t>In the sidebar under 'Your work' click 'Message templates'.</t>
         </is>
       </c>
       <c r="E246" s="11" t="inlineStr">
         <is>
-          <t>The 'Messages' page opens with messages grouped under headings such as 'Sign-in', 'Consent', 'Rights' and 'Staff'.</t>
+          <t>The 'Message templates' page opens with messages grouped under headings such as 'Sign-in', 'Consent', 'Rights' and 'Staff'.</t>
         </is>
       </c>
       <c r="F246" s="16" t="n"/>
@@ -20308,7 +20308,7 @@
       </c>
       <c r="D253" s="11" t="inlineStr">
         <is>
-          <t>Click 'Messages' and find the card 'Staff sign-in code' under 'Sign-in'.</t>
+          <t>In the sidebar under 'Oversight' click 'Message templates' and find the card 'Staff sign-in code' under 'Sign-in'.</t>
         </is>
       </c>
       <c r="E253" s="11" t="inlineStr">
@@ -20443,12 +20443,12 @@
       </c>
       <c r="D258" s="11" t="inlineStr">
         <is>
-          <t>In the sidebar under 'Oversight' click 'Delegate'.</t>
+          <t>In the sidebar under 'Oversight' click 'Delegations'.</t>
         </is>
       </c>
       <c r="E258" s="11" t="inlineStr">
         <is>
-          <t>The 'Delegate' page opens with a 'Delegate my work' button and the cards 'My delegations' ('You have not delegated your work to anybody') and 'Work delegated to me'.</t>
+          <t>The 'Delegations' page opens with a 'Delegate my work' button and the cards 'My delegations' ('You have not delegated your work to anybody') and 'Work delegated to me'.</t>
         </is>
       </c>
       <c r="F258" s="16" t="n"/>
@@ -20578,7 +20578,7 @@
       </c>
       <c r="D263" s="11" t="inlineStr">
         <is>
-          <t>Click 'Delegate'.</t>
+          <t>Click 'Delegations' in the sidebar.</t>
         </is>
       </c>
       <c r="E263" s="11" t="inlineStr">
@@ -20659,7 +20659,7 @@
       </c>
       <c r="D266" s="11" t="inlineStr">
         <is>
-          <t>Click 'Delegate' and click 'End now' on the UAT DCO 01 arrangement.</t>
+          <t>Click 'Delegations' and click 'End now' on the UAT DCO 01 arrangement.</t>
         </is>
       </c>
       <c r="E266" s="11" t="inlineStr">
@@ -20718,7 +20718,7 @@
       </c>
       <c r="E268" s="11" t="inlineStr">
         <is>
-          <t>There is no 'Delegate' entry; the address shows 'Not part of your account' with 'Back to your dashboard'.</t>
+          <t>There is no 'Delegations' entry; the address shows 'Not part of your account' with 'Back to your dashboard'.</t>
         </is>
       </c>
       <c r="F268" s="16" t="n"/>
@@ -20794,7 +20794,7 @@
       </c>
       <c r="D271" s="11" t="inlineStr">
         <is>
-          <t>Click 'Delegate'.</t>
+          <t>Under 'Oversight' click 'Delegations'.</t>
         </is>
       </c>
       <c r="E271" s="11" t="inlineStr">
@@ -20875,7 +20875,7 @@
       </c>
       <c r="D274" s="11" t="inlineStr">
         <is>
-          <t>Click 'Delegate', then 'Delegate my work'.</t>
+          <t>Under 'Oversight' click 'Delegations', then 'Delegate my work'.</t>
         </is>
       </c>
       <c r="E274" s="11" t="inlineStr">
@@ -21339,7 +21339,7 @@
       </c>
       <c r="E291" s="11" t="inlineStr">
         <is>
-          <t>It reads 'Currently In Draft. These are the moves your role can make from here.' and shows one row 'Move to Pending Approval'.</t>
+          <t>It reads 'Currently In Draft. These are the moves your role can make from here.' and shows one row 'Moves the project to Pending Approval' with a 'Submit for approval' button.</t>
         </is>
       </c>
       <c r="F291" s="16" t="n"/>
@@ -21361,7 +21361,7 @@
       </c>
       <c r="D292" s="11" t="inlineStr">
         <is>
-          <t>Read the warning lines under 'Move to Pending Approval'.</t>
+          <t>Read the warning lines under 'Moves the project to Pending Approval'.</t>
         </is>
       </c>
       <c r="E292" s="11" t="inlineStr">
@@ -21388,7 +21388,7 @@
       </c>
       <c r="D293" s="11" t="inlineStr">
         <is>
-          <t>Try to click the 'Pending Approval' button on that row.</t>
+          <t>Try to click the 'Submit for approval' button on that row.</t>
         </is>
       </c>
       <c r="E293" s="11" t="inlineStr">
@@ -21420,7 +21420,7 @@
       </c>
       <c r="E294" s="11" t="inlineStr">
         <is>
-          <t>It shows 'No notice yet' with the buttons 'Upload a notice document' and 'Use an existing notice'.</t>
+          <t>It shows 'No notice yet' with the buttons 'Upload a notice document' and 'Copy an existing notice'.</t>
         </is>
       </c>
       <c r="F294" s="16" t="n"/>
@@ -21474,7 +21474,7 @@
       </c>
       <c r="E296" s="11" t="inlineStr">
         <is>
-          <t>'Edit', 'Upload a notice document', 'Use an existing notice', 'Upload approval' and 'Add site' are shown. There is NO 'New notice' button.</t>
+          <t>'Edit', 'Upload a notice document', 'Copy an existing notice', 'Upload approval' and 'Add site' are shown. There is NO 'New notice' button.</t>
         </is>
       </c>
       <c r="F296" s="16" t="n"/>
@@ -21852,7 +21852,7 @@
       </c>
       <c r="E310" s="11" t="inlineStr">
         <is>
-          <t>It lists 'NTC-UAT-STUDY-01-2026 v1' with '9 purpose(s) · 1 language(s)' and the status badge 'Draft'.</t>
+          <t>It lists 'NTC-UAT-STUDY-01-2026 v1' with '9 purposes · 1 language(s)' and the status badge 'Draft'.</t>
         </is>
       </c>
       <c r="F310" s="16" t="n"/>
@@ -21879,7 +21879,7 @@
       </c>
       <c r="E311" s="11" t="inlineStr">
         <is>
-          <t>Under 'Move to Pending Approval' only one line remains: 'No approval with a proof file'. The 'Pending Approval' button is still disabled.</t>
+          <t>Under 'Moves the project to Pending Approval' only one line remains: 'No approval with a proof file'. The 'Submit for approval' button is still disabled.</t>
         </is>
       </c>
       <c r="F311" s="16" t="n"/>
@@ -21955,12 +21955,12 @@
       </c>
       <c r="D314" s="11" t="inlineStr">
         <is>
-          <t>In the 'Notices' card click 'Use an existing notice'.</t>
+          <t>In the 'Notices' card click 'Copy an existing notice'.</t>
         </is>
       </c>
       <c r="E314" s="11" t="inlineStr">
         <is>
-          <t>A dialog 'Use an existing notice' opens: 'Copies the wording, the purposes and every language rendition into this project as a fresh draft.' with a 'Notice to copy' list and a disabled 'Copy into this project' button.</t>
+          <t>A dialog 'Copy an existing notice' opens: 'Copies the wording, the purposes and every language rendition into this project as a fresh draft.' with a 'Notice to copy' list and a disabled 'Copy into this project' button.</t>
         </is>
       </c>
       <c r="F314" s="16" t="n"/>
@@ -22122,7 +22122,7 @@
       </c>
       <c r="E320" s="11" t="inlineStr">
         <is>
-          <t>'Upload a notice document' and 'Use an existing notice' are shown; there is NO 'New notice' button.</t>
+          <t>'Upload a notice document' and 'Copy an existing notice' are shown; there is NO 'New notice' button.</t>
         </is>
       </c>
       <c r="F320" s="16" t="n"/>
@@ -22203,7 +22203,7 @@
       </c>
       <c r="E323" s="11" t="inlineStr">
         <is>
-          <t>The English wording is displayed read-only with 'Not legally approved — the project cannot be approved until it is'. There is NO 'Edit this rendition' button.</t>
+          <t>The English wording is displayed read-only with 'Not legally approved — the project cannot be approved until it is'. There is NO 'Edit English text' button.</t>
         </is>
       </c>
       <c r="F323" s="16" t="n"/>
@@ -22230,7 +22230,7 @@
       </c>
       <c r="E324" s="11" t="inlineStr">
         <is>
-          <t>Each purpose shows the 'Draft' status. There is NO 'Manage', NO 'Activate' and NO 'Narrow for this notice' button.</t>
+          <t>Each purpose shows the 'Draft' status. There is NO 'Manage', NO 'Activate' and NO 'Customise for this notice' button.</t>
         </is>
       </c>
       <c r="F324" s="16" t="n"/>
@@ -22257,7 +22257,7 @@
       </c>
       <c r="E325" s="11" t="inlineStr">
         <is>
-          <t>The english row shows 'Not legally approved'. There is NO 'Add a rendition', NO 'Edit' and NO 'Approve' button.</t>
+          <t>The english row shows 'Not legally approved'. There is NO 'Add language', NO 'Edit' and NO 'Approve' button.</t>
         </is>
       </c>
       <c r="F325" s="16" t="n"/>
@@ -22419,7 +22419,7 @@
       </c>
       <c r="E331" s="11" t="inlineStr">
         <is>
-          <t>'Move to Pending Approval' has no warning lines and the 'Pending Approval' button is active (highlighted).</t>
+          <t>'Moves the project to Pending Approval' has no warning lines and the 'Submit for approval' button is active (highlighted).</t>
         </is>
       </c>
       <c r="F331" s="16" t="n"/>
@@ -22446,7 +22446,7 @@
       </c>
       <c r="E332" s="11" t="inlineStr">
         <is>
-          <t>A 'Next steps' card repeats 'Move to Pending Approval' with the same active 'Pending Approval' button, and under 'Other actions' the buttons from the top of the page (for example 'Upload approval') with the status badge. Nothing at the top of the page has gone.</t>
+          <t>A 'Next steps' card repeats 'Moves the project to Pending Approval' with the same active 'Submit for approval' button, and under 'Other actions' the buttons from the top of the page (for example 'Upload approval') with the status badge. Nothing at the top of the page has gone.</t>
         </is>
       </c>
       <c r="F332" s="16" t="n"/>
@@ -22468,7 +22468,7 @@
       </c>
       <c r="D333" s="11" t="inlineStr">
         <is>
-          <t>Click 'Pending Approval' (at the top or in 'Next steps' - either one).</t>
+          <t>Click 'Submit for approval' (at the top or in 'Next steps' - either one).</t>
         </is>
       </c>
       <c r="E333" s="11" t="inlineStr">
@@ -22522,7 +22522,7 @@
       </c>
       <c r="D335" s="11" t="inlineStr">
         <is>
-          <t>On the 'Dashboard' look at 'Needs you today'.</t>
+          <t>On the 'Dashboard' look at 'Needs attention'.</t>
         </is>
       </c>
       <c r="E335" s="11" t="inlineStr">
@@ -22581,7 +22581,7 @@
       </c>
       <c r="E337" s="11" t="inlineStr">
         <is>
-          <t>It reads 'Currently Pending Approval.' and offers two rows: 'Move to Approved' (with the tag 'publishes the notice') and 'Move to In Draft'.</t>
+          <t>It reads 'Currently Pending Approval.' and offers two rows: 'Moves the project to Approved' (with the tag 'publishes the notice' and an 'Approve project' button) and 'Moves the project to In Draft' (with a 'Return to draft' button).</t>
         </is>
       </c>
       <c r="F337" s="16" t="n"/>
@@ -22603,12 +22603,12 @@
       </c>
       <c r="D338" s="11" t="inlineStr">
         <is>
-          <t>Read the warning lines under 'Move to Approved'.</t>
+          <t>Read the warning lines under 'Moves the project to Approved'.</t>
         </is>
       </c>
       <c r="E338" s="11" t="inlineStr">
         <is>
-          <t>Both DPO-side blockers are listed: 'The notice text is not legally approved - approve every language on the notice first' with a link 'Approve the notice', and 'The notice carries purposes that are not activated - activate them before approving' with a link 'Open the notice'. The 'Approved' button is disabled.</t>
+          <t>Both DPO-side blockers are listed: 'The notice text is not legally approved - approve every language on the notice first' with a link 'Approve the notice', and 'The notice carries purposes that are not activated - activate them before approving' with a link 'Open the notice'. The 'Approve project' button is disabled.</t>
         </is>
       </c>
       <c r="F338" s="16" t="n"/>
@@ -22630,12 +22630,12 @@
       </c>
       <c r="D339" s="11" t="inlineStr">
         <is>
-          <t>Under 'Move to In Draft' note the hint, then click the 'In Draft' button.</t>
+          <t>Under 'Moves the project to In Draft' note the hint, then click the 'Return to draft' button.</t>
         </is>
       </c>
       <c r="E339" s="11" t="inlineStr">
         <is>
-          <t>The hint reads 'A reason is required and is recorded in the history.' A panel 'Move to In Draft' opens with a required 'Reason' box.</t>
+          <t>The hint reads 'A reason is required and is recorded in the history.' A panel 'Return to draft' opens with a required 'Reason' box.</t>
         </is>
       </c>
       <c r="F339" s="16" t="n"/>
@@ -22657,7 +22657,7 @@
       </c>
       <c r="D340" s="11" t="inlineStr">
         <is>
-          <t>Leave 'Reason' empty and click 'Confirm'.</t>
+          <t>Leave 'Reason' empty and click 'Return to draft' in the panel.</t>
         </is>
       </c>
       <c r="E340" s="11" t="inlineStr">
@@ -22900,12 +22900,12 @@
       </c>
       <c r="D349" s="11" t="inlineStr">
         <is>
-          <t>On notice NTC-UAT-STUDY-01-2026 v1, find the 'Notice text' card and click 'Edit this rendition'.</t>
+          <t>On notice NTC-UAT-STUDY-01-2026 v1, find the 'Notice text' card and click 'Edit English text'.</t>
         </is>
       </c>
       <c r="E349" s="11" t="inlineStr">
         <is>
-          <t>A dialog 'Edit english' opens: 'This exact text is hashed at publication and becomes the record of what was agreed to.' 'Language' is locked to English; 'Notice text' holds the current wording.</t>
+          <t>A dialog 'Edit English text' opens: 'This exact text is hashed at publication and becomes the record of what was agreed to.' 'Language' is locked to English; 'Notice text' holds the current wording.</t>
         </is>
       </c>
       <c r="F349" s="16" t="n"/>
@@ -22927,7 +22927,7 @@
       </c>
       <c r="D350" s="11" t="inlineStr">
         <is>
-          <t>Add the extra sentence at the end of the text and click 'Save rendition'.</t>
+          <t>Add the extra sentence at the end of the text and click 'Save text'.</t>
         </is>
       </c>
       <c r="E350" s="11" t="inlineStr">
@@ -22954,12 +22954,12 @@
       </c>
       <c r="D351" s="11" t="inlineStr">
         <is>
-          <t>In the 'Legal approval, per language' card click 'Add a rendition'.</t>
+          <t>In the 'Legal approval, per language' card click 'Add language'.</t>
         </is>
       </c>
       <c r="E351" s="11" t="inlineStr">
         <is>
-          <t>A dialog 'Add a rendition' opens with 'Language' and 'Notice text'.</t>
+          <t>A dialog 'Add language' opens with 'Language' and 'Notice text'.</t>
         </is>
       </c>
       <c r="F351" s="16" t="n"/>
@@ -22981,7 +22981,7 @@
       </c>
       <c r="D352" s="11" t="inlineStr">
         <is>
-          <t>Choose Language 'Hindi', paste the Hindi text and click 'Save rendition'.</t>
+          <t>Choose Language 'Hindi', paste the Hindi text and click 'Save text'.</t>
         </is>
       </c>
       <c r="E352" s="11" t="inlineStr">
@@ -23143,12 +23143,12 @@
       </c>
       <c r="D358" s="11" t="inlineStr">
         <is>
-          <t>Look at 'Move to Approved' in 'What happens next'.</t>
+          <t>Look at 'Moves the project to Approved' in 'What happens next'.</t>
         </is>
       </c>
       <c r="E358" s="11" t="inlineStr">
         <is>
-          <t>No warning lines remain; the 'Approved' button is active and the row carries the tag 'publishes the notice'.</t>
+          <t>No warning lines remain; the 'Approve project' button is active and the row carries the tag 'publishes the notice'.</t>
         </is>
       </c>
       <c r="F358" s="16" t="n"/>
@@ -23170,12 +23170,12 @@
       </c>
       <c r="D359" s="11" t="inlineStr">
         <is>
-          <t>Click 'Approved'.</t>
+          <t>Click 'Approve project'.</t>
         </is>
       </c>
       <c r="E359" s="11" t="inlineStr">
         <is>
-          <t>A panel 'Move to Approved' opens with a yellow warning: 'This publishes the project's notice. Its text and hash are frozen at that moment and cannot be edited afterwards - a correction requires a new version...' and an optional 'Note (optional)' box.</t>
+          <t>A panel 'Approve project' opens with a yellow warning: 'This publishes the project's notice. Its text and hash are frozen at that moment and cannot be edited afterwards - a correction requires a new version...' and an optional 'Note (optional)' box.</t>
         </is>
       </c>
       <c r="F359" s="16" t="n"/>
@@ -23197,7 +23197,7 @@
       </c>
       <c r="D360" s="11" t="inlineStr">
         <is>
-          <t>Type the note and click 'Confirm'.</t>
+          <t>Type the note and click 'Approve project' in the panel.</t>
         </is>
       </c>
       <c r="E360" s="11" t="inlineStr">
@@ -23364,7 +23364,7 @@
       </c>
       <c r="E366" s="11" t="inlineStr">
         <is>
-          <t>There is NO 'Edit' in the header, NO 'Edit this rendition', NO 'Manage', NO 'Activate', NO 'Narrow for this notice', NO 'Add a rendition' and NO 'Publish this notice'. The 'Publication checklist' card is not shown.</t>
+          <t>There is NO 'Edit' in the header, NO 'Edit English text', NO 'Manage', NO 'Activate', NO 'Customise for this notice', NO 'Add language' and NO 'Publish this notice'. The 'Publication checklist' card is not shown.</t>
         </is>
       </c>
       <c r="F366" s="16" t="n"/>
@@ -25114,7 +25114,7 @@
       </c>
       <c r="D431" s="11" t="inlineStr">
         <is>
-          <t>Open project 'UAT Study 01'. In the header click 'Use an existing notice', choose 'NTC-GAIT-2026 v1 — Gait Identification Study 2026' and click 'Copy into this project'.</t>
+          <t>Open project 'UAT Study 01'. In the header click 'Copy an existing notice', choose 'NTC-GAIT-2026 v1 — Gait Identification Study 2026' and click 'Copy into this project'.</t>
         </is>
       </c>
       <c r="E431" s="11" t="inlineStr">
@@ -25222,7 +25222,7 @@
       </c>
       <c r="D435" s="11" t="inlineStr">
         <is>
-          <t>In a private window open the CIT 'new URL' saved in PRJ-19. Send a code to +91 90000 00001, type the relayed code and click 'Confirm and read the notice'.</t>
+          <t>In a private window open the CIT 'new URL' saved in PRJ-19. Send a code to +91 90000 00001, type the relayed code and click 'Verify and continue'.</t>
         </is>
       </c>
       <c r="E435" s="11" t="inlineStr">
@@ -25281,7 +25281,7 @@
       </c>
       <c r="E437" s="11" t="inlineStr">
         <is>
-          <t>The page opens with a coloured banner showing 'Gait Identification Study 2026' and 'CIT'. A step bar shows 'Your details', 'Confirm', 'The notice', 'Done' with 'Your details' current. A card 'Your details' says consent is recorded against your account so you can read and withdraw it.</t>
+          <t>The page opens with a coloured banner showing 'Gait Identification Study 2026' and 'CIT'. A step bar shows 'Your details', 'Confirm', 'The notice', 'Done' with 'Your details' current. A card 'Your details' says 'Confirm your mobile number or email to read the notice and make your choices.' Because this notice is in more than one language, a 'Read the notice in' drop-down showing 'English' is above 'Send my code to'.</t>
         </is>
       </c>
       <c r="F437" s="16" t="n"/>
@@ -25335,7 +25335,7 @@
       </c>
       <c r="E439" s="11" t="inlineStr">
         <is>
-          <t>The card changes to 'Confirm your mobile': 'We have sent a six-digit code to +91 90000 00001. It expires in ten minutes.' The step bar moves to 'Confirm'.</t>
+          <t>The card changes to 'Confirm your mobile': 'We have sent a six-digit code to +91 90000 00001. It expires in ten minutes.' Below the code box are 'Send a new code' and 'Use a different contact'. The step bar moves to 'Confirm'.</t>
         </is>
       </c>
       <c r="F439" s="16" t="n"/>
@@ -25362,7 +25362,7 @@
       </c>
       <c r="E440" s="11" t="inlineStr">
         <is>
-          <t>The box accepts digits only, and 'Confirm and read the notice' stays greyed out.</t>
+          <t>The box accepts digits only, and 'Verify and continue' stays greyed out.</t>
         </is>
       </c>
       <c r="F440" s="16" t="n"/>
@@ -25384,7 +25384,7 @@
       </c>
       <c r="D441" s="11" t="inlineStr">
         <is>
-          <t>Complete the code with the one the coordinator relays and click 'Confirm and read the notice'.</t>
+          <t>Complete the code with the one the coordinator relays and click 'Verify and continue'.</t>
         </is>
       </c>
       <c r="E441" s="11" t="inlineStr">
@@ -25497,7 +25497,7 @@
       </c>
       <c r="E445" s="11" t="inlineStr">
         <is>
-          <t>The step bar moves to 'Done'. A green tick and the heading 'Your choices are recorded' appear, with 'We have sent you a receipt. You can review or withdraw your consent at any time - withdrawing is as easy as this was.' Below: 'Your reference:' followed by a long code (write it down), and the links 'Review your consents' and 'Your rights'.</t>
+          <t>The step bar moves to 'Done'. A green tick and the heading 'Your choices are recorded' appear, with 'A receipt is on its way to you. You can review or withdraw your consent at any time - withdrawing is as easy as this was.' Below: 'Your reference:' followed by a long code (write it down), and the links 'Review your consents' and 'Your rights'.</t>
         </is>
       </c>
       <c r="F445" s="16" t="n"/>
@@ -25551,7 +25551,7 @@
       </c>
       <c r="E447" s="11" t="inlineStr">
         <is>
-          <t>The portal page 'Your consents' opens, signed in as Anjali, with a card 'Gait Identification Study 2026', status 'Consented' and the line 'You agreed to 2 of 2 purpose(s).'</t>
+          <t>The portal page 'My consents' opens, signed in as Anjali, with a card 'Gait Identification Study 2026', status 'Consented' and the line 'You agreed to both purposes.'</t>
         </is>
       </c>
       <c r="F447" s="16" t="n"/>
@@ -25654,7 +25654,7 @@
       </c>
       <c r="D451" s="11" t="inlineStr">
         <is>
-          <t>Type 123456 in 'Six-digit code' and click 'Confirm and read the notice'.</t>
+          <t>Type 123456 in 'Six-digit code' and click 'Verify and continue'.</t>
         </is>
       </c>
       <c r="E451" s="11" t="inlineStr">
@@ -25735,7 +25735,7 @@
       </c>
       <c r="D454" s="11" t="inlineStr">
         <is>
-          <t>Type 123456 (not the code that was sent) and click 'Confirm and read the notice'.</t>
+          <t>Type 123456 (not the code that was sent) and click 'Verify and continue'.</t>
         </is>
       </c>
       <c r="E454" s="11" t="inlineStr">
@@ -25762,7 +25762,7 @@
       </c>
       <c r="D455" s="11" t="inlineStr">
         <is>
-          <t>Clear the box, type the correct code relayed by the coordinator and click 'Confirm and read the notice'.</t>
+          <t>Clear the box, type the correct code relayed by the coordinator and click 'Verify and continue'.</t>
         </is>
       </c>
       <c r="E455" s="11" t="inlineStr">
@@ -25924,7 +25924,7 @@
       </c>
       <c r="D461" s="11" t="inlineStr">
         <is>
-          <t>Type the code the coordinator relays and click 'Confirm and read the notice'.</t>
+          <t>Type the code the coordinator relays and click 'Verify and continue'.</t>
         </is>
       </c>
       <c r="E461" s="11" t="inlineStr">
@@ -26037,7 +26037,7 @@
       </c>
       <c r="E465" s="11" t="inlineStr">
         <is>
-          <t>'Your consents' opens with a card 'Gait Identification Study 2026' whose small line reads 'NTC-GAIT-2026 v1 · hindi · &lt;date and time&gt;', status 'Partial', and 'You agreed to 1 of 2 purpose(s).'</t>
+          <t>'My consents' opens with a card 'Gait Identification Study 2026' whose small line reads 'NTC-GAIT-2026 v1 · hindi · &lt;date and time&gt;', status 'Partial', and 'You agreed to 1 of 2 purposes.'</t>
         </is>
       </c>
       <c r="F465" s="16" t="n"/>
@@ -26145,7 +26145,7 @@
       </c>
       <c r="E469" s="11" t="inlineStr">
         <is>
-          <t>You are signed in and 'Your consents' opens with the empty message 'No consent records' / 'When you agree to a notice, it will appear here.'</t>
+          <t>You are signed in and 'My consents' opens with the empty message 'No consent records' / 'When you agree to a notice, it will appear here.'</t>
         </is>
       </c>
       <c r="F469" s="16" t="n"/>
@@ -26167,7 +26167,7 @@
       </c>
       <c r="D470" s="11" t="inlineStr">
         <is>
-          <t>In the same browser window open the CIT consent link. Leave 'Mobile' selected, type +91 98100 00022, click 'Send the code', type the relayed code and click 'Confirm and read the notice'.</t>
+          <t>In the same browser window open the CIT consent link. Leave 'Mobile' selected, type +91 98100 00022, click 'Send the code', type the relayed code and click 'Verify and continue'.</t>
         </is>
       </c>
       <c r="E470" s="11" t="inlineStr">
@@ -26226,7 +26226,7 @@
       </c>
       <c r="E472" s="11" t="inlineStr">
         <is>
-          <t>The card 'Gait Identification Study 2026' shows status 'Declined' and 'You were asked about 2 purpose(s) and agreed to none.' The first button reads 'See what you were asked'. There is no 'Withdraw everything' button.</t>
+          <t>The card 'Gait Identification Study 2026' shows status 'Declined' and 'You were asked about 2 purposes and agreed to none.' The first button reads 'See what you were asked'. There is no 'Withdraw everything' button.</t>
         </is>
       </c>
       <c r="F472" s="16" t="n"/>
@@ -26302,7 +26302,7 @@
       </c>
       <c r="D475" s="11" t="inlineStr">
         <is>
-          <t>Type the code the coordinator relays and click 'Confirm and read the notice'.</t>
+          <t>Type the code the coordinator relays and click 'Verify and continue'.</t>
         </is>
       </c>
       <c r="E475" s="11" t="inlineStr">
@@ -26442,7 +26442,7 @@
       </c>
       <c r="E480" s="11" t="inlineStr">
         <is>
-          <t>'Your consents' shows the card 'Gait Identification Study 2026' with status 'Consented' and 'You agreed to 2 of 2 purpose(s).'</t>
+          <t>'My consents' shows the card 'Gait Identification Study 2026' with status 'Consented' and 'You agreed to both purposes.'</t>
         </is>
       </c>
       <c r="F480" s="16" t="n"/>
@@ -26464,7 +26464,7 @@
       </c>
       <c r="D481" s="11" t="inlineStr">
         <is>
-          <t>Open the CIT consent link again in a new private window, identify with dcoadmin@cmp.local and the new code, and click 'Confirm and read the notice'.</t>
+          <t>Open the CIT consent link again in a new private window, identify with dcoadmin@cmp.local and the new code, and click 'Verify and continue'.</t>
         </is>
       </c>
       <c r="E481" s="11" t="inlineStr">
@@ -26680,7 +26680,7 @@
       </c>
       <c r="D489" s="11" t="inlineStr">
         <is>
-          <t>Type the relayed code and click 'Confirm and read the notice'.</t>
+          <t>Type the relayed code and click 'Verify and continue'.</t>
         </is>
       </c>
       <c r="E489" s="11" t="inlineStr">
@@ -26820,7 +26820,7 @@
       </c>
       <c r="E494" s="11" t="inlineStr">
         <is>
-          <t>'Your consents' shows 'No consent records'.</t>
+          <t>'My consents' shows 'No consent records'.</t>
         </is>
       </c>
       <c r="F494" s="16" t="n"/>
@@ -26842,7 +26842,7 @@
       </c>
       <c r="D495" s="11" t="inlineStr">
         <is>
-          <t>Click 'Your profile' in the sidebar and look at 'Date of birth'.</t>
+          <t>Click your name at the top right to open the account menu, click 'My profile' and look at 'Date of birth'.</t>
         </is>
       </c>
       <c r="E495" s="11" t="inlineStr">
@@ -27063,7 +27063,7 @@
       </c>
       <c r="E503" s="11" t="inlineStr">
         <is>
-          <t>After 'Send me a code' a blue box 'Check your messages' says 'If tester01@example.org is registered with us, a six-digit code is on its way. It expires in ten minutes.' After 'Verify' the page 'Your consents' opens and 'My consents' is highlighted in the sidebar.</t>
+          <t>After 'Send me a code' a blue box 'Check your messages' says 'If tester01@example.org is registered with us, a six-digit code is on its way. It expires in ten minutes.' After 'Verify' the page 'My consents' opens and 'My consents' is highlighted in the sidebar.</t>
         </is>
       </c>
       <c r="F503" s="16" t="n"/>
@@ -27090,7 +27090,7 @@
       </c>
       <c r="E504" s="11" t="inlineStr">
         <is>
-          <t>Description: 'Everything you have agreed to, the exact wording you were shown, and who it has been shared with. You can withdraw at any time.' The card shows 'NTC-GAIT-2026 v1 · hindi · &lt;date and time&gt;', status 'Partial', 'You agreed to 1 of 2 purpose(s).' and the buttons 'See what you agreed to', 'What was recorded', 'Withdraw everything' and 'Ask about this consent'.</t>
+          <t>Description: 'Everything you have agreed to, the exact wording you were shown, and who it has been shared with. You can withdraw at any time.' The card shows 'NTC-GAIT-2026 v1 · hindi · &lt;date and time&gt;', status 'Partial', 'You agreed to 1 of 2 purposes.' and the buttons 'See what you agreed to', 'What was recorded', 'Withdraw everything' and 'Ask about this consent'.</t>
         </is>
       </c>
       <c r="F504" s="16" t="n"/>
@@ -27198,7 +27198,7 @@
       </c>
       <c r="E508" s="11" t="inlineStr">
         <is>
-          <t>Before any export (CON-14): 'Not shared with anyone' / 'No export containing your record has been generated.' After CON-14: an entry naming the processor 'SEED' with the project name and date.</t>
+          <t>Before any export (CON-14): 'No sharing recorded here' / 'This lists every file of your details this platform has sent to a processor. None has been sent.' After CON-14: an entry naming the processor 'SEED' with the project name and date.</t>
         </is>
       </c>
       <c r="F508" s="16" t="n"/>
@@ -27252,7 +27252,7 @@
       </c>
       <c r="E510" s="11" t="inlineStr">
         <is>
-          <t>After 'Send me a code' a blue box 'Check your messages' says 'If dcoadmin@cmp.local is registered with us, a six-digit code is on its way. It expires in ten minutes.' After 'Verify' the page 'Your consents' opens and 'My consents' is highlighted in the sidebar.</t>
+          <t>After 'Send me a code' a blue box 'Check your messages' says 'If dcoadmin@cmp.local is registered with us, a six-digit code is on its way. It expires in ten minutes.' After 'Verify' the page 'My consents' opens and 'My consents' is highlighted in the sidebar.</t>
         </is>
       </c>
       <c r="F510" s="16" t="n"/>
@@ -27274,7 +27274,7 @@
       </c>
       <c r="D511" s="11" t="inlineStr">
         <is>
-          <t>On the card 'Gait Identification Study 2026' (status 'Consented', 'You agreed to 2 of 2 purpose(s).') click 'Withdraw everything'.</t>
+          <t>On the card 'Gait Identification Study 2026' (status 'Consented', 'You agreed to both purposes.') click 'Withdraw everything'.</t>
         </is>
       </c>
       <c r="E511" s="11" t="inlineStr">
@@ -27360,7 +27360,7 @@
       </c>
       <c r="E514" s="11" t="inlineStr">
         <is>
-          <t>The status is 'Withdrawn' and the text reads 'You were asked about 2 purpose(s) and agreed to none.' The 'Withdraw everything' button is gone.</t>
+          <t>The status is 'Withdrawn' and the text reads 'You were asked about 2 purposes and agreed to none.' The 'Withdraw everything' button is gone.</t>
         </is>
       </c>
       <c r="F514" s="16" t="n"/>
@@ -27468,7 +27468,7 @@
       </c>
       <c r="E518" s="11" t="inlineStr">
         <is>
-          <t>'Your consents' opens — it is NOT replaced by a date-of-birth question. A blue note 'We need your date of birth' reads 'You can withdraw a consent or make a request without it, but we need it before you give a new consent.' with a link 'Add it now'.</t>
+          <t>'My consents' opens — it is NOT replaced by a date-of-birth question. A blue note 'We need your date of birth' reads 'You can withdraw a consent or make a request without it, but we need it before you give a new consent.' with a link 'Add it now'.</t>
         </is>
       </c>
       <c r="F518" s="16" t="n"/>
@@ -27522,7 +27522,7 @@
       </c>
       <c r="E520" s="11" t="inlineStr">
         <is>
-          <t>'Your profile' opens and shows the card 'Your date of birth' with 'Save and continue'. Do not enter a date.</t>
+          <t>'My profile' opens and shows the card 'Your date of birth' with 'Save and continue'. Do not enter a date.</t>
         </is>
       </c>
       <c r="F520" s="16" t="n"/>
@@ -27571,7 +27571,7 @@
       </c>
       <c r="D522" s="11" t="inlineStr">
         <is>
-          <t>Click 'Your profile' in the sidebar.</t>
+          <t>Click your name at the top right to open the account menu, then click 'My profile'.</t>
         </is>
       </c>
       <c r="E522" s="11" t="inlineStr">
@@ -27603,7 +27603,7 @@
       </c>
       <c r="E523" s="11" t="inlineStr">
         <is>
-          <t>'Your consents' opens again, with the note.</t>
+          <t>'My consents' opens again, with the note.</t>
         </is>
       </c>
       <c r="F523" s="16" t="n"/>
@@ -28030,7 +28030,7 @@
       </c>
       <c r="D539" s="11" t="inlineStr">
         <is>
-          <t>As the RCO click 'Projects', type 'Gait Identification' in 'Search' (the list updates as you type), open 'Gait Identification Study 2026', click 'Generate export' and then 'Generate the export'.</t>
+          <t>As the RCO click 'My projects', type 'Gait Identification' in 'Search' (the list updates as you type), open 'Gait Identification Study 2026', click 'Generate export' and then 'Generate the export'.</t>
         </is>
       </c>
       <c r="E539" s="11" t="inlineStr">
@@ -29790,7 +29790,7 @@
       </c>
       <c r="E604" s="11" t="inlineStr">
         <is>
-          <t>After 'Send me a code' a blue box 'Check your messages' says 'If +91 90000 00001 is registered with us, a six-digit code is on its way. It expires in ten minutes.' After 'Verify' the page 'Your consents' opens and 'My consents' is highlighted in the sidebar.</t>
+          <t>After 'Send me a code' a blue box 'Check your messages' says 'If +91 90000 00001 is registered with us, a six-digit code is on its way. It expires in ten minutes.' After 'Verify' the page 'My consents' opens and 'My consents' is highlighted in the sidebar.</t>
         </is>
       </c>
       <c r="F604" s="16" t="n"/>
@@ -29898,7 +29898,7 @@
       </c>
       <c r="E608" s="11" t="inlineStr">
         <is>
-          <t>The line reads 'You agreed to 1 of 2 purpose(s).' 'Recording quality assurance' now shows 'Declined' and 'Gait model training' still shows 'Consented'. The status badge reads 'Partial', not 'Withdrawn'.</t>
+          <t>The line reads 'You agreed to 1 of 2 purposes.' 'Recording quality assurance' now shows 'Declined' and 'Gait model training' still shows 'Consented'. The status badge reads 'Partial', not 'Withdrawn'.</t>
         </is>
       </c>
       <c r="F608" s="16" t="n"/>
@@ -30060,7 +30060,7 @@
       </c>
       <c r="E614" s="11" t="inlineStr">
         <is>
-          <t>The page 'Your requests' opens with the text 'Ask for access to your data, a correction, erasure, or raise a grievance...' and a 'Make a request' button at the top right. Lower down is the card 'Somebody to act for you'.</t>
+          <t>The page 'My requests' opens with the text 'Ask for access to your data, a correction or erasure, or raise a complaint...' and a 'Make a request' button at the top right. At the foot of the page a line says naming someone to act for you is under 'My nominations'.</t>
         </is>
       </c>
       <c r="F614" s="16" t="n"/>
@@ -30595,7 +30595,7 @@
       </c>
       <c r="D634" s="11" t="inlineStr">
         <is>
-          <t>In the same dialog change 'What are you asking for' to 'Grievance (s.13)'.</t>
+          <t>In the same dialog change 'What are you asking for' to 'Complaint (grievance) (s.13)'.</t>
         </is>
       </c>
       <c r="E634" s="11" t="inlineStr">
@@ -31221,7 +31221,7 @@
       </c>
       <c r="E657" s="11" t="inlineStr">
         <is>
-          <t>The Dashboard opens, signed in as Priya Menon (DPO). The sidebar shows 'Rights requests' under 'Oversight'.</t>
+          <t>The Dashboard opens, signed in as Priya Menon (DPO). The sidebar shows 'Rights requests' under 'Your work'.</t>
         </is>
       </c>
       <c r="F657" s="16" t="n"/>
@@ -31788,7 +31788,7 @@
       </c>
       <c r="E678" s="11" t="inlineStr">
         <is>
-          <t>It reads 'Third-party data removed. The DPO signs off - nothing releases automatically. An access response is a file she downloads from her own account.' There is no yellow warning, and 'Outcome' shows 'Complete'.</t>
+          <t>It reads 'Third-party data removed. The DPO signs off - nothing releases automatically. An access response is a file the requester downloads from their own account.' There is no yellow warning, and 'Outcome' shows 'Complete'.</t>
         </is>
       </c>
       <c r="F678" s="16" t="n"/>
@@ -31869,7 +31869,7 @@
       </c>
       <c r="E681" s="11" t="inlineStr">
         <is>
-          <t>The message 'Released and closed' with 'She has been told; 1 file released with the response.' appears. The header badge reads 'Complete'. A 'Response' card shows 'Complete · &lt;date&gt; · downloadable by her until &lt;date&gt;', the response text, a 'Download the file' button and 'Released with the response' listing access-extract.pdf.</t>
+          <t>The message 'Released and closed' with 'The requester has been told; 1 file released with the response.' appears. The header badge reads 'Complete'. A 'Response' card shows 'Complete · &lt;date&gt; · downloadable by the requester until &lt;date&gt;', the response text, a 'Download the file' button and 'Released with the response' listing access-extract.pdf.</t>
         </is>
       </c>
       <c r="F681" s="16" t="n"/>
@@ -32085,7 +32085,7 @@
       </c>
       <c r="E689" s="11" t="inlineStr">
         <is>
-          <t>It is headed 'Does she mean erasure, or withdrawal?' and explains 'Withdrawal stops future processing and is hers to do from her consent record... Confirm which before anything is deleted.' with buttons 'She means erasure' and 'She meant withdrawal'.</t>
+          <t>It is headed 'Does the requester mean erasure, or withdrawal?' and explains 'Withdrawal stops future processing, and the requester can do it from their consent record... Confirm which before anything is deleted.' with buttons 'They mean erasure' and 'They meant withdrawal'.</t>
         </is>
       </c>
       <c r="F689" s="16" t="n"/>
@@ -32161,7 +32161,7 @@
       </c>
       <c r="D692" s="11" t="inlineStr">
         <is>
-          <t>Click 'She means erasure'.</t>
+          <t>Click 'They mean erasure'.</t>
         </is>
       </c>
       <c r="E692" s="11" t="inlineStr">
@@ -32242,7 +32242,7 @@
       </c>
       <c r="D695" s="11" t="inlineStr">
         <is>
-          <t>In Browser B open RR-W and click 'She meant withdrawal'.</t>
+          <t>In Browser B open RR-W and click 'They meant withdrawal'.</t>
         </is>
       </c>
       <c r="E695" s="11" t="inlineStr">
@@ -32490,7 +32490,7 @@
       </c>
       <c r="E704" s="11" t="inlineStr">
         <is>
-          <t>A blue note reads 'Consent artefacts are never erased. They are the evidence that past processing was lawful...' and the card says 'No scope yet. Derive it from the records she appears in.' with a button 'Derive from asset_consent'.</t>
+          <t>A blue note reads 'Consent artefacts are never erased. They are the evidence that past processing was lawful...' and the card says 'No scope yet. Derive it from the records the requester appears in.' with a button 'Derive from asset_consent'.</t>
         </is>
       </c>
       <c r="F704" s="16" t="n"/>
@@ -32517,7 +32517,7 @@
       </c>
       <c r="E705" s="11" t="inlineStr">
         <is>
-          <t>'Scope derived' with '2 appearances of her in collected assets.' appears. Two rows show: asset A with its type badge and 'only her', and asset B with a warning badge 'holds 1 other person'. Each row names the project, source (SRC-SRIB-SE), 'held by SRIB' and the collection date.</t>
+          <t>'Scope derived' with '2 appearances of the requester in collected assets.' appears. Two rows show: asset A with its type badge and 'only the requester', and asset B with a warning badge 'holds 1 other person'. Each row names the project, source (SRC-SRIB-SE), 'held by SRIB' and the collection date.</t>
         </is>
       </c>
       <c r="F705" s="16" t="n"/>
@@ -32544,7 +32544,7 @@
       </c>
       <c r="E706" s="11" t="inlineStr">
         <is>
-          <t>'Decision' shows 'Erase - the asset holds only her'. 'Basis' is empty and 'Record the decision' is greyed out.</t>
+          <t>'Decision' shows 'Erase - the asset holds only the requester'. 'Basis' is empty and 'Record the decision' is greyed out.</t>
         </is>
       </c>
       <c r="F706" s="16" t="n"/>
@@ -32647,7 +32647,7 @@
       </c>
       <c r="D710" s="11" t="inlineStr">
         <is>
-          <t>Change 'Decision' to 'Erase - the asset holds only her', replace the basis with the erase basis and click 'Record the decision'.</t>
+          <t>Change 'Decision' to 'Erase - the asset holds only the requester', replace the basis with the erase basis and click 'Record the decision'.</t>
         </is>
       </c>
       <c r="E710" s="11" t="inlineStr">
@@ -32679,7 +32679,7 @@
       </c>
       <c r="E711" s="11" t="inlineStr">
         <is>
-          <t>The four options are 'Erase - the asset holds only her', 'Redact - remove her, keep the others', 'Retain - a floor binds, erased when it passes' and 'Quarantine - removal cannot be assured; the DPO decides'.</t>
+          <t>The four options are 'Erase - the asset holds only the requester', 'Redact - remove the requester, keep the others', 'Retain - a floor binds, erased when it passes' and 'Quarantine - removal cannot be assured; the DPO decides'.</t>
         </is>
       </c>
       <c r="F711" s="16" t="n"/>
@@ -32706,7 +32706,7 @@
       </c>
       <c r="E712" s="11" t="inlineStr">
         <is>
-          <t>The row carries the warning badge 'holds 1 other person'. 'Decision' is preset to 'Redact - remove her, keep the others'. Beside the button: 'Erase is not offered: deleting this asset would erase the other people's validly given consent.'</t>
+          <t>The row carries the warning badge 'holds 1 other person'. 'Decision' is preset to 'Redact - remove the requester, keep the others'. Beside the button: 'Erase is not offered: deleting this asset would erase the other people's validly given consent.'</t>
         </is>
       </c>
       <c r="F712" s="16" t="n"/>
@@ -32728,7 +32728,7 @@
       </c>
       <c r="D713" s="11" t="inlineStr">
         <is>
-          <t>Open 'Decision' and try to choose 'Erase - the asset holds only her'.</t>
+          <t>Open 'Decision' and try to choose 'Erase - the asset holds only the requester'.</t>
         </is>
       </c>
       <c r="E713" s="11" t="inlineStr">
@@ -32755,7 +32755,7 @@
       </c>
       <c r="D714" s="11" t="inlineStr">
         <is>
-          <t>Keep 'Redact - remove her, keep the others', type the redact basis and click 'Record the decision'.</t>
+          <t>Keep 'Redact - remove the requester, keep the others', type the redact basis and click 'Record the decision'.</t>
         </is>
       </c>
       <c r="E714" s="11" t="inlineStr">
@@ -33030,7 +33030,7 @@
       </c>
       <c r="E724" s="11" t="inlineStr">
         <is>
-          <t>RR-E shows 'Awaiting holders'. Nothing on her card says her data has been erased.</t>
+          <t>RR-E shows 'Waiting for responses'. Nothing on her card says her data has been erased.</t>
         </is>
       </c>
       <c r="F724" s="16" t="n"/>
@@ -33044,7 +33044,7 @@
       </c>
       <c r="B725" s="11" t="inlineStr">
         <is>
-          <t>In-house respondent answers the ticket on 'Tickets for you' (thread, attach file, return)</t>
+          <t>In-house respondent answers the ticket on 'My tasks' (thread, attach file, return)</t>
         </is>
       </c>
       <c r="C725" s="11" t="n">
@@ -33057,7 +33057,7 @@
       </c>
       <c r="E725" s="11" t="inlineStr">
         <is>
-          <t>Meera Iyer's dashboard opens. Under 'You' the sidebar shows 'Tickets for you' with a count; there is no 'Rights requests' link.</t>
+          <t>Meera Iyer's dashboard opens. Under 'Your work' the sidebar shows 'My tasks' with a count; there is no 'Rights requests' link.</t>
         </is>
       </c>
       <c r="F725" s="16" t="n"/>
@@ -33071,7 +33071,7 @@
       </c>
       <c r="B726" s="11" t="inlineStr">
         <is>
-          <t>In-house respondent answers the ticket on 'Tickets for you' (thread, attach file, return)</t>
+          <t>In-house respondent answers the ticket on 'My tasks' (thread, attach file, return)</t>
         </is>
       </c>
       <c r="C726" s="11" t="n">
@@ -33098,7 +33098,7 @@
       </c>
       <c r="B727" s="11" t="inlineStr">
         <is>
-          <t>In-house respondent answers the ticket on 'Tickets for you' (thread, attach file, return)</t>
+          <t>In-house respondent answers the ticket on 'My tasks' (thread, attach file, return)</t>
         </is>
       </c>
       <c r="C727" s="11" t="n">
@@ -33106,12 +33106,12 @@
       </c>
       <c r="D727" s="11" t="inlineStr">
         <is>
-          <t>Click 'Tickets for you'.</t>
+          <t>Click 'My tasks'.</t>
         </is>
       </c>
       <c r="E727" s="11" t="inlineStr">
         <is>
-          <t>The page 'Tickets for you' shows tiles 'Open', 'Overdue', 'Due within 7 days', 'Unread from the Privacy Office' and a section 'Open · 1'. The ticket card shows RR-E, 'Erasure · s.12(3)', 'Issued', 'For SRIB · about Anjali Verma · issued &lt;date&gt;', the due date and an 'Instruction'.</t>
+          <t>The page 'My tasks' shows tiles 'Open', 'Overdue', 'Due within 7 days', 'Unread from the Privacy Office' and a section 'Open · 1'. The ticket card shows RR-E, 'Erasure · s.12(3)', 'Issued', 'For SRIB · about Anjali Verma · issued &lt;date&gt;', the due date and an 'Instruction'.</t>
         </is>
       </c>
       <c r="F727" s="16" t="n"/>
@@ -33125,7 +33125,7 @@
       </c>
       <c r="B728" s="11" t="inlineStr">
         <is>
-          <t>In-house respondent answers the ticket on 'Tickets for you' (thread, attach file, return)</t>
+          <t>In-house respondent answers the ticket on 'My tasks' (thread, attach file, return)</t>
         </is>
       </c>
       <c r="C728" s="11" t="n">
@@ -33152,7 +33152,7 @@
       </c>
       <c r="B729" s="11" t="inlineStr">
         <is>
-          <t>In-house respondent answers the ticket on 'Tickets for you' (thread, attach file, return)</t>
+          <t>In-house respondent answers the ticket on 'My tasks' (thread, attach file, return)</t>
         </is>
       </c>
       <c r="C729" s="11" t="n">
@@ -33179,7 +33179,7 @@
       </c>
       <c r="B730" s="11" t="inlineStr">
         <is>
-          <t>In-house respondent answers the ticket on 'Tickets for you' (thread, attach file, return)</t>
+          <t>In-house respondent answers the ticket on 'My tasks' (thread, attach file, return)</t>
         </is>
       </c>
       <c r="C730" s="11" t="n">
@@ -33206,7 +33206,7 @@
       </c>
       <c r="B731" s="11" t="inlineStr">
         <is>
-          <t>In-house respondent answers the ticket on 'Tickets for you' (thread, attach file, return)</t>
+          <t>In-house respondent answers the ticket on 'My tasks' (thread, attach file, return)</t>
         </is>
       </c>
       <c r="C731" s="11" t="n">
@@ -33233,7 +33233,7 @@
       </c>
       <c r="B732" s="11" t="inlineStr">
         <is>
-          <t>In-house respondent answers the ticket on 'Tickets for you' (thread, attach file, return)</t>
+          <t>In-house respondent answers the ticket on 'My tasks' (thread, attach file, return)</t>
         </is>
       </c>
       <c r="C732" s="11" t="n">
@@ -33260,7 +33260,7 @@
       </c>
       <c r="B733" s="11" t="inlineStr">
         <is>
-          <t>In-house respondent answers the ticket on 'Tickets for you' (thread, attach file, return)</t>
+          <t>In-house respondent answers the ticket on 'My tasks' (thread, attach file, return)</t>
         </is>
       </c>
       <c r="C733" s="11" t="n">
@@ -33268,7 +33268,7 @@
       </c>
       <c r="D733" s="11" t="inlineStr">
         <is>
-          <t>In Browser C reload 'Tickets for you'.</t>
+          <t>In Browser C reload 'My tasks'.</t>
         </is>
       </c>
       <c r="E733" s="11" t="inlineStr">
@@ -33287,7 +33287,7 @@
       </c>
       <c r="B734" s="11" t="inlineStr">
         <is>
-          <t>In-house respondent answers the ticket on 'Tickets for you' (thread, attach file, return)</t>
+          <t>In-house respondent answers the ticket on 'My tasks' (thread, attach file, return)</t>
         </is>
       </c>
       <c r="C734" s="11" t="n">
@@ -33314,7 +33314,7 @@
       </c>
       <c r="B735" s="11" t="inlineStr">
         <is>
-          <t>In-house respondent answers the ticket on 'Tickets for you' (thread, attach file, return)</t>
+          <t>In-house respondent answers the ticket on 'My tasks' (thread, attach file, return)</t>
         </is>
       </c>
       <c r="C735" s="11" t="n">
@@ -33341,7 +33341,7 @@
       </c>
       <c r="B736" s="11" t="inlineStr">
         <is>
-          <t>In-house respondent answers the ticket on 'Tickets for you' (thread, attach file, return)</t>
+          <t>In-house respondent answers the ticket on 'My tasks' (thread, attach file, return)</t>
         </is>
       </c>
       <c r="C736" s="11" t="n">
@@ -33368,7 +33368,7 @@
       </c>
       <c r="B737" s="11" t="inlineStr">
         <is>
-          <t>In-house respondent answers the ticket on 'Tickets for you' (thread, attach file, return)</t>
+          <t>In-house respondent answers the ticket on 'My tasks' (thread, attach file, return)</t>
         </is>
       </c>
       <c r="C737" s="11" t="n">
@@ -33462,7 +33462,7 @@
       </c>
       <c r="E740" s="11" t="inlineStr">
         <is>
-          <t>'Released and closed' with 'She has been told the response is ready.' appears. The header badge reads 'Complete' and a 'Response' card shows 'Complete · &lt;date&gt; ...'.</t>
+          <t>'Released and closed' with 'The requester has been told the response is ready.' appears. The header badge reads 'Complete' and a 'Response' card shows 'Complete · &lt;date&gt; ...'.</t>
         </is>
       </c>
       <c r="F740" s="16" t="n"/>
@@ -33646,7 +33646,7 @@
       </c>
       <c r="D747" s="11" t="inlineStr">
         <is>
-          <t>In Browser B open RR-H: click 'Confirm classification', then 'She means erasure', then 'In progress' in 'What happens next'.</t>
+          <t>In Browser B open RR-H: click 'Confirm classification', then 'They mean erasure', then 'In progress' in 'What happens next'.</t>
         </is>
       </c>
       <c r="E747" s="11" t="inlineStr">
@@ -33700,12 +33700,12 @@
       </c>
       <c r="D749" s="11" t="inlineStr">
         <is>
-          <t>In the scope card click 'Derive from asset_consent'. On asset H keep 'Erase - the asset holds only her', type the erase basis and click 'Record the decision'.</t>
+          <t>In the scope card click 'Derive from asset_consent'. On asset H keep 'Erase - the asset holds only the requester', type the erase basis and click 'Record the decision'.</t>
         </is>
       </c>
       <c r="E749" s="11" t="inlineStr">
         <is>
-          <t>'Scope derived' shows 1 appearance; asset H shows 'only her' and 'decided: erase'.</t>
+          <t>'Scope derived' shows 1 appearance; asset H shows 'only the requester' and 'decided: erase'.</t>
         </is>
       </c>
       <c r="F749" s="16" t="n"/>
@@ -33808,7 +33808,7 @@
       </c>
       <c r="D753" s="11" t="inlineStr">
         <is>
-          <t>In Browser C (Meera) open 'Tickets for you', click 'Respond' on RR-H, type the return text, tick 'This is my return - close the ticket with it' and click 'Return the ticket'.</t>
+          <t>In Browser C (Meera) open 'My tasks', click 'Respond' on RR-H, type the return text, tick 'This is my return - close the ticket with it' and click 'Return the ticket'.</t>
         </is>
       </c>
       <c r="E753" s="11" t="inlineStr">
@@ -33997,7 +33997,7 @@
       </c>
       <c r="D760" s="11" t="inlineStr">
         <is>
-          <t>In Browser B open RR-P, click 'Confirm classification', 'She means erasure' and then 'In progress'. Do NOT derive or add holders.</t>
+          <t>In Browser B open RR-P, click 'Confirm classification', 'They mean erasure' and then 'In progress'. Do NOT derive or add holders.</t>
         </is>
       </c>
       <c r="E760" s="11" t="inlineStr">
@@ -34029,7 +34029,7 @@
       </c>
       <c r="E761" s="11" t="inlineStr">
         <is>
-          <t>One row, asset P, 'only her', undecided.</t>
+          <t>One row, asset P, 'only the requester', undecided.</t>
         </is>
       </c>
       <c r="F761" s="16" t="n"/>
@@ -34380,7 +34380,7 @@
       </c>
       <c r="E774" s="11" t="inlineStr">
         <is>
-          <t>The hint reads 'What she is being given, and what could not be provided.' 'Released and closed' appears and the badge reads 'Partial'.</t>
+          <t>The hint reads 'What the requester is being given, and what could not be provided.' 'Released and closed' appears and the badge reads 'Partial'.</t>
         </is>
       </c>
       <c r="F774" s="16" t="n"/>
@@ -34515,7 +34515,7 @@
       </c>
       <c r="E779" s="11" t="inlineStr">
         <is>
-          <t>RR-G shows 'Grievance · s.13', 'Received' and a box 'What you disputed' naming RR-A with 'Complete: &lt;start of the answer&gt;' and 'See RR-A in full'. RR-A shows 'You disputed this in RR-G' with 'See it'.</t>
+          <t>RR-G shows 'Complaint (grievance) · s.13', 'Received' and a box 'What you disputed' naming RR-A with 'Complete: &lt;start of the answer&gt;' and 'See RR-A in full'. RR-A shows 'You disputed this in RR-G' with 'See it'.</t>
         </is>
       </c>
       <c r="F779" s="16" t="n"/>
@@ -34569,7 +34569,7 @@
       </c>
       <c r="E781" s="11" t="inlineStr">
         <is>
-          <t>The line under the heading reads 'Grievance · s.13 · Portal'. 'About' shows RR-A with 'the request under dispute, shown below', and a card 'The request under dispute' shows RR-A's dates, what was asked and its answer.</t>
+          <t>The line under the heading reads 'Complaint (grievance) · s.13 · Portal'. 'About' shows RR-A with 'the request under dispute, shown below', and a card 'The request under dispute' shows RR-A's dates, what was asked and its answer.</t>
         </is>
       </c>
       <c r="F781" s="16" t="n"/>
@@ -34618,7 +34618,7 @@
       </c>
       <c r="D783" s="11" t="inlineStr">
         <is>
-          <t>Click 'Confirm classification' (Grievance (s.13)) and then 'In progress'.</t>
+          <t>Click 'Confirm classification' (Complaint (grievance) (s.13)) and then 'In progress'.</t>
         </is>
       </c>
       <c r="E783" s="11" t="inlineStr">
@@ -34699,7 +34699,7 @@
       </c>
       <c r="D786" s="11" t="inlineStr">
         <is>
-          <t>In Browser A click 'Make a request', choose 'Grievance (s.13)', type the text, tick 'This complaint is about the Data Protection Officer's own decisions.' and click 'Send the request'.</t>
+          <t>In Browser A click 'Make a request', choose 'Complaint (grievance) (s.13)', type the text, tick 'This complaint is about the Data Protection Officer's own decisions.' and click 'Send the request'.</t>
         </is>
       </c>
       <c r="E786" s="11" t="inlineStr">
@@ -35023,7 +35023,7 @@
       </c>
       <c r="D798" s="11" t="inlineStr">
         <is>
-          <t>In Browser A on 'My requests' scroll to 'Somebody to act for you'.</t>
+          <t>In Browser A click 'My nominations' in the sidebar and find the card 'Somebody to act for you'.</t>
         </is>
       </c>
       <c r="E798" s="11" t="inlineStr">
@@ -35050,7 +35050,7 @@
       </c>
       <c r="D799" s="11" t="inlineStr">
         <is>
-          <t>Fill in the test data, untick 'Correction (s.12)' and 'Grievance (s.13)', and click 'Nominate'.</t>
+          <t>Fill in the test data, untick 'Correction (s.12)' and 'Complaint (grievance) (s.13)', and click 'Nominate'.</t>
         </is>
       </c>
       <c r="E799" s="11" t="inlineStr">
@@ -35239,7 +35239,7 @@
       </c>
       <c r="D806" s="11" t="inlineStr">
         <is>
-          <t>In Browser A reload 'My requests'.</t>
+          <t>In Browser A reload 'My nominations'.</t>
         </is>
       </c>
       <c r="E806" s="11" t="inlineStr">
@@ -35536,12 +35536,12 @@
       </c>
       <c r="D817" s="11" t="inlineStr">
         <is>
-          <t>In Browser A (Anjali) reload 'My requests'.</t>
+          <t>In Browser A (Anjali) open 'My nominations'.</t>
         </is>
       </c>
       <c r="E817" s="11" t="inlineStr">
         <is>
-          <t>The nomination card shows 'Rahul Verma acted for you on &lt;date&gt;' with 'They reported that you cannot act for yourself. You keep this account and can follow the request they made. Their request is RR-N, under your requests above. The Privacy Office found the event evidenced on &lt;date&gt;.'</t>
+          <t>The nomination card shows 'Rahul Verma acted for you on &lt;date&gt;' with 'They reported that you cannot act for yourself. You keep this account and can follow the request they made. Their request is RR-N, under My requests. The Privacy Office found the event evidenced on &lt;date&gt;.'</t>
         </is>
       </c>
       <c r="F817" s="16" t="n"/>
@@ -35563,7 +35563,7 @@
       </c>
       <c r="D818" s="11" t="inlineStr">
         <is>
-          <t>In Browser D sign in at http://localhost:3001/sign-in with 'Mobile' and +91 90000 00077 (code from the coordinator), then open 'My requests'.</t>
+          <t>In Browser D sign in at http://localhost:3001/sign-in with 'Mobile' and +91 90000 00077 (code from the coordinator), then open 'My nominations'.</t>
         </is>
       </c>
       <c r="E818" s="11" t="inlineStr">
@@ -35698,7 +35698,7 @@
       </c>
       <c r="D823" s="11" t="inlineStr">
         <is>
-          <t>In Browser A on 'My requests' click 'Revoke this nomination'.</t>
+          <t>In Browser A on 'My nominations' click 'Revoke this nomination'.</t>
         </is>
       </c>
       <c r="E823" s="11" t="inlineStr">
@@ -35779,7 +35779,7 @@
       </c>
       <c r="D826" s="11" t="inlineStr">
         <is>
-          <t>In Browser D (signed in as the nominee) reload 'My requests'.</t>
+          <t>In Browser D (signed in as the nominee) reload 'My nominations'.</t>
         </is>
       </c>
       <c r="E826" s="11" t="inlineStr">
@@ -36022,12 +36022,12 @@
       </c>
       <c r="D835" s="11" t="inlineStr">
         <is>
-          <t>Look at the first card, 'Needs you today'.</t>
+          <t>Look at the first card, 'Needs attention'.</t>
         </is>
       </c>
       <c r="E835" s="11" t="inlineStr">
         <is>
-          <t>Each row shows a number, a label and an arrow, and the card's top right says how many things there are (e.g. '3 things'). Every label is one of: 'Tickets past their date', 'Rights requests overdue', 'Rights requests due within 7 days', 'Requests awaiting verification', 'Teams have written on their tickets', 'Grievances about the DPO to escalate', 'Retention floors passed, erasure due', 'Tickets addressed to you', 'Notice text awaiting approval', 'Projects pending approval', 'New collectors awaiting your decision'. If nothing is waiting the card says 'Nothing needs you today. The queues below are clear or waiting on somebody else.'</t>
+          <t>Each row shows a number, a label and an arrow; the card's heading carries no overall count. Every label is one of: 'Breach duties overdue', 'Breach duties outstanding', 'Tickets past their date', 'Rights requests overdue', 'Rights requests due within 7 days', 'Requests awaiting verification', 'Teams have written on their tickets', 'Grievances about the DPO to escalate', 'Retention floors passed, erasure due', 'Tickets addressed to you', 'Notice text awaiting approval', 'Projects pending approval', 'New collectors awaiting your decision'. If nothing is waiting the card says 'Nothing needs your attention. The queues below are clear or waiting on somebody else.'</t>
         </is>
       </c>
       <c r="F835" s="16" t="n"/>
@@ -36054,7 +36054,7 @@
       </c>
       <c r="E836" s="11" t="inlineStr">
         <is>
-          <t>There is no row about lockouts, sign-ins, access denials, 'Staff invitations not yet accepted', 'Sites awaiting a data source', 'Sources with nobody accountable' or 'Imports that did not reconcile'.</t>
+          <t>There is no row about lockouts, sign-ins, access denials, 'Staff invitations not yet accepted', 'Sites awaiting a data source', 'Sources without an owner' or 'Imports that did not reconcile'.</t>
         </is>
       </c>
       <c r="F836" s="16" t="n"/>
@@ -36076,7 +36076,7 @@
       </c>
       <c r="D837" s="11" t="inlineStr">
         <is>
-          <t>Click one of the rows in 'Needs you today' (for example 'Projects pending approval' or 'Rights requests due within 7 days').</t>
+          <t>Click one of the rows in 'Needs attention' (for example 'Projects pending approval' or 'Rights requests due within 7 days').</t>
         </is>
       </c>
       <c r="E837" s="11" t="inlineStr">
@@ -36103,12 +36103,12 @@
       </c>
       <c r="D838" s="11" t="inlineStr">
         <is>
-          <t>Scroll down past 'Needs you today' to the queue cards.</t>
+          <t>Scroll down past 'Needs attention' to the queue cards.</t>
         </is>
       </c>
       <c r="E838" s="11" t="inlineStr">
         <is>
-          <t>Queues with work appear as cards named from: 'Rights requests, soonest due first', 'Tickets past their date', 'Teams have written on their tickets', 'Drafts whose purposes are not activated', 'Pending Approval', 'New collectors awaiting your decision', 'Retention floors passed - erasure due'. Each card shows a count badge. Empty queues are listed together in one grey line that starts 'Clear:'. People's names in queue rows are readable.</t>
+          <t>Queues with work appear as cards, in this order: 'Tickets past their date', 'Rights requests, soonest due first', 'Teams have written on their tickets', 'Retention floors passed - erasure due', 'Pending Approval', 'New collectors awaiting your decision', 'Drafts whose purposes are not activated'. Each card shows a count badge; a queue at its 25-row limit shows '25+' and a 'See all' link. Empty queues are listed together in one grey line that starts 'Clear:'. People's names in queue rows are readable.</t>
         </is>
       </c>
       <c r="F838" s="16" t="n"/>
@@ -36135,7 +36135,7 @@
       </c>
       <c r="E839" s="11" t="inlineStr">
         <is>
-          <t>'Projects by stage' shows bars labelled 'In draft', 'Pending approval' and 'Approved' with numbers; 'Consent position' shows one bar split into 'Still standing' and 'Withdrawn' with the caption 'Every record counted once, at its current state.'</t>
+          <t>'Projects by stage' shows bars labelled 'In draft', 'Pending approval' and 'Approved' with numbers; 'Consent position' shows one bar split into 'Agreed to all purposes', 'Agreed to some', 'Declined' and 'Withdrawn' with the caption 'Every record counted once, at its current state.'</t>
         </is>
       </c>
       <c r="F839" s="16" t="n"/>
@@ -36243,7 +36243,7 @@
       </c>
       <c r="E843" s="11" t="inlineStr">
         <is>
-          <t>It reads 'Accounts, lockouts, and the state of the processor and source registry.'</t>
+          <t>It reads 'Invitations waiting, access problems, grievances about the DPO, and the processor and source registry.'</t>
         </is>
       </c>
       <c r="F843" s="16" t="n"/>
@@ -36265,12 +36265,12 @@
       </c>
       <c r="D844" s="11" t="inlineStr">
         <is>
-          <t>Look at 'Needs you today'.</t>
+          <t>Look at 'Needs attention'.</t>
         </is>
       </c>
       <c r="E844" s="11" t="inlineStr">
         <is>
-          <t>Only these labels can appear (each only when its count is above zero): 'Staff invitations not yet accepted', 'Grievances about the DPO to review', 'Tickets addressed to you'. Otherwise the card says 'Nothing needs you today. The queues below are clear or waiting on somebody else.'</t>
+          <t>Only these labels can appear (each only when its count is above zero): 'Staff invitations not yet accepted', 'Grievances about the DPO to review', 'Tickets addressed to you'. Otherwise the card says 'Nothing needs your attention. The queues below are clear or waiting on somebody else.'</t>
         </is>
       </c>
       <c r="F844" s="16" t="n"/>
@@ -36292,7 +36292,7 @@
       </c>
       <c r="D845" s="11" t="inlineStr">
         <is>
-          <t>Check 'Needs you today' for rows the administrator cannot act on.</t>
+          <t>Check 'Needs attention' for rows the administrator cannot act on.</t>
         </is>
       </c>
       <c r="E845" s="11" t="inlineStr">
@@ -36351,7 +36351,7 @@
       </c>
       <c r="E847" s="11" t="inlineStr">
         <is>
-          <t>The queues are 'Grievances about the DPO - yours to review', 'Lockouts (24h)' and 'Suspended sources and processors' (as cards, or named in the 'Clear:' line when empty). A lockout from the last 24 hours appears as a row in 'Lockouts (24h)' with the person's readable name - here, and not in 'Needs you today'.</t>
+          <t>The queues are 'Grievances about the DPO - yours to review', 'Lockouts (24h)' and 'Suspended sources and processors' (as cards, or named in the 'Clear:' line when empty). A lockout from the last 24 hours appears as a row in 'Lockouts (24h)' with the person's readable name - here, and not in 'Needs attention'.</t>
         </is>
       </c>
       <c r="F847" s="16" t="n"/>
@@ -36454,12 +36454,12 @@
       </c>
       <c r="D851" s="11" t="inlineStr">
         <is>
-          <t>Read the line under the heading, then look at 'Needs you today'.</t>
+          <t>Read the line under the heading, then look at 'Needs attention'.</t>
         </is>
       </c>
       <c r="E851" s="11" t="inlineStr">
         <is>
-          <t>The line reads 'Your approved projects, the links collecting against them, and anything that failed to reconcile on import.' 'Needs you today' holds only rows from: 'Tickets past their date', 'Tickets addressed to you', 'Imports that did not reconcile', 'Assets with unmapped subjects' - or the sentence 'Nothing needs you today. ...'.</t>
+          <t>The line reads 'Your approved projects, the links collecting against them, and anything that failed to reconcile on import.' 'Needs attention' holds only rows from: 'Tickets past their date', 'Tickets addressed to you', 'Imports that did not reconcile', 'Assets with unmapped subjects' - or the sentence 'Nothing needs your attention. ...'.</t>
         </is>
       </c>
       <c r="F851" s="16" t="n"/>
@@ -36481,7 +36481,7 @@
       </c>
       <c r="D852" s="11" t="inlineStr">
         <is>
-          <t>Check 'Needs you today' for rows belonging to other roles.</t>
+          <t>Check 'Needs attention' for rows belonging to other roles.</t>
         </is>
       </c>
       <c r="E852" s="11" t="inlineStr">
@@ -36513,7 +36513,7 @@
       </c>
       <c r="E853" s="11" t="inlineStr">
         <is>
-          <t>A card row names a collection and a project and says '&lt;n&gt; declared, &lt;m&gt; mapped — &lt;k&gt; unaccounted for'. Clicking it opens that collection's page (not 'Not part of your account'). Use Back to return.</t>
+          <t>The queues are 'Import exceptions' and 'Approved projects ready to collect' (as cards, or named in the 'Clear:' line). An 'Import exceptions' row names a collection and a project and says '&lt;n&gt; declared, &lt;m&gt; mapped — &lt;k&gt; unaccounted for'. Clicking it opens that collection's page (not 'Not part of your account'). Use Back to return.</t>
         </is>
       </c>
       <c r="F853" s="16" t="n"/>
@@ -36589,12 +36589,12 @@
       </c>
       <c r="D856" s="11" t="inlineStr">
         <is>
-          <t>Read the line under the heading and 'Needs you today'.</t>
+          <t>Read the line under the heading and 'Needs attention'.</t>
         </is>
       </c>
       <c r="E856" s="11" t="inlineStr">
         <is>
-          <t>The line reads 'The collection your team runs itself — your approved projects, the links collecting against them, and anything that failed to reconcile on import.' 'Needs you today' uses the same four DCO labels only.</t>
+          <t>The line reads 'The collection your team runs itself — your approved projects, the links collecting against them, and anything that failed to reconcile on import.' 'Needs attention' uses the same four DCO labels only.</t>
         </is>
       </c>
       <c r="F856" s="16" t="n"/>
@@ -36670,12 +36670,12 @@
       </c>
       <c r="D859" s="11" t="inlineStr">
         <is>
-          <t>Read the line under the heading and look at 'Needs you today'.</t>
+          <t>Read the line under the heading and look at 'Needs attention'.</t>
         </is>
       </c>
       <c r="E859" s="11" t="inlineStr">
         <is>
-          <t>The line reads 'Projects collected by a third party: which sites are still waiting for a data source, and who picks them up when you attach one.' Rows come only from: 'Tickets past their date', 'Sites awaiting a data source', 'Sources with nobody accountable', 'Processors with no collection set up', 'Tickets addressed to you'.</t>
+          <t>The line reads 'Projects collected by a third party: which sites are still waiting for a data source, and who picks them up when you attach one.' Rows come only from: 'Tickets past their date', 'Sites awaiting a data source', 'Sources without an owner', 'Processors with no collection set up', 'Tickets addressed to you'.</t>
         </is>
       </c>
       <c r="F859" s="16" t="n"/>
@@ -36724,7 +36724,7 @@
       </c>
       <c r="D861" s="11" t="inlineStr">
         <is>
-          <t>If 'Sources with nobody accountable' is listed, click it.</t>
+          <t>If 'Sources without an owner' is listed, click it.</t>
         </is>
       </c>
       <c r="E861" s="11" t="inlineStr">
@@ -36805,7 +36805,7 @@
       </c>
       <c r="D864" s="11" t="inlineStr">
         <is>
-          <t>Read the line under the heading and look at 'Needs you today'.</t>
+          <t>Read the line under the heading and look at 'Needs attention'.</t>
         </is>
       </c>
       <c r="E864" s="11" t="inlineStr">
@@ -36864,7 +36864,7 @@
       </c>
       <c r="E866" s="11" t="inlineStr">
         <is>
-          <t>'Projects by stage' is shown (counting only Kavya's projects); there is no 'Consent position' card; 'Recent activity' has no 'Full audit trail' link.</t>
+          <t>A 'Waiting for DPO review' queue lists Kavya's projects pending approval (or is named in the 'Clear:' line). 'Projects by stage' is shown (counting only Kavya's projects); there is no 'Consent position' card; 'Recent activity' has no 'Full audit trail' link.</t>
         </is>
       </c>
       <c r="F866" s="16" t="n"/>
@@ -36918,7 +36918,7 @@
       </c>
       <c r="E868" s="11" t="inlineStr">
         <is>
-          <t>In this order: OVERVIEW - Dashboard; GOVERNANCE - Projects, Approvals, Notices, Purposes; CONSENT - Consents, Consent links, Collection sites; REGISTRY - Processors, Data sources; DATA MOVEMENT - Collections, Exports, Imports; OVERSIGHT - Rights requests, Audit trail, Users, Delegate, Messages; YOU - Tickets for you, Notifications, Your profile. A 'Sign out' button sits at the bottom.</t>
+          <t>In this order: YOUR WORK - Dashboard, Rights requests, Breaches, My tasks, Projects, Notices; GOVERNANCE - Approval documents, Purposes; CONSENT - Consents, Consent links, Collection sites; REGISTRY - Processors, Data sources; DATA MOVEMENT - Collections, Exports, Imports; OVERSIGHT - Audit trail, Users, Delegations, Message templates. There is no 'My profile' or 'Notifications' entry: 'My profile' is in the account menu (click your name at the top right) and notifications open from the bell in the header. A 'Sign out' button sits at the bottom.</t>
         </is>
       </c>
       <c r="F868" s="16" t="n"/>
@@ -36945,7 +36945,7 @@
       </c>
       <c r="E869" s="11" t="inlineStr">
         <is>
-          <t>Every link opens a page with its own heading. None shows 'This page could not be found' or 'Not part of your account'. The link for the open page is highlighted.</t>
+          <t>Every link opens a page with its own heading. None shows 'We can't find that page' or 'Not part of your account'. The link for the open page is highlighted.</t>
         </is>
       </c>
       <c r="F869" s="16" t="n"/>
@@ -36999,7 +36999,7 @@
       </c>
       <c r="E871" s="11" t="inlineStr">
         <is>
-          <t>OVERVIEW - Dashboard; REGISTRY - Processors, Data sources; OVERSIGHT - Grievances about the DPO, Audit trail, Users, Delegate, Messages; YOU - Tickets for you, Notifications, Your profile.</t>
+          <t>YOUR WORK - Dashboard, Users, Grievances about the DPO, Message templates, Processors, Data sources, Audit trail; OVERSIGHT - Delegations; YOU - My tasks.</t>
         </is>
       </c>
       <c r="F871" s="16" t="n"/>
@@ -37026,7 +37026,7 @@
       </c>
       <c r="E872" s="11" t="inlineStr">
         <is>
-          <t>There are no GOVERNANCE, CONSENT or DATA MOVEMENT headings and no links to Projects, Approvals, Notices, Purposes, Consents, Consent links, Collection sites, Collections, Exports or Imports. There is no 'Rights requests' link - that slot reads 'Grievances about the DPO'.</t>
+          <t>There are no GOVERNANCE, CONSENT, REGISTRY or DATA MOVEMENT headings and no links to Projects, Approval documents, Notices, Purposes, Consents, Consent links, Collection sites, Collections, Exports or Imports. There is no 'Rights requests' link - that slot reads 'Grievances about the DPO'.</t>
         </is>
       </c>
       <c r="F872" s="16" t="n"/>
@@ -37080,7 +37080,7 @@
       </c>
       <c r="E874" s="11" t="inlineStr">
         <is>
-          <t>Every link opens a page with its own heading; none shows 'This page could not be found' or 'Not part of your account'.</t>
+          <t>Every link opens a page with its own heading; none shows 'We can't find that page' or 'Not part of your account'.</t>
         </is>
       </c>
       <c r="F874" s="16" t="n"/>
@@ -37134,7 +37134,7 @@
       </c>
       <c r="E876" s="11" t="inlineStr">
         <is>
-          <t>OVERVIEW - Dashboard; GOVERNANCE - Projects; CONSENT - Consents, Consent links, Collection sites; REGISTRY - Data sources; DATA MOVEMENT - Collections, Exports, Imports; OVERSIGHT - Delegate; YOU - Tickets for you, Notifications, Your profile.</t>
+          <t>YOUR WORK - Dashboard, My projects, Collection sites, Consent links, My tasks, Collections; CONSENT - Consents; REGISTRY - Data sources; DATA MOVEMENT - Exports, Imports; OVERSIGHT - Delegations. 'My profile' is in the account menu and notifications open from the bell in the header.</t>
         </is>
       </c>
       <c r="F876" s="16" t="n"/>
@@ -37161,7 +37161,7 @@
       </c>
       <c r="E877" s="11" t="inlineStr">
         <is>
-          <t>OVERSIGHT holds only 'Delegate'. There is no 'Audit trail', 'Users', 'Rights requests' or 'Messages', and no 'Approvals', 'Notices', 'Purposes' or 'Processors' anywhere in the sidebar.</t>
+          <t>OVERSIGHT holds only 'Delegations'. There is no 'Audit trail', 'Users', 'Rights requests' or 'Message templates', and no 'Approval documents', 'Notices', 'Purposes' or 'Processors' anywhere in the sidebar.</t>
         </is>
       </c>
       <c r="F877" s="16" t="n"/>
@@ -37188,7 +37188,7 @@
       </c>
       <c r="E878" s="11" t="inlineStr">
         <is>
-          <t>Every link opens a page with its own heading; none shows 'This page could not be found' or 'Not part of your account'.</t>
+          <t>Every link opens a page with its own heading; none shows 'We can't find that page' or 'Not part of your account'.</t>
         </is>
       </c>
       <c r="F878" s="16" t="n"/>
@@ -37242,7 +37242,7 @@
       </c>
       <c r="E880" s="11" t="inlineStr">
         <is>
-          <t>Exactly the same links as the DCO; no 'Audit trail', 'Users', 'Rights requests', 'Messages', 'Approvals', 'Notices', 'Purposes' or 'Processors'.</t>
+          <t>YOUR WORK - Dashboard, Collection sites, Data sources, My tasks, Consent links, Projects; CONSENT - Consents; DATA MOVEMENT - Collections, Exports, Imports; OVERSIGHT - Delegations. These are the DCO's pages in a different order, and the projects link reads 'Projects' (not 'My projects'). No 'Audit trail', 'Users', 'Rights requests', 'Message templates', 'Approval documents', 'Notices', 'Purposes' or 'Processors'.</t>
         </is>
       </c>
       <c r="F880" s="16" t="n"/>
@@ -37296,7 +37296,7 @@
       </c>
       <c r="E882" s="11" t="inlineStr">
         <is>
-          <t>Exactly the same links as the DCO; no 'Audit trail' and none of the other absent links.</t>
+          <t>Exactly the same links, in the same order, as the DCO (including 'My projects'); no 'Audit trail' and none of the other absent links.</t>
         </is>
       </c>
       <c r="F882" s="16" t="n"/>
@@ -37350,7 +37350,7 @@
       </c>
       <c r="E884" s="11" t="inlineStr">
         <is>
-          <t>OVERVIEW - Dashboard; GOVERNANCE - Projects, Approvals, Notices; REGISTRY - Processors; DATA MOVEMENT - Collections, Imports; YOU - Tickets for you, Notifications, Your profile.</t>
+          <t>YOUR WORK - Dashboard, My projects, Approval documents, My tasks, Notices; REGISTRY - Processors; DATA MOVEMENT - Collections, Imports. 'My profile' is in the account menu and notifications open from the bell in the header.</t>
         </is>
       </c>
       <c r="F884" s="16" t="n"/>
@@ -37377,7 +37377,7 @@
       </c>
       <c r="E885" s="11" t="inlineStr">
         <is>
-          <t>There is no CONSENT heading and no OVERSIGHT heading. There are no links to Purposes, Consents, Consent links, Collection sites, Data sources, Exports, Rights requests, Audit trail, Users, Delegate or Messages.</t>
+          <t>There is no CONSENT heading and no OVERSIGHT heading. There are no links to Purposes, Consents, Consent links, Collection sites, Data sources, Exports, Rights requests, Audit trail, Users, Delegations or Message templates.</t>
         </is>
       </c>
       <c r="F885" s="16" t="n"/>
@@ -37431,7 +37431,7 @@
       </c>
       <c r="E887" s="11" t="inlineStr">
         <is>
-          <t>Every link opens a page with its own heading; none shows 'This page could not be found' or 'Not part of your account'.</t>
+          <t>Every link opens a page with its own heading; none shows 'We can't find that page' or 'Not part of your account'.</t>
         </is>
       </c>
       <c r="F887" s="16" t="n"/>
@@ -37750,7 +37750,7 @@
       </c>
       <c r="D899" s="11" t="inlineStr">
         <is>
-          <t>In the sidebar under YOU, click 'Notifications' (the bell icon).</t>
+          <t>Click the bell icon at the top right of the header (its label is 'Notifications').</t>
         </is>
       </c>
       <c r="E899" s="11" t="inlineStr">
@@ -37863,7 +37863,7 @@
       </c>
       <c r="E903" s="11" t="inlineStr">
         <is>
-          <t>The consent record page opens, headed with the person's name and an 'All consents' back link - not 'Not part of your account' and not 'This page could not be found'.</t>
+          <t>The consent record page opens, headed with the person's name and an 'All consents' back link - not 'Not part of your account' and not 'We can't find that page'.</t>
         </is>
       </c>
       <c r="F903" s="16" t="n"/>
@@ -37917,7 +37917,7 @@
       </c>
       <c r="E905" s="11" t="inlineStr">
         <is>
-          <t>Each link opens a page the DPO can use; none shows 'Not part of your account' or 'This page could not be found'.</t>
+          <t>Each link opens a page the DPO can use; none shows 'Not part of your account' or 'We can't find that page'.</t>
         </is>
       </c>
       <c r="F905" s="16" t="n"/>
@@ -37966,7 +37966,7 @@
       </c>
       <c r="D907" s="11" t="inlineStr">
         <is>
-          <t>In the sidebar under YOU, click 'Notifications'.</t>
+          <t>Click the bell icon at the top right of the header.</t>
         </is>
       </c>
       <c r="E907" s="11" t="inlineStr">
@@ -38155,7 +38155,7 @@
       </c>
       <c r="D914" s="11" t="inlineStr">
         <is>
-          <t>Click 'Notifications' in the sidebar and read the list.</t>
+          <t>Click the bell icon in the header to open 'Notifications', and read the list.</t>
         </is>
       </c>
       <c r="E914" s="11" t="inlineStr">
@@ -38209,12 +38209,12 @@
       </c>
       <c r="D916" s="11" t="inlineStr">
         <is>
-          <t>Note the project named on two entries, then click 'Projects' in the sidebar.</t>
+          <t>Note the project named on two entries, then click 'My projects' in the sidebar.</t>
         </is>
       </c>
       <c r="E916" s="11" t="inlineStr">
         <is>
-          <t>Both projects are in Arun's Projects list - no entry concerns a project he cannot see.</t>
+          <t>Both projects are in Arun's projects list - no entry concerns a project he cannot see.</t>
         </is>
       </c>
       <c r="F916" s="16" t="n"/>
@@ -38317,7 +38317,7 @@
       </c>
       <c r="D920" s="11" t="inlineStr">
         <is>
-          <t>Click 'Notifications' and read the list.</t>
+          <t>Click the bell icon in the header and read the 'Notifications' list.</t>
         </is>
       </c>
       <c r="E920" s="11" t="inlineStr">
@@ -39667,7 +39667,7 @@
       </c>
       <c r="D970" s="11" t="inlineStr">
         <is>
-          <t>Click 'Consents', open a record, then open a project from 'Projects'.</t>
+          <t>Click 'Consents', open a record, then open a project from 'My projects'.</t>
         </is>
       </c>
       <c r="E970" s="11" t="inlineStr">
@@ -39915,7 +39915,7 @@
       </c>
       <c r="E979" s="11" t="inlineStr">
         <is>
-          <t>The details show 'Reason given' yes/no and no reason text. The button opens the 'Delegate' page. If it shows 'This page could not be found', record a defect.</t>
+          <t>The details show 'Reason given' yes/no and no reason text. The button opens the 'Delegations' page. If it shows 'We can't find that page', record a defect.</t>
         </is>
       </c>
       <c r="F979" s="16" t="n"/>
@@ -40212,7 +40212,7 @@
       </c>
       <c r="E990" s="11" t="inlineStr">
         <is>
-          <t>The 'Your consents' page opens. The sidebar shows YOUR DATA - 'My consents', 'My requests' and YOU - 'Notifications', 'Your profile', and nothing else.</t>
+          <t>The 'My consents' page opens. The sidebar shows YOUR DATA - 'My consents', 'My requests', 'My nominations' and 'Updates', and nothing else; 'My profile' is in the account menu under her name at the top right.</t>
         </is>
       </c>
       <c r="F990" s="16" t="n"/>
@@ -40234,12 +40234,12 @@
       </c>
       <c r="D991" s="11" t="inlineStr">
         <is>
-          <t>Click 'Notifications'.</t>
+          <t>Click 'Updates'.</t>
         </is>
       </c>
       <c r="E991" s="11" t="inlineStr">
         <is>
-          <t>The page 'Notifications' opens with 'What has happened that concerns you, taken from the audit trail itself.' Entries are about Anjali only, e.g. 'Consent given', 'Consent withdrawn', 'Notice served', 'Subject registered', 'Rights request received'. If there are none it says 'Nothing to report'.</t>
+          <t>The page 'Updates' opens with 'What has happened that concerns you, taken from the audit trail itself.' Entries are about Anjali only, e.g. 'Consent given', 'Consent withdrawn', 'Notice served', 'Subject registered', 'Rights request received'. If there are none it says 'Nothing to report'.</t>
         </is>
       </c>
       <c r="F991" s="16" t="n"/>
@@ -40320,7 +40320,7 @@
       </c>
       <c r="E994" s="11" t="inlineStr">
         <is>
-          <t>The 'Your consents' page on the portal opens - not a staff page and not 'Not part of your account'.</t>
+          <t>The 'My consents' page on the portal opens - not a staff page and not 'Not part of your account'.</t>
         </is>
       </c>
       <c r="F994" s="16" t="n"/>
@@ -40342,12 +40342,12 @@
       </c>
       <c r="D995" s="11" t="inlineStr">
         <is>
-          <t>Back on 'Notifications', click the record link on a rights request entry (if present) and on a 'Subject registered' entry ('Account: Anjali Verma' / 'Open account').</t>
+          <t>Back on 'Updates', click the record link on a rights request entry (if present) and on a 'Subject registered' entry ('Account: Anjali Verma' / 'Open account').</t>
         </is>
       </c>
       <c r="E995" s="11" t="inlineStr">
         <is>
-          <t>The request link opens 'My requests'. The account link opens her own account page ('Your account'). If either shows 'This page could not be found', record a defect.</t>
+          <t>The request link opens 'My requests'. The account link opens her own account page ('My profile'). If either shows 'We can't find that page', record a defect.</t>
         </is>
       </c>
       <c r="F995" s="16" t="n"/>
@@ -40374,7 +40374,7 @@
       </c>
       <c r="E996" s="11" t="inlineStr">
         <is>
-          <t>Both show the '404 | This page could not be found.' page - no staff screen exists on the portal.</t>
+          <t>Both show the portal's 404 page, headed 'We can't find that page', with the buttons 'Go to My consents' and 'Your rights' - no staff screen exists on the portal.</t>
         </is>
       </c>
       <c r="F996" s="16" t="n"/>
@@ -40428,7 +40428,7 @@
       </c>
       <c r="E998" s="11" t="inlineStr">
         <is>
-          <t>A breadcrumb reads 'Governance › Projects'. In the header are a box 'Search or jump to…' showing ⌘K (on a Mac) or Ctrl K, a help (?) button, a bell, and Priya's name with the 'DPO' badge and her initials.</t>
+          <t>A breadcrumb reads 'Governance › Projects'. In the header are a box 'Jump to page…' showing ⌘K (on a Mac) or Ctrl K, a help (?) button, a bell, and Priya's name with the 'DPO' badge and her initials.</t>
         </is>
       </c>
       <c r="F998" s="16" t="n"/>
@@ -40450,7 +40450,7 @@
       </c>
       <c r="D999" s="11" t="inlineStr">
         <is>
-          <t>Press Ctrl+K (⌘K on a Mac), or click 'Search or jump to…'. Type 'aud'.</t>
+          <t>Press Ctrl+K (⌘K on a Mac), or click 'Jump to page…'. Type 'aud'.</t>
         </is>
       </c>
       <c r="E999" s="11" t="inlineStr">
@@ -40536,7 +40536,7 @@
       </c>
       <c r="E1002" s="11" t="inlineStr">
         <is>
-          <t>An account menu opens showing 'Priya Menon' and 'DPO', then 'Your profile', 'Help manual', 'Switch to dark theme' and 'Sign out'. Press Esc: it closes and nothing else changes.</t>
+          <t>An account menu opens showing 'Priya Menon' and 'DPO', then 'My profile', 'Help manual', 'Switch to dark theme' and 'Sign out'. Press Esc: it closes and nothing else changes.</t>
         </is>
       </c>
       <c r="F1002" s="16" t="n"/>
@@ -40563,7 +40563,7 @@
       </c>
       <c r="E1003" s="11" t="inlineStr">
         <is>
-          <t>The first click folds away Projects, Approvals, Notices and Purposes; the second brings them back. The group holding the page you are on cannot be folded away.</t>
+          <t>The first click folds away 'Approval documents' and 'Purposes'; the second brings them back. The group holding the page you are on cannot be folded away.</t>
         </is>
       </c>
       <c r="F1003" s="16" t="n"/>
@@ -40752,7 +40752,7 @@
       </c>
       <c r="E1010" s="11" t="inlineStr">
         <is>
-          <t>The manual opens already set to 'For the DCO', reading '15 of 24 sections for the DCO'. Section numbers keep their places (for example 8, 12, 13, 14). The top-right button now reads 'Back to the console'.</t>
+          <t>The manual opens already set to 'For the DCO', reading '15 of 24 sections for the DCO'. Section numbers keep their places (for example 8, 12, 13, 14). The top-right button now reads 'Back to where you were'.</t>
         </is>
       </c>
       <c r="F1010" s="16" t="n"/>
@@ -40774,7 +40774,7 @@
       </c>
       <c r="D1011" s="11" t="inlineStr">
         <is>
-          <t>Choose 'Every role' in the role box. Then click 'Back to the console', press Ctrl+K (⌘K) and choose 'Open the help manual'.</t>
+          <t>Choose 'Every role' in the role box. Then click 'Back to where you were', press Ctrl+K (⌘K) and choose 'Open the help manual'.</t>
         </is>
       </c>
       <c r="E1011" s="11" t="inlineStr">

</xml_diff>

<commit_message>
docs: package 4 in the help manuals, the UAT pack and the changelog
- Both help manuals describe the project workspace, the request summary and
  "Show details" on My requests.
- UAT pack v1.5 quotes build ce91d31: project steps open the tab that holds
  the card (Setup, Consent, Collections & exchanges, Activity); the "Next
  steps" step is replaced by its absence; portal steps open a request with
  "Show details" before reading its response; OVS-21 checks the request
  summary and the folded Clock and path. Still 130 cases.
- best-practices §18: a card inside a tab is an address; the top of a record
  says where it stands, and each action sits once.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/uat/COMPASS-CMP-UAT-Test-Cases.xlsx
+++ b/docs/uat/COMPASS-CMP-UAT-Test-Cases.xlsx
@@ -582,7 +582,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Branch sprint-3/breach-and-correction, commit ebac9f4 - 5 October 2026</t>
+          <t>Branch sprint-3/breach-and-correction, commit ce91d31 - 5 October 2026</t>
         </is>
       </c>
     </row>
@@ -4962,8 +4962,8 @@
 5. Also tick 'SRIB' (collected in-house).
 6. Click 'Register project'.
 7. Look at the page that opens.
-8. Look at the 'Details' card on the right.
-9. Look at the 'Who is collecting' card.
+8. Look at the 'Details' card at the top right, beside 'What happens next'.
+9. Look at the tabs under it, then click 'Setup' and look at the 'Who is collecting' card.
 10. Click 'All projects' at the top of the page.</t>
         </is>
       </c>
@@ -4977,7 +4977,7 @@
 6. The dialog closes and a green toast 'Project registered' says 'It starts in draft. Attach a notice and an approval, then send it to the DPO.'
 7. The project's own page opens with the heading 'UAT Study 01', status badge 'In Draft', and the progress bar showing In Draft &gt; Pending Approval &gt; Approved.
 8. Internal name 'UAT-01', Requesting team 'Computer Vision', Data Collection Owner 'Not assigned', Created by 'Kavya Rao'.
-9. SEED and SRIB are both listed with the chip 'approved'; SEED says 'collected by a third party' and SRIB says 'collected in-house'.
+9. The tabs read 'Overview' (selected), 'Setup', 'Consent', 'Collections &amp; exchanges' and 'Activity'. In 'Setup', SEED and SRIB are both listed with the chip 'approved'; SEED says 'collected by a third party' and SRIB says 'collected in-house'.
 10. The Projects list shows 'UAT Study 01' with status 'In Draft' and Created by 'Kavya Rao'.</t>
         </is>
       </c>
@@ -5139,7 +5139,7 @@
 2. Find the card titled 'What happens next'.
 3. Read the warning lines under 'Moves the project to Pending Approval'.
 4. Try to click the 'Submit for approval' button on that row.
-5. Look at the 'Notices' card.
+5. Click the 'Setup' tab and look at the 'Notices' card.
 6. Look at the 'Approvals' card.
 7. Look at the buttons at the top of the page.</t>
         </is>
@@ -5150,9 +5150,9 @@
 2. It reads 'Currently In Draft. These are the moves your role can make from here.' and shows one row 'Moves the project to Pending Approval' with a 'Submit for approval' button.
 3. All six missing items are listed at once, each with a warning icon: 'The project has no notice'; 'The notice has no purposes attached'; 'The notice is missing required Rule 3 elements'; 'The notice does not say who it applies to'; 'The notice has no text yet - add at least one language'; 'No approval with a proof file'.
 4. The button is greyed out (disabled); nothing happens and the status stays 'In Draft'.
-5. It shows 'No notice yet' with the buttons 'Upload a notice document' and 'Copy an existing notice'.
+5. It shows 'No notice yet' with the buttons 'Upload a notice document' and 'Copy an existing notice'. There is NO 'New notice' button.
 6. It shows count 0, 'No approval uploaded', the text 'A security approval with its proof file is what unlocks the move to pending approval.' and an 'Upload an approval' button.
-7. 'Edit', 'Upload a notice document', 'Copy an existing notice', 'Upload approval' and 'Add site' are shown. There is NO 'New notice' button.</t>
+7. Only the status badge 'In Draft' and 'Edit' are shown. Adding a notice, an approval or a site is done on its own card in the tabs, not here.</t>
         </is>
       </c>
       <c r="M44" s="11" t="inlineStr">
@@ -5226,7 +5226,7 @@
       <c r="K45" s="11" t="inlineStr">
         <is>
           <t>1. Open project 'UAT Study 01' (Projects &gt; search &gt; click the name).
-2. In the 'Notices' card click 'Upload a notice document'.
+2. Click the 'Setup' tab, then 'Upload a notice document' in the 'Notices' card.
 3. Click 'Download it'.
 4. Under 'Notice document' use the browser's file chooser ('Choose File') to pick the blank template you just downloaded.
 5. Click 'Check the document'.
@@ -5317,7 +5317,7 @@
       </c>
       <c r="K46" s="11" t="inlineStr">
         <is>
-          <t>1. Open project 'UAT Study 01' and in the 'Notices' card click 'Upload a notice document'.
+          <t>1. Open project 'UAT Study 01', click the 'Setup' tab and in the 'Notices' card click 'Upload a notice document'.
 2. Under 'Notice document' choose the filled .docx.
 3. Click 'Check the document'.
 4. Read any yellow warnings under the green box.
@@ -5414,7 +5414,7 @@
       <c r="K47" s="11" t="inlineStr">
         <is>
           <t>1. Click 'Projects' &gt; 'Register a project'. Enter the name and description from the test data, tick 'SEED' and click 'Register project'.
-2. In the 'Notices' card click 'Copy an existing notice'.
+2. Click the 'Setup' tab, then 'Copy an existing notice' in the 'Notices' card.
 3. Open 'Notice to copy'.
 4. Choose 'NTC-GAIT-2026 v1 — Gait Identification Study 2026'.
 5. Click 'Copy into this project'.
@@ -5503,7 +5503,7 @@
       </c>
       <c r="K48" s="11" t="inlineStr">
         <is>
-          <t>1. Open project 'UAT Study 01' and look at the buttons at the top of the page.
+          <t>1. Open project 'UAT Study 01', click the 'Setup' tab and look at the buttons on the 'Notices' card.
 2. Click 'NTC-UAT-STUDY-01-2026 v1' in the 'Notices' card.
 3. Look at the 'Publication checklist' card.
 4. Look at the 'Notice text' card.
@@ -5593,15 +5593,15 @@
       </c>
       <c r="K49" s="11" t="inlineStr">
         <is>
-          <t>1. Open project 'UAT Study 01' and click 'Upload approval' at the top of the page.
+          <t>1. Open project 'UAT Study 01', click the 'Setup' tab and click 'Upload an approval' in the 'Approvals' card.
 2. Leave 'Reference number' and 'Proof document' empty, set 'Approved on' to a future date, and click 'Upload approval'.
 3. Enter 'SEC-UAT-0001', set 'Approved on' to today, choose the proof file and click 'Upload approval'.
 4. Look at the 'Approvals' card.
 5. Click 'Proof'.
 6. Look at 'What happens next'.
 7. Scroll to the bottom of the page.
-8. Click 'Submit for approval' (at the top or in 'Next steps' - either one).
-9. Look at 'What happens next' again, and at the 'History' card.</t>
+8. Click 'Submit for approval'.
+9. Look at 'What happens next' again, then click the 'Activity' tab and look at the 'History' card.</t>
         </is>
       </c>
       <c r="L49" s="11" t="inlineStr">
@@ -5612,7 +5612,7 @@
 4. Count 1; the row reads 'Security SEC-UAT-0001', 'Approved &lt;today&gt; · uploaded ... by Kavya Rao', a short hash, and a 'Proof' button.
 5. The file downloads and a toast 'Proof downloaded' says 'Hash matches the record.'
 6. 'Moves the project to Pending Approval' has no warning lines and the 'Submit for approval' button is active (highlighted).
-7. A 'Next steps' card repeats 'Moves the project to Pending Approval' with the same active 'Submit for approval' button, and under 'Other actions' the buttons from the top of the page (for example 'Upload approval') with the status badge. Nothing at the top of the page has gone.
+7. The page ends with the tabbed sections. The move is not repeated at the foot: 'Submit for approval' is only in 'What happens next' at the top.
 8. Toast 'Moved to Pending Approval'. The status badge changes to 'Pending Approval' and the progress bar moves to its second step.
 9. 'What happens next' reads 'There is nothing for your role to do at this stage.' History shows 'In Draft → Pending Approval' by 'Kavya Rao (Rnd user)' with the time. The 'Edit' button is no longer shown in the page header.</t>
         </is>
@@ -5963,9 +5963,9 @@
 3. Click 'Approve project'.
 4. Type the note and click 'Approve project' in the panel.
 5. Check the page header and progress bar.
-6. Look at the 'Notices' card.
-7. Look at the 'History' card.
-8. Look at the right-hand column.</t>
+6. Click the 'Setup' tab and look at the 'Notices' card.
+7. Click the 'Activity' tab and look at the 'History' card.
+8. Click the 'Consent' tab.</t>
         </is>
       </c>
       <c r="L53" s="11" t="inlineStr">
@@ -5977,7 +5977,7 @@
 5. Status badge 'Approved'; progress bar at the last step.
 6. 'NTC-UAT-STUDY-01-2026 v1' shows the badge 'Published' and '· published &lt;date/time&gt;'.
 7. The newest entry is 'Pending Approval → Approved' by 'Priya Menon (Dpo)' with the note shown in quotes.
-8. An info note reads 'Adding a site now is a material change: it adds a recipient to a published notice, so it requires a new notice version before collection starts there.'</t>
+8. Above 'Collection sites' an info note reads 'Adding a site now is a material change: it adds a recipient to a published notice, so it requires a new notice version before collection starts there.'</t>
         </is>
       </c>
       <c r="M53" s="11" t="inlineStr">
@@ -6055,7 +6055,7 @@
 2. Look for editing controls across the page.
 3. Read the info note in the right-hand column.
 4. Look at 'Rule 3 elements' &gt; 'Recipients'.
-5. Sign out and sign in as rnd@cmp.local. Open project 'UAT Study 01' and click 'Upload a notice document'.
+5. Sign out and sign in as rnd@cmp.local. Open project 'UAT Study 01', click the 'Setup' tab and click 'Upload a notice document' in the 'Notices' card.
 6. Choose the filled .docx and click 'Check the document'.
 7. Click 'Cancel'.</t>
         </is>
@@ -6144,13 +6144,13 @@
       <c r="K55" s="11" t="inlineStr">
         <is>
           <t>1. Click 'Projects' in the sidebar, set 'Status' to 'Approved' and open 'UAT Study 01'.
-2. Look at the 'Who is collecting' card.
-3. Click 'Add site' at the top of the page.
+2. Click the 'Setup' tab and look at the 'Who is collecting' card.
+3. Click the 'Consent' tab, then 'Add site' in the 'Collection sites' card.
 4. Open 'Data source'.
 5. Choose 'CIT · SEED · Arun Shetty'.
 6. Type the Location and click 'Add collection site'.
 7. Look at the 'Collection sites' card.
-8. Look at 'Details' on the right.
+8. Look at 'Details' at the top right.
 9. Click 'Who runs it' on the CIT row.
 10. Click 'Cancel'.</t>
         </is>
@@ -6242,7 +6242,7 @@
       <c r="K56" s="11" t="inlineStr">
         <is>
           <t>1. As Kavya Rao open project 'UAT Study 01'.
-2. Click 'Add site'.
+2. Click the 'Consent' tab, then 'Add site'.
 3. Choose Data source 'SE · SRIB · Meera Iyer', enter the Location, and click 'Add collection site'.
 4. Look at the new 'SE' row in 'Collection sites'.
 5. Click 'Who runs it' on the SE row.
@@ -6252,13 +6252,13 @@
       </c>
       <c r="L56" s="11" t="inlineStr">
         <is>
-          <t>1. Status 'Approved'. 'What happens next' says 'There is nothing for your role to do at this stage.' The 'Who is collecting' button now reads 'Request a collector'.
+          <t>1. Status 'Approved'. 'What happens next' says 'There is nothing for your role to do at this stage.' In the 'Setup' tab, the 'Who is collecting' button now reads 'Request a collector'.
 2. The 'Add a collection site' dialog opens with the material-change note.
 3. Before saving the note reads 'Meera Iyer owns SRC-SRIB-SE and will pick up this site.' After saving, toast 'Collection site added'.
 4. Owner line 'SE · Meera Iyer' with the tag 'in-house'; buttons 'Change source' and 'Who runs it' are available to the R&amp;D owner. There is NO 'Create link' button for the R&amp;D User.
 5. Dialog 'Who runs SE?' opens; the field is labelled 'R&amp;D Collection Owner' and lists R&amp;D Collection Owners (e.g. Meera Iyer · rco@cmp.local), not Data Collection Owners. Click 'Cancel'.
 6. The list includes 'SE' with project 'UAT Study 01', 'Operated by' SRIB. The 'CIT' site of UAT Study 01 is NOT listed.
-7. The project page opens. In 'Collection sites', the SE row shows a 'Create link' button; Meera has no link control for CIT.</t>
+7. The project page opens on its 'Consent' tab. In 'Collection sites', the SE row shows a 'Create link' button; Meera has no link control for CIT.</t>
         </is>
       </c>
       <c r="M56" s="11" t="inlineStr">
@@ -6442,7 +6442,7 @@
       <c r="L58" s="11" t="inlineStr">
         <is>
           <t>1. The list shows 'CIT' for project 'UAT Study 01'. The 'SE' site of UAT Study 01 is NOT listed for the DCO.
-2. The project page opens. The CIT site row shows a 'Create link' button.
+2. The project page opens on its 'Consent' tab. The CIT site row shows a 'Create link' button.
 3. Dialog 'Consent link for CIT' opens: 'The token is shown once and cannot be retrieved again.' Fields 'Expires at' (required; hint 'Required, with no default and no maximum...'), 'Maximum uses', 'Field agent reference'. 'Expires at' is empty - there is no default.
 4. The dialog stays open with 'The expiry is required' under 'Expires at'. No link is created.
 5. 'The expiry has to be in the future' is shown. No link is created.
@@ -6522,12 +6522,12 @@
       </c>
       <c r="K59" s="11" t="inlineStr">
         <is>
-          <t>1. On project 'UAT Study 01' click 'Create link' on the CIT row.
+          <t>1. On project 'UAT Study 01' click the 'Consent' tab, then 'Create link' on the CIT row.
 2. Fill in the test data and click 'Create link'.
 3. Read the URL.
 4. Click 'Copy link'.
 5. Click 'Done'.
-6. Look at the 'Consent links' card on the right.
+6. Look at the 'Consent links' card under 'Collection sites'.
 7. Click 'Copy link' on the CIT row.
 8. Open the saved URL in a private/incognito browser window.</t>
         </is>
@@ -6880,7 +6880,7 @@
       </c>
       <c r="K63" s="11" t="inlineStr">
         <is>
-          <t>1. Open project 'UAT Study 01'. In the header click 'Copy an existing notice', choose 'NTC-GAIT-2026 v1 — Gait Identification Study 2026' and click 'Copy into this project'.
+          <t>1. Open project 'UAT Study 01', click the 'Setup' tab and in the 'Notices' card click 'Copy an existing notice', choose 'NTC-GAIT-2026 v1 — Gait Identification Study 2026' and click 'Copy into this project'.
 2. Open the new notice. In 'Legal approval, per language' click 'Approve' on each language row.
 3. Click 'Publish this notice', then 'Publish and freeze'.
 4. Return to the project and look at the 'Notices' card.
@@ -8110,7 +8110,7 @@
           <t>1. Sign in as dco@cmp.local and click 'Consents'.
 2. Open one of them.
 3. Sign out, sign in as rco@cmp.local and click 'Consents'.
-4. As the RCO click 'My projects', type 'Gait Identification' in 'Search' (the list updates as you type), open 'Gait Identification Study 2026', click 'Generate export' and then 'Generate the export'.
+4. As the RCO click 'My projects', type 'Gait Identification' in 'Search' (the list updates as you type), open 'Gait Identification Study 2026', click the 'Collections &amp; exchanges' tab, then 'Generate export' and 'Generate the export'.
 5. Sign out, sign in as rnd@cmp.local and look at the sidebar.
 6. Type http://localhost:3000/consents in the address bar, then http://localhost:3000/exports.
 7. Sign out, sign in as admin@cmp.local and look at the sidebar; then open http://localhost:3000/consents.</t>
@@ -8200,7 +8200,7 @@
         <is>
           <t>1. In the sidebar click 'Processors'.
 2. Click 'Projects', type 'Gait Identification' in 'Search' (the list updates as you type) and open 'Gait Identification Study 2026'.
-3. Click 'Generate export'.
+3. Click the 'Collections &amp; exchanges' tab, then 'Generate export' on the 'Exports' card.
 4. Click 'Cancel'.
 5. Click 'Generate export' again, then 'Generate the export'.
 6. In the sidebar click 'Exports'.
@@ -8213,7 +8213,7 @@
       <c r="L77" s="11" t="inlineStr">
         <is>
           <t>1. The 'Country' column shows 'IN' for 'SEED', 'SRIB' and 'Pune Motion Lab Pvt Ltd'. If any shows something else, set it back to IN (Edit, Country, Save changes) before continuing.
-2. The project page opens with the status approved and a 'Generate export' button in the header.
+2. The project page opens with the status approved.
 3. A dialog 'Generate an export' opens with a warning ('This CSV contains personal data — name, email and mobile number for every person who consented. Generating it writes one disclosure row each…'), an information box ('One row per consent… People who have withdrawn are included and marked…') and the buttons 'Cancel' and 'Generate the export'. There is nothing to choose.
 4. The dialog closes and nothing is generated.
 5. The notice 'Export generated' says '&lt;N&gt; consent(s). Download it from the Exports page — downloading is repeatable.' The dialog closes. Write down N.
@@ -8301,7 +8301,7 @@
 2. Replace the country with 1N and click 'Save changes'.
 3. Replace it with SG and click 'Save changes'.
 4. Scroll down to the card 'Restricted countries (s.16)'. Type SG in 'Country' and UAT-TEST-NOTIF-01 in 'Notification' and click 'Restrict'.
-5. Open 'Projects' &gt; 'Gait Identification Study 2026', click 'Generate export', then 'Generate the export'.
+5. Open 'Projects' &gt; 'Gait Identification Study 2026', click the 'Collections &amp; exchanges' tab, then 'Generate export' and 'Generate the export'.
 6. Click 'Cancel' and open 'Exports'.
 7. Go back to 'Processors'; in 'Restricted countries (s.16)' click 'Lift' on SG.
 8. Restore: on the 'SEED' row click 'Edit', set 'Country' to IN and click 'Save changes'.</t>
@@ -8393,10 +8393,10 @@
         <is>
           <t>1. Click 'Processors'; on 'SEED' click 'Edit', set 'Country' to SG and click 'Save changes'.
 2. Check the 'Restricted countries (s.16)' card.
-3. Open 'Gait Identification Study 2026', click 'Generate export', then 'Generate the export'.
+3. Open 'Gait Identification Study 2026', click the 'Collections &amp; exchanges' tab, then 'Generate export' and 'Generate the export'.
 4. Click 'Cancel' and open 'Exports'.
 5. Restore: 'Processors' &gt; 'SEED' &gt; 'Edit', set 'Country' to IN, 'Save changes'.
-6. Open the project again, click 'Generate export', then 'Generate the export'.
+6. Open the project again, click the 'Collections &amp; exchanges' tab, then 'Generate export' and 'Generate the export'.
 7. Open 'Exports' and click 'Download' on the new top row, then open the CSV.</t>
         </is>
       </c>
@@ -8483,10 +8483,10 @@
         <is>
           <t>1. Click 'Processors', then 'Register processor'. Fill 'Registered legal name', 'Type', 'Contract reference' and 'Security confirmed on' from the test data, leave 'Country' empty and click 'Register processor'.
 2. Find the coordinator's prepared processor in the list.
-3. Open the prepared project, click 'Generate export', then 'Generate the export'.
+3. Open the prepared project, click the 'Collections &amp; exchanges' tab, then 'Generate export' and 'Generate the export'.
 4. Click 'Cancel' and open 'Exports'.
 5. Go to 'Processors', click 'Edit' on the prepared processor, set 'Country' to IN and click 'Save changes'.
-6. Open the prepared project again and click 'Generate export', then 'Generate the export'.
+6. Open the prepared project again, click the 'Collections &amp; exchanges' tab, then 'Generate export' and 'Generate the export'.
 7. Clean-up: on the 'UAT No Country Lab Pvt Ltd' row click 'Suspend'.</t>
         </is>
       </c>
@@ -8969,7 +8969,7 @@
 5. Leave 'About' on 'Everything you hold about me'. Type the test text in 'Your request'. Click 'Send the request'.
 6. Look at the new card for RR-A at the top of the list.
 7. Look at the lower half of the card (it opens already expanded after sending).
-8. Click 'Hide progress', then 'Show progress'.
+8. Click 'Hide details', then 'Show details'.
 9. Click 'Show what was recorded' on the card.
 10. Ask the coordinator to check the outbox for an acknowledgement sent to subject@cmp.local.</t>
         </is>
@@ -8982,8 +8982,8 @@
 4. A blue note under it reads 'A summary of the personal data we hold about you, what we do with it, and who it has been shared with.'
 5. The dialog closes. A message 'Recorded as RR-YYYY-NNNNNN' appears with 'You will hear from us by &lt;date&gt;.' Write down the reference (RR-A).
 6. The card shows the reference, the badges 'Access · s.11' and 'Received', and the line 'Received &lt;date and time&gt; · you will hear by &lt;date&gt;'. Your request text is shown. There is NO yellow box saying 'We have not yet confirmed this came from you'.
-7. Two columns are shown: 'Clock' with the checkpoints, and 'The path' with steps including 'Request received', 'Acknowledge', 'Identity verified?', 'A valid access request?' and 'The CMP answers its own records'. The button reads 'Hide progress'.
-8. The Clock and path collapse and open again.
+7. Two columns are shown: 'Clock' with the checkpoints, and 'The path' with steps including 'Request received', 'Acknowledge', 'Identity verified?', 'A valid access request?' and 'The CMP answers its own records'. The button reads 'Hide details'.
+8. The card folds to a summary - reference, badges, dates and the first lines of your request - and opens again.
 9. A list of recorded events opens, oldest first, starting with the request being received. The button now reads 'Hide what was recorded'.
 10. An acknowledgement for RR-A is in the outbox, quoting the reference and the date by which she will hear.</t>
         </is>
@@ -9742,7 +9742,7 @@
 4. Click 'Release and close'.
 5. Look at 'What happens next'.
 6. Ask the coordinator to check the outbox for the response mail to subject@cmp.local.
-7. In Browser A reload 'My requests' and look at RR-A.
+7. In Browser A reload 'My requests'. RR-A's folded card shows 'Our response is ready' with 'Download the file'; click 'Show details' on it.
 8. Click 'Download the file'.
 9. Open the downloaded file in a text editor.
 10. Click 'Download' next to access-extract.pdf.</t>
@@ -9843,7 +9843,7 @@
 6. In 'What happens next' click 'In progress'.
 7. In Browser A, on 'My requests', make a new request: 'Erasure (s.12(3))' with the RR-W text. Note its reference (RR-W).
 8. In Browser B open RR-W and click 'They meant withdrawal'.
-9. In Browser A reload 'My requests' and look at RR-W, then open 'My consents'.</t>
+9. In Browser A reload 'My requests', click 'Show details' on RR-W, then open 'My consents'.</t>
         </is>
       </c>
       <c r="L94" s="11" t="inlineStr">
@@ -10413,7 +10413,7 @@
 3. Type the response and click 'Release and close'.
 4. Look at the scope card.
 5. Ask the coordinator to show the response mail to subject@cmp.local.
-6. In Browser A reload 'My requests' and look at RR-E.
+6. In Browser A reload 'My requests' and click 'Show details' on RR-E.
 7. Click 'Download the file' and open the saved .json file.
 8. In the same file look at 'consents'.</t>
         </is>
@@ -10719,7 +10719,7 @@
 3. Without adding any holder, click 'Collating' in 'What happens next'.
 4. Read the warning on '9–10 · Collate, review, release' and open 'Outcome'.
 5. Read the hint under 'The response', type the response and click 'Release and close'.
-6. In Browser A reload 'My requests' and look at RR-C.</t>
+6. In Browser A reload 'My requests' and click 'Show details' on RR-C.</t>
         </is>
       </c>
       <c r="L103" s="11" t="inlineStr">
@@ -10807,16 +10807,16 @@
       </c>
       <c r="K104" s="11" t="inlineStr">
         <is>
-          <t>1. In Browser A on 'My requests' click 'Dispute this response' on RR-A.
+          <t>1. In Browser A on 'My requests' click 'Show details' on RR-A, then 'Dispute this response'.
 2. Type 'short' in 'What was wrong' and click 'Raise the grievance'.
 3. Type the full text, leave the checkbox unticked and click 'Raise the grievance'.
-4. Look at the RR-G and RR-A cards.
+4. Click 'Show details' on the RR-G card.
 5. Click 'See RR-A in full'.
 6. In Browser B open RR-G from 'Rights requests'.
 7. Look at '4 · Linked, and about whom?'.
 8. Click 'Confirm classification' (Complaint (grievance) (s.13)) and then 'In progress'.
 9. Change 'Decision' to 'Not upheld', type the finding and click 'Decide and close'.
-10. In Browser A reload 'My requests' and look at RR-G.</t>
+10. In Browser A reload 'My requests' and click 'Show details' on RR-G.</t>
         </is>
       </c>
       <c r="L104" s="11" t="inlineStr">
@@ -10824,8 +10824,8 @@
           <t>1. A dialog 'Dispute RR-A' opens: 'A grievance under section 13. Say what was wrong with the handling - late, incomplete, sent the wrong way, or the outcome itself.' with 'What was wrong', the checkbox 'This is about the Data Protection Officer's own decisions.', 'Cancel' and 'Raise the grievance'.
 2. The error 'Say what you are asking for, in a sentence or two.' appears; nothing is recorded.
 3. 'Grievance recorded as RR-...' with 'It is linked to the original request.' appears. Note RR-G.
-4. RR-G shows 'Complaint (grievance) · s.13', 'Received' and a box 'What you disputed' naming RR-A with 'Complete: &lt;start of the answer&gt;' and 'See RR-A in full'. RR-A shows 'You disputed this in RR-G' with 'See it'.
-5. The page scrolls to RR-A and briefly highlights it.
+4. RR-G shows 'Complaint (grievance) · s.13', 'Received' and a box 'What you disputed' naming RR-A with 'Complete: &lt;start of the answer&gt;' and 'See RR-A in full'.
+5. The page scrolls to RR-A, opens it and briefly highlights it. RR-A shows 'You disputed this in RR-G' with 'See it'.
 6. The line under the heading reads 'Complaint (grievance) · s.13 · Portal'. 'About' shows RR-A with 'the request under dispute, shown below', and a card 'The request under dispute' shows RR-A's dates, what was asked and its answer.
 7. It contains 'Is the complaint about the DPO?' with the text '...Recuse if this concerns your handling.' and a button 'This is about me - escalate' (do not click it).
 8. The request is 'In progress' and a card '6 · Is it upheld?' appears with 'Decision' ('Upheld'), 'What was found, and why', 'Remedy' and a ticked checkbox 'Re-run RR-A as a new request linked to this decision.' 'Decide and close' is greyed out.
@@ -10922,7 +10922,7 @@
 9. In 'What happens next' click 'In progress'.
 10. In Browser B (DPO) reload RR-D, choose 'Not upheld', type a finding and click 'Decide and close'.
 11. In Browser C keep 'Upheld', type a finding in 'What was found, and why' and the remedy in 'Remedy', and click 'Decide and close'.
-12. In Browser A reload 'My requests' and look at RR-D.</t>
+12. In Browser A reload 'My requests' and click 'Show details' on RR-D.</t>
         </is>
       </c>
       <c r="L105" s="11" t="inlineStr">
@@ -11321,7 +11321,7 @@
 3. Click 'Closed'.
 4. Click 'Open'.
 5. Click 'All', then type the number part of RR-A's reference (for example 000123) in the search box.
-6. Click 'Show all requests'. Type 'grievance' in the search box, so that only grievances remain, and on RR-G (RGT-20) click 'See RR-A in full'.</t>
+6. Click 'Show all requests'. Type 'grievance' in the search box, so that only grievances remain. On RR-G (RGT-20) click 'Show details', then 'See RR-A in full'.</t>
         </is>
       </c>
       <c r="L109" s="11" t="inlineStr">
@@ -11331,7 +11331,7 @@
 3. Only answered or closed requests remain, for example RR-A with the badge 'Complete'. No 'Received' or 'In progress' request is listed.
 4. Only requests still being worked on remain. The count beside 'Open' equals the number of cards shown.
 5. Only RR-A remains. Typing 'grievance' instead shows only grievances; typing 'zzz' shows 'No requests match' with a 'Show all requests' button.
-6. RR-A was hidden by the search, so the search is cleared and 'All' selected; the page scrolls to RR-A and briefly highlights it.</t>
+6. RR-A was hidden by the search, so the search is cleared and 'All' selected; the page scrolls to RR-A, opens it and briefly highlights it.</t>
         </is>
       </c>
       <c r="M109" s="11" t="inlineStr">
@@ -13315,7 +13315,7 @@
 6. Click Priya's name at the top right of the header.
 7. In the sidebar click the heading 'GOVERNANCE', then click it again.
 8. Click 'Collapse sidebar' at the bottom of the sidebar, then reload the page.
-9. Open 'Rights requests', open any request, and click the card 'Clock and path'.</t>
+9. Open 'Rights requests', open any request, look at the top of the page, then click the card 'Clock and path'.</t>
         </is>
       </c>
       <c r="L130" s="11" t="inlineStr">
@@ -13328,7 +13328,7 @@
 6. An account menu opens showing 'Priya Menon' and 'DPO', then 'My profile', 'Help manual', 'Switch to dark theme' and 'Sign out'. Press Esc: it closes and nothing else changes.
 7. The first click folds away 'Approval documents' and 'Purposes'; the second brings them back. The group holding the page you are on cannot be folded away.
 8. The sidebar becomes a narrow strip of icons (hovering an icon shows its name) and stays that way after the reload. Click 'Expand sidebar' to restore it.
-9. The card folds to its heading, so the working cards below move up. Clicking it again unfolds it. On a project page, the 'History' card folds the same way and shows its number of entries.</t>
+9. The page opens on a summary: 'Due' with the date and days left, 'Current step', 'With' and 'Next'. 'Clock and path' starts folded to its heading; clicking it opens the checkpoints and the path, and clicking again folds it. On a project page the sections are tabs - 'Overview', 'Setup', 'Consent', 'Collections &amp; exchanges' and 'Activity' (which holds 'History', with its number of entries on the tab).</t>
         </is>
       </c>
       <c r="M130" s="11" t="inlineStr">
@@ -21091,7 +21091,7 @@
       </c>
       <c r="D282" s="11" t="inlineStr">
         <is>
-          <t>Look at the 'Details' card on the right.</t>
+          <t>Look at the 'Details' card at the top right, beside 'What happens next'.</t>
         </is>
       </c>
       <c r="E282" s="11" t="inlineStr">
@@ -21118,12 +21118,12 @@
       </c>
       <c r="D283" s="11" t="inlineStr">
         <is>
-          <t>Look at the 'Who is collecting' card.</t>
+          <t>Look at the tabs under it, then click 'Setup' and look at the 'Who is collecting' card.</t>
         </is>
       </c>
       <c r="E283" s="11" t="inlineStr">
         <is>
-          <t>SEED and SRIB are both listed with the chip 'approved'; SEED says 'collected by a third party' and SRIB says 'collected in-house'.</t>
+          <t>The tabs read 'Overview' (selected), 'Setup', 'Consent', 'Collections &amp; exchanges' and 'Activity'. In 'Setup', SEED and SRIB are both listed with the chip 'approved'; SEED says 'collected by a third party' and SRIB says 'collected in-house'.</t>
         </is>
       </c>
       <c r="F283" s="16" t="n"/>
@@ -21415,12 +21415,12 @@
       </c>
       <c r="D294" s="11" t="inlineStr">
         <is>
-          <t>Look at the 'Notices' card.</t>
+          <t>Click the 'Setup' tab and look at the 'Notices' card.</t>
         </is>
       </c>
       <c r="E294" s="11" t="inlineStr">
         <is>
-          <t>It shows 'No notice yet' with the buttons 'Upload a notice document' and 'Copy an existing notice'.</t>
+          <t>It shows 'No notice yet' with the buttons 'Upload a notice document' and 'Copy an existing notice'. There is NO 'New notice' button.</t>
         </is>
       </c>
       <c r="F294" s="16" t="n"/>
@@ -21474,7 +21474,7 @@
       </c>
       <c r="E296" s="11" t="inlineStr">
         <is>
-          <t>'Edit', 'Upload a notice document', 'Copy an existing notice', 'Upload approval' and 'Add site' are shown. There is NO 'New notice' button.</t>
+          <t>Only the status badge 'In Draft' and 'Edit' are shown. Adding a notice, an approval or a site is done on its own card in the tabs, not here.</t>
         </is>
       </c>
       <c r="F296" s="16" t="n"/>
@@ -21523,7 +21523,7 @@
       </c>
       <c r="D298" s="11" t="inlineStr">
         <is>
-          <t>In the 'Notices' card click 'Upload a notice document'.</t>
+          <t>Click the 'Setup' tab, then 'Upload a notice document' in the 'Notices' card.</t>
         </is>
       </c>
       <c r="E298" s="11" t="inlineStr">
@@ -21685,7 +21685,7 @@
       </c>
       <c r="D304" s="11" t="inlineStr">
         <is>
-          <t>Open project 'UAT Study 01' and in the 'Notices' card click 'Upload a notice document'.</t>
+          <t>Open project 'UAT Study 01', click the 'Setup' tab and in the 'Notices' card click 'Upload a notice document'.</t>
         </is>
       </c>
       <c r="E304" s="11" t="inlineStr">
@@ -21955,7 +21955,7 @@
       </c>
       <c r="D314" s="11" t="inlineStr">
         <is>
-          <t>In the 'Notices' card click 'Copy an existing notice'.</t>
+          <t>Click the 'Setup' tab, then 'Copy an existing notice' in the 'Notices' card.</t>
         </is>
       </c>
       <c r="E314" s="11" t="inlineStr">
@@ -22117,7 +22117,7 @@
       </c>
       <c r="D320" s="11" t="inlineStr">
         <is>
-          <t>Open project 'UAT Study 01' and look at the buttons at the top of the page.</t>
+          <t>Open project 'UAT Study 01', click the 'Setup' tab and look at the buttons on the 'Notices' card.</t>
         </is>
       </c>
       <c r="E320" s="11" t="inlineStr">
@@ -22279,7 +22279,7 @@
       </c>
       <c r="D326" s="11" t="inlineStr">
         <is>
-          <t>Open project 'UAT Study 01' and click 'Upload approval' at the top of the page.</t>
+          <t>Open project 'UAT Study 01', click the 'Setup' tab and click 'Upload an approval' in the 'Approvals' card.</t>
         </is>
       </c>
       <c r="E326" s="11" t="inlineStr">
@@ -22446,7 +22446,7 @@
       </c>
       <c r="E332" s="11" t="inlineStr">
         <is>
-          <t>A 'Next steps' card repeats 'Moves the project to Pending Approval' with the same active 'Submit for approval' button, and under 'Other actions' the buttons from the top of the page (for example 'Upload approval') with the status badge. Nothing at the top of the page has gone.</t>
+          <t>The page ends with the tabbed sections. The move is not repeated at the foot: 'Submit for approval' is only in 'What happens next' at the top.</t>
         </is>
       </c>
       <c r="F332" s="16" t="n"/>
@@ -22468,7 +22468,7 @@
       </c>
       <c r="D333" s="11" t="inlineStr">
         <is>
-          <t>Click 'Submit for approval' (at the top or in 'Next steps' - either one).</t>
+          <t>Click 'Submit for approval'.</t>
         </is>
       </c>
       <c r="E333" s="11" t="inlineStr">
@@ -22495,7 +22495,7 @@
       </c>
       <c r="D334" s="11" t="inlineStr">
         <is>
-          <t>Look at 'What happens next' again, and at the 'History' card.</t>
+          <t>Look at 'What happens next' again, then click the 'Activity' tab and look at the 'History' card.</t>
         </is>
       </c>
       <c r="E334" s="11" t="inlineStr">
@@ -23251,7 +23251,7 @@
       </c>
       <c r="D362" s="11" t="inlineStr">
         <is>
-          <t>Look at the 'Notices' card.</t>
+          <t>Click the 'Setup' tab and look at the 'Notices' card.</t>
         </is>
       </c>
       <c r="E362" s="11" t="inlineStr">
@@ -23278,7 +23278,7 @@
       </c>
       <c r="D363" s="11" t="inlineStr">
         <is>
-          <t>Look at the 'History' card.</t>
+          <t>Click the 'Activity' tab and look at the 'History' card.</t>
         </is>
       </c>
       <c r="E363" s="11" t="inlineStr">
@@ -23305,12 +23305,12 @@
       </c>
       <c r="D364" s="11" t="inlineStr">
         <is>
-          <t>Look at the right-hand column.</t>
+          <t>Click the 'Consent' tab.</t>
         </is>
       </c>
       <c r="E364" s="11" t="inlineStr">
         <is>
-          <t>An info note reads 'Adding a site now is a material change: it adds a recipient to a published notice, so it requires a new notice version before collection starts there.'</t>
+          <t>Above 'Collection sites' an info note reads 'Adding a site now is a material change: it adds a recipient to a published notice, so it requires a new notice version before collection starts there.'</t>
         </is>
       </c>
       <c r="F364" s="16" t="n"/>
@@ -23440,7 +23440,7 @@
       </c>
       <c r="D369" s="11" t="inlineStr">
         <is>
-          <t>Sign out and sign in as rnd@cmp.local. Open project 'UAT Study 01' and click 'Upload a notice document'.</t>
+          <t>Sign out and sign in as rnd@cmp.local. Open project 'UAT Study 01', click the 'Setup' tab and click 'Upload a notice document' in the 'Notices' card.</t>
         </is>
       </c>
       <c r="E369" s="11" t="inlineStr">
@@ -23548,7 +23548,7 @@
       </c>
       <c r="D373" s="11" t="inlineStr">
         <is>
-          <t>Look at the 'Who is collecting' card.</t>
+          <t>Click the 'Setup' tab and look at the 'Who is collecting' card.</t>
         </is>
       </c>
       <c r="E373" s="11" t="inlineStr">
@@ -23575,7 +23575,7 @@
       </c>
       <c r="D374" s="11" t="inlineStr">
         <is>
-          <t>Click 'Add site' at the top of the page.</t>
+          <t>Click the 'Consent' tab, then 'Add site' in the 'Collection sites' card.</t>
         </is>
       </c>
       <c r="E374" s="11" t="inlineStr">
@@ -23710,7 +23710,7 @@
       </c>
       <c r="D379" s="11" t="inlineStr">
         <is>
-          <t>Look at 'Details' on the right.</t>
+          <t>Look at 'Details' at the top right.</t>
         </is>
       </c>
       <c r="E379" s="11" t="inlineStr">
@@ -23796,7 +23796,7 @@
       </c>
       <c r="E382" s="11" t="inlineStr">
         <is>
-          <t>Status 'Approved'. 'What happens next' says 'There is nothing for your role to do at this stage.' The 'Who is collecting' button now reads 'Request a collector'.</t>
+          <t>Status 'Approved'. 'What happens next' says 'There is nothing for your role to do at this stage.' In the 'Setup' tab, the 'Who is collecting' button now reads 'Request a collector'.</t>
         </is>
       </c>
       <c r="F382" s="16" t="n"/>
@@ -23818,7 +23818,7 @@
       </c>
       <c r="D383" s="11" t="inlineStr">
         <is>
-          <t>Click 'Add site'.</t>
+          <t>Click the 'Consent' tab, then 'Add site'.</t>
         </is>
       </c>
       <c r="E383" s="11" t="inlineStr">
@@ -23958,7 +23958,7 @@
       </c>
       <c r="E388" s="11" t="inlineStr">
         <is>
-          <t>The project page opens. In 'Collection sites', the SE row shows a 'Create link' button; Meera has no link control for CIT.</t>
+          <t>The project page opens on its 'Consent' tab. In 'Collection sites', the SE row shows a 'Create link' button; Meera has no link control for CIT.</t>
         </is>
       </c>
       <c r="F388" s="16" t="n"/>
@@ -24228,7 +24228,7 @@
       </c>
       <c r="E398" s="11" t="inlineStr">
         <is>
-          <t>The project page opens. The CIT site row shows a 'Create link' button.</t>
+          <t>The project page opens on its 'Consent' tab. The CIT site row shows a 'Create link' button.</t>
         </is>
       </c>
       <c r="F398" s="16" t="n"/>
@@ -24385,7 +24385,7 @@
       </c>
       <c r="D404" s="11" t="inlineStr">
         <is>
-          <t>On project 'UAT Study 01' click 'Create link' on the CIT row.</t>
+          <t>On project 'UAT Study 01' click the 'Consent' tab, then 'Create link' on the CIT row.</t>
         </is>
       </c>
       <c r="E404" s="11" t="inlineStr">
@@ -24520,7 +24520,7 @@
       </c>
       <c r="D409" s="11" t="inlineStr">
         <is>
-          <t>Look at the 'Consent links' card on the right.</t>
+          <t>Look at the 'Consent links' card under 'Collection sites'.</t>
         </is>
       </c>
       <c r="E409" s="11" t="inlineStr">
@@ -25114,7 +25114,7 @@
       </c>
       <c r="D431" s="11" t="inlineStr">
         <is>
-          <t>Open project 'UAT Study 01'. In the header click 'Copy an existing notice', choose 'NTC-GAIT-2026 v1 — Gait Identification Study 2026' and click 'Copy into this project'.</t>
+          <t>Open project 'UAT Study 01', click the 'Setup' tab and in the 'Notices' card click 'Copy an existing notice', choose 'NTC-GAIT-2026 v1 — Gait Identification Study 2026' and click 'Copy into this project'.</t>
         </is>
       </c>
       <c r="E431" s="11" t="inlineStr">
@@ -28030,7 +28030,7 @@
       </c>
       <c r="D539" s="11" t="inlineStr">
         <is>
-          <t>As the RCO click 'My projects', type 'Gait Identification' in 'Search' (the list updates as you type), open 'Gait Identification Study 2026', click 'Generate export' and then 'Generate the export'.</t>
+          <t>As the RCO click 'My projects', type 'Gait Identification' in 'Search' (the list updates as you type), open 'Gait Identification Study 2026', click the 'Collections &amp; exchanges' tab, then 'Generate export' and 'Generate the export'.</t>
         </is>
       </c>
       <c r="E539" s="11" t="inlineStr">
@@ -28170,7 +28170,7 @@
       </c>
       <c r="E544" s="11" t="inlineStr">
         <is>
-          <t>The project page opens with the status approved and a 'Generate export' button in the header.</t>
+          <t>The project page opens with the status approved.</t>
         </is>
       </c>
       <c r="F544" s="16" t="n"/>
@@ -28192,7 +28192,7 @@
       </c>
       <c r="D545" s="11" t="inlineStr">
         <is>
-          <t>Click 'Generate export'.</t>
+          <t>Click the 'Collections &amp; exchanges' tab, then 'Generate export' on the 'Exports' card.</t>
         </is>
       </c>
       <c r="E545" s="11" t="inlineStr">
@@ -28516,7 +28516,7 @@
       </c>
       <c r="D557" s="11" t="inlineStr">
         <is>
-          <t>Open 'Projects' &gt; 'Gait Identification Study 2026', click 'Generate export', then 'Generate the export'.</t>
+          <t>Open 'Projects' &gt; 'Gait Identification Study 2026', click the 'Collections &amp; exchanges' tab, then 'Generate export' and 'Generate the export'.</t>
         </is>
       </c>
       <c r="E557" s="11" t="inlineStr">
@@ -28678,7 +28678,7 @@
       </c>
       <c r="D563" s="11" t="inlineStr">
         <is>
-          <t>Open 'Gait Identification Study 2026', click 'Generate export', then 'Generate the export'.</t>
+          <t>Open 'Gait Identification Study 2026', click the 'Collections &amp; exchanges' tab, then 'Generate export' and 'Generate the export'.</t>
         </is>
       </c>
       <c r="E563" s="11" t="inlineStr">
@@ -28759,7 +28759,7 @@
       </c>
       <c r="D566" s="11" t="inlineStr">
         <is>
-          <t>Open the project again, click 'Generate export', then 'Generate the export'.</t>
+          <t>Open the project again, click the 'Collections &amp; exchanges' tab, then 'Generate export' and 'Generate the export'.</t>
         </is>
       </c>
       <c r="E566" s="11" t="inlineStr">
@@ -28867,7 +28867,7 @@
       </c>
       <c r="D570" s="11" t="inlineStr">
         <is>
-          <t>Open the prepared project, click 'Generate export', then 'Generate the export'.</t>
+          <t>Open the prepared project, click the 'Collections &amp; exchanges' tab, then 'Generate export' and 'Generate the export'.</t>
         </is>
       </c>
       <c r="E570" s="11" t="inlineStr">
@@ -28948,7 +28948,7 @@
       </c>
       <c r="D573" s="11" t="inlineStr">
         <is>
-          <t>Open the prepared project again and click 'Generate export', then 'Generate the export'.</t>
+          <t>Open the prepared project again, click the 'Collections &amp; exchanges' tab, then 'Generate export' and 'Generate the export'.</t>
         </is>
       </c>
       <c r="E573" s="11" t="inlineStr">
@@ -30195,7 +30195,7 @@
       </c>
       <c r="E619" s="11" t="inlineStr">
         <is>
-          <t>Two columns are shown: 'Clock' with the checkpoints, and 'The path' with steps including 'Request received', 'Acknowledge', 'Identity verified?', 'A valid access request?' and 'The CMP answers its own records'. The button reads 'Hide progress'.</t>
+          <t>Two columns are shown: 'Clock' with the checkpoints, and 'The path' with steps including 'Request received', 'Acknowledge', 'Identity verified?', 'A valid access request?' and 'The CMP answers its own records'. The button reads 'Hide details'.</t>
         </is>
       </c>
       <c r="F619" s="16" t="n"/>
@@ -30217,12 +30217,12 @@
       </c>
       <c r="D620" s="11" t="inlineStr">
         <is>
-          <t>Click 'Hide progress', then 'Show progress'.</t>
+          <t>Click 'Hide details', then 'Show details'.</t>
         </is>
       </c>
       <c r="E620" s="11" t="inlineStr">
         <is>
-          <t>The Clock and path collapse and open again.</t>
+          <t>The card folds to a summary - reference, badges, dates and the first lines of your request - and opens again.</t>
         </is>
       </c>
       <c r="F620" s="16" t="n"/>
@@ -31945,7 +31945,7 @@
       </c>
       <c r="D684" s="11" t="inlineStr">
         <is>
-          <t>In Browser A reload 'My requests' and look at RR-A.</t>
+          <t>In Browser A reload 'My requests'. RR-A's folded card shows 'Our response is ready' with 'Download the file'; click 'Show details' on it.</t>
         </is>
       </c>
       <c r="E684" s="11" t="inlineStr">
@@ -32269,7 +32269,7 @@
       </c>
       <c r="D696" s="11" t="inlineStr">
         <is>
-          <t>In Browser A reload 'My requests' and look at RR-W, then open 'My consents'.</t>
+          <t>In Browser A reload 'My requests', click 'Show details' on RR-W, then open 'My consents'.</t>
         </is>
       </c>
       <c r="E696" s="11" t="inlineStr">
@@ -33538,7 +33538,7 @@
       </c>
       <c r="D743" s="11" t="inlineStr">
         <is>
-          <t>In Browser A reload 'My requests' and look at RR-E.</t>
+          <t>In Browser A reload 'My requests' and click 'Show details' on RR-E.</t>
         </is>
       </c>
       <c r="E743" s="11" t="inlineStr">
@@ -34402,7 +34402,7 @@
       </c>
       <c r="D775" s="11" t="inlineStr">
         <is>
-          <t>In Browser A reload 'My requests' and look at RR-C.</t>
+          <t>In Browser A reload 'My requests' and click 'Show details' on RR-C.</t>
         </is>
       </c>
       <c r="E775" s="11" t="inlineStr">
@@ -34429,7 +34429,7 @@
       </c>
       <c r="D776" s="11" t="inlineStr">
         <is>
-          <t>In Browser A on 'My requests' click 'Dispute this response' on RR-A.</t>
+          <t>In Browser A on 'My requests' click 'Show details' on RR-A, then 'Dispute this response'.</t>
         </is>
       </c>
       <c r="E776" s="11" t="inlineStr">
@@ -34510,12 +34510,12 @@
       </c>
       <c r="D779" s="11" t="inlineStr">
         <is>
-          <t>Look at the RR-G and RR-A cards.</t>
+          <t>Click 'Show details' on the RR-G card.</t>
         </is>
       </c>
       <c r="E779" s="11" t="inlineStr">
         <is>
-          <t>RR-G shows 'Complaint (grievance) · s.13', 'Received' and a box 'What you disputed' naming RR-A with 'Complete: &lt;start of the answer&gt;' and 'See RR-A in full'. RR-A shows 'You disputed this in RR-G' with 'See it'.</t>
+          <t>RR-G shows 'Complaint (grievance) · s.13', 'Received' and a box 'What you disputed' naming RR-A with 'Complete: &lt;start of the answer&gt;' and 'See RR-A in full'.</t>
         </is>
       </c>
       <c r="F779" s="16" t="n"/>
@@ -34542,7 +34542,7 @@
       </c>
       <c r="E780" s="11" t="inlineStr">
         <is>
-          <t>The page scrolls to RR-A and briefly highlights it.</t>
+          <t>The page scrolls to RR-A, opens it and briefly highlights it. RR-A shows 'You disputed this in RR-G' with 'See it'.</t>
         </is>
       </c>
       <c r="F780" s="16" t="n"/>
@@ -34672,7 +34672,7 @@
       </c>
       <c r="D785" s="11" t="inlineStr">
         <is>
-          <t>In Browser A reload 'My requests' and look at RR-G.</t>
+          <t>In Browser A reload 'My requests' and click 'Show details' on RR-G.</t>
         </is>
       </c>
       <c r="E785" s="11" t="inlineStr">
@@ -34996,7 +34996,7 @@
       </c>
       <c r="D797" s="11" t="inlineStr">
         <is>
-          <t>In Browser A reload 'My requests' and look at RR-D.</t>
+          <t>In Browser A reload 'My requests' and click 'Show details' on RR-D.</t>
         </is>
       </c>
       <c r="E797" s="11" t="inlineStr">
@@ -35941,12 +35941,12 @@
       </c>
       <c r="D832" s="11" t="inlineStr">
         <is>
-          <t>Click 'Show all requests'. Type 'grievance' in the search box, so that only grievances remain, and on RR-G (RGT-20) click 'See RR-A in full'.</t>
+          <t>Click 'Show all requests'. Type 'grievance' in the search box, so that only grievances remain. On RR-G (RGT-20) click 'Show details', then 'See RR-A in full'.</t>
         </is>
       </c>
       <c r="E832" s="11" t="inlineStr">
         <is>
-          <t>RR-A was hidden by the search, so the search is cleared and 'All' selected; the page scrolls to RR-A and briefly highlights it.</t>
+          <t>RR-A was hidden by the search, so the search is cleared and 'All' selected; the page scrolls to RR-A, opens it and briefly highlights it.</t>
         </is>
       </c>
       <c r="F832" s="16" t="n"/>
@@ -40612,12 +40612,12 @@
       </c>
       <c r="D1005" s="11" t="inlineStr">
         <is>
-          <t>Open 'Rights requests', open any request, and click the card 'Clock and path'.</t>
+          <t>Open 'Rights requests', open any request, look at the top of the page, then click the card 'Clock and path'.</t>
         </is>
       </c>
       <c r="E1005" s="11" t="inlineStr">
         <is>
-          <t>The card folds to its heading, so the working cards below move up. Clicking it again unfolds it. On a project page, the 'History' card folds the same way and shows its number of entries.</t>
+          <t>The page opens on a summary: 'Due' with the date and days left, 'Current step', 'With' and 'Next'. 'Clock and path' starts folded to its heading; clicking it opens the checkpoints and the path, and clicking again folds it. On a project page the sections are tabs - 'Overview', 'Setup', 'Consent', 'Collections &amp; exchanges' and 'Activity' (which holds 'History', with its number of entries on the tab).</t>
         </is>
       </c>
       <c r="F1005" s="16" t="n"/>

</xml_diff>